<commit_message>
#45 Reading List: updated to 2025-05-16.
</commit_message>
<xml_diff>
--- a/data/Reading List.xlsx
+++ b/data/Reading List.xlsx
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5286" uniqueCount="1123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5310" uniqueCount="1129">
   <si>
     <t>Format</t>
   </si>
@@ -3410,6 +3410,24 @@
   </si>
   <si>
     <t>Useless. This book is a mix between a debugging guide for super-beginners and a hundreds page long mind masturbation about the topic.</t>
+  </si>
+  <si>
+    <t>Getting Started with an Antinet Zettelkasten</t>
+  </si>
+  <si>
+    <t>2025-05-15</t>
+  </si>
+  <si>
+    <t>Useless. It's positive to have a book specifically about Antinets, but it should be more pragmatic. This one is a collection of rants and of "Please trust me on this" packaged in a funky layout.</t>
+  </si>
+  <si>
+    <t>Web App Development Made Simple with Streamlit</t>
+  </si>
+  <si>
+    <t>2025-05-16</t>
+  </si>
+  <si>
+    <t>Useless. This book dedicates only few pages at the beginning about Streamlit, and then talks about random Python libraries for the rest of the book. Additionally, instead of using textual code listings, it shows them as screenshots with small font and black background, making them unreadable.</t>
   </si>
 </sst>
 </file>
@@ -31650,7 +31668,7 @@
         <v>159</v>
       </c>
       <c r="S314" s="17">
-        <f t="shared" ref="S314:S340" si="123">LEN(P314)</f>
+        <f t="shared" ref="S314:S342" si="123">LEN(P314)</f>
         <v>35</v>
       </c>
       <c r="T314" s="49">
@@ -33348,48 +33366,134 @@
       </c>
     </row>
     <row r="341" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A341" s="13"/>
-      <c r="B341" s="9"/>
-      <c r="C341" s="9"/>
-      <c r="D341" s="9"/>
-      <c r="E341" s="9"/>
-      <c r="F341" s="9"/>
-      <c r="G341" s="9"/>
-      <c r="H341" s="9"/>
-      <c r="I341" s="9"/>
-      <c r="J341" s="9"/>
-      <c r="K341" s="9"/>
-      <c r="L341" s="9"/>
-      <c r="M341" s="9"/>
-      <c r="N341" s="9"/>
-      <c r="O341" s="9"/>
-      <c r="P341" s="13"/>
-      <c r="Q341" s="9"/>
-      <c r="R341" s="9"/>
-      <c r="S341" s="17"/>
-      <c r="T341" s="9"/>
+      <c r="A341" s="13" t="s">
+        <v>1123</v>
+      </c>
+      <c r="B341" s="17">
+        <v>2023</v>
+      </c>
+      <c r="C341" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D341" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E341" s="9" t="s">
+        <v>666</v>
+      </c>
+      <c r="F341" s="17">
+        <v>63</v>
+      </c>
+      <c r="G341" s="9" t="s">
+        <v>1124</v>
+      </c>
+      <c r="H341" s="9">
+        <f t="shared" ref="H341" si="163">YEAR(G341)</f>
+        <v>2025</v>
+      </c>
+      <c r="I341" s="9">
+        <f t="shared" ref="I341" si="164">MONTH(G341)</f>
+        <v>5</v>
+      </c>
+      <c r="J341" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="K341" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="L341" s="9" t="s">
+        <v>602</v>
+      </c>
+      <c r="M341" s="17">
+        <v>1</v>
+      </c>
+      <c r="N341" s="43">
+        <v>0</v>
+      </c>
+      <c r="O341" s="9" t="s">
+        <v>664</v>
+      </c>
+      <c r="P341" s="13" t="s">
+        <v>1125</v>
+      </c>
+      <c r="Q341" s="9" t="s">
+        <v>876</v>
+      </c>
+      <c r="R341" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="S341" s="17">
+        <f t="shared" si="123"/>
+        <v>194</v>
+      </c>
+      <c r="T341" s="17">
+        <v>0</v>
+      </c>
     </row>
     <row r="342" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A342" s="13"/>
-      <c r="B342" s="9"/>
-      <c r="C342" s="9"/>
-      <c r="D342" s="9"/>
-      <c r="E342" s="9"/>
-      <c r="F342" s="9"/>
-      <c r="G342" s="9"/>
-      <c r="H342" s="9"/>
-      <c r="I342" s="9"/>
-      <c r="J342" s="9"/>
-      <c r="K342" s="9"/>
-      <c r="L342" s="9"/>
-      <c r="M342" s="9"/>
-      <c r="N342" s="9"/>
-      <c r="O342" s="9"/>
-      <c r="P342" s="13"/>
-      <c r="Q342" s="9"/>
-      <c r="R342" s="9"/>
-      <c r="S342" s="17"/>
-      <c r="T342" s="9"/>
+      <c r="A342" s="13" t="s">
+        <v>1126</v>
+      </c>
+      <c r="B342" s="17">
+        <v>2024</v>
+      </c>
+      <c r="C342" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D342" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E342" s="9" t="s">
+        <v>666</v>
+      </c>
+      <c r="F342" s="17">
+        <v>350</v>
+      </c>
+      <c r="G342" s="9" t="s">
+        <v>1127</v>
+      </c>
+      <c r="H342" s="9">
+        <f t="shared" ref="H342" si="165">YEAR(G342)</f>
+        <v>2025</v>
+      </c>
+      <c r="I342" s="9">
+        <f t="shared" ref="I342" si="166">MONTH(G342)</f>
+        <v>5</v>
+      </c>
+      <c r="J342" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="K342" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="L342" s="9" t="s">
+        <v>365</v>
+      </c>
+      <c r="M342" s="17">
+        <v>1</v>
+      </c>
+      <c r="N342" s="43">
+        <v>39.99</v>
+      </c>
+      <c r="O342" s="9" t="s">
+        <v>664</v>
+      </c>
+      <c r="P342" s="16" t="s">
+        <v>1128</v>
+      </c>
+      <c r="Q342" s="9" t="s">
+        <v>569</v>
+      </c>
+      <c r="R342" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="S342" s="17">
+        <f t="shared" si="123"/>
+        <v>293</v>
+      </c>
+      <c r="T342" s="17">
+        <v>0</v>
+      </c>
     </row>
     <row r="343" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A343" s="13"/>

</xml_diff>

<commit_message>
#47 Reading List: updated to 2025-06-12.
</commit_message>
<xml_diff>
--- a/data/Reading List.xlsx
+++ b/data/Reading List.xlsx
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5310" uniqueCount="1129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5382" uniqueCount="1146">
   <si>
     <t>Format</t>
   </si>
@@ -3428,6 +3428,57 @@
   </si>
   <si>
     <t>Useless. This book dedicates only few pages at the beginning about Streamlit, and then talks about random Python libraries for the rest of the book. Additionally, instead of using textual code listings, it shows them as screenshots with small font and black background, making them unreadable.</t>
+  </si>
+  <si>
+    <t>UX Fundamentals for Non-UX Professionals</t>
+  </si>
+  <si>
+    <t>2025-05-29</t>
+  </si>
+  <si>
+    <t>Useful. It contains minimally useful advices, but it would be a better book if stripped down of all the random facts.</t>
+  </si>
+  <si>
+    <t>Web Automation Testing Using Playwright</t>
+  </si>
+  <si>
+    <t>2025-05-30</t>
+  </si>
+  <si>
+    <t>Useful. Ok as a basic Getting Started guide, but nothing more. Due of all the repetitions and the redudancy, it could be shrinked by 75% without loss of information.</t>
+  </si>
+  <si>
+    <t>Colorwise</t>
+  </si>
+  <si>
+    <t>Useful. It contains some useful hints, but it's definitely not a breakthrough book.</t>
+  </si>
+  <si>
+    <t>Ultimate Figma For UI/UX Design</t>
+  </si>
+  <si>
+    <t>2025-06-06</t>
+  </si>
+  <si>
+    <t>Useless. Just a list of Figma Features and random design principles as bullet points.</t>
+  </si>
+  <si>
+    <t>English For Programmers</t>
+  </si>
+  <si>
+    <t>2025-06-12</t>
+  </si>
+  <si>
+    <t>Useful. A good idea and first iteration, hopefully additional iterations with more pages will come.</t>
+  </si>
+  <si>
+    <t>Power Up Product Management</t>
+  </si>
+  <si>
+    <t>Routledge</t>
+  </si>
+  <si>
+    <t>Useful. Ok as a Getting Started book for beginners.</t>
   </si>
 </sst>
 </file>
@@ -11245,7 +11296,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet5"/>
-  <dimension ref="A1:T356"/>
+  <dimension ref="A1:T365"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="57.42578125" style="1" customWidth="1"/>
@@ -31668,7 +31719,7 @@
         <v>159</v>
       </c>
       <c r="S314" s="17">
-        <f t="shared" ref="S314:S342" si="123">LEN(P314)</f>
+        <f t="shared" ref="S314:S348" si="123">LEN(P314)</f>
         <v>35</v>
       </c>
       <c r="T314" s="49">
@@ -32958,7 +33009,7 @@
       <c r="O334" s="9" t="s">
         <v>664</v>
       </c>
-      <c r="P334" s="13" t="s">
+      <c r="P334" s="16" t="s">
         <v>1108</v>
       </c>
       <c r="Q334" s="9" t="s">
@@ -33496,139 +33547,397 @@
       </c>
     </row>
     <row r="343" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A343" s="13"/>
-      <c r="B343" s="9"/>
-      <c r="C343" s="9"/>
-      <c r="D343" s="9"/>
-      <c r="E343" s="9"/>
-      <c r="F343" s="9"/>
-      <c r="G343" s="9"/>
-      <c r="H343" s="9"/>
-      <c r="I343" s="9"/>
-      <c r="J343" s="9"/>
-      <c r="K343" s="9"/>
-      <c r="L343" s="9"/>
-      <c r="M343" s="9"/>
-      <c r="N343" s="9"/>
-      <c r="O343" s="9"/>
-      <c r="P343" s="13"/>
-      <c r="Q343" s="9"/>
-      <c r="R343" s="9"/>
-      <c r="S343" s="17"/>
-      <c r="T343" s="9"/>
+      <c r="A343" s="13" t="s">
+        <v>1129</v>
+      </c>
+      <c r="B343" s="17">
+        <v>2018</v>
+      </c>
+      <c r="C343" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D343" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E343" s="9" t="s">
+        <v>666</v>
+      </c>
+      <c r="F343" s="17">
+        <v>331</v>
+      </c>
+      <c r="G343" s="9" t="s">
+        <v>1130</v>
+      </c>
+      <c r="H343" s="9">
+        <f t="shared" ref="H343" si="167">YEAR(G343)</f>
+        <v>2025</v>
+      </c>
+      <c r="I343" s="9">
+        <f t="shared" ref="I343" si="168">MONTH(G343)</f>
+        <v>5</v>
+      </c>
+      <c r="J343" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="K343" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="L343" s="9" t="s">
+        <v>372</v>
+      </c>
+      <c r="M343" s="17">
+        <v>2</v>
+      </c>
+      <c r="N343" s="17">
+        <v>64.989999999999995</v>
+      </c>
+      <c r="O343" s="9" t="s">
+        <v>664</v>
+      </c>
+      <c r="P343" s="16" t="s">
+        <v>1131</v>
+      </c>
+      <c r="Q343" s="9" t="s">
+        <v>1107</v>
+      </c>
+      <c r="R343" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="S343" s="17">
+        <f t="shared" si="123"/>
+        <v>117</v>
+      </c>
+      <c r="T343" s="17">
+        <v>0</v>
+      </c>
     </row>
     <row r="344" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A344" s="13"/>
-      <c r="B344" s="9"/>
-      <c r="C344" s="9"/>
-      <c r="D344" s="9"/>
-      <c r="E344" s="9"/>
-      <c r="F344" s="9"/>
-      <c r="G344" s="9"/>
-      <c r="H344" s="9"/>
-      <c r="I344" s="9"/>
-      <c r="J344" s="9"/>
-      <c r="K344" s="9"/>
-      <c r="L344" s="9"/>
-      <c r="M344" s="9"/>
-      <c r="N344" s="9"/>
-      <c r="O344" s="9"/>
-      <c r="P344" s="13"/>
-      <c r="Q344" s="9"/>
-      <c r="R344" s="9"/>
-      <c r="S344" s="17"/>
-      <c r="T344" s="9"/>
+      <c r="A344" s="13" t="s">
+        <v>1132</v>
+      </c>
+      <c r="B344" s="17">
+        <v>2025</v>
+      </c>
+      <c r="C344" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D344" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E344" s="9" t="s">
+        <v>666</v>
+      </c>
+      <c r="F344" s="17">
+        <v>433</v>
+      </c>
+      <c r="G344" s="9" t="s">
+        <v>1133</v>
+      </c>
+      <c r="H344" s="9">
+        <f t="shared" ref="H344" si="169">YEAR(G344)</f>
+        <v>2025</v>
+      </c>
+      <c r="I344" s="9">
+        <f t="shared" ref="I344" si="170">MONTH(G344)</f>
+        <v>5</v>
+      </c>
+      <c r="J344" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="K344" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="L344" s="9" t="s">
+        <v>880</v>
+      </c>
+      <c r="M344" s="17">
+        <v>2</v>
+      </c>
+      <c r="N344" s="17">
+        <v>39.950000000000003</v>
+      </c>
+      <c r="O344" s="9" t="s">
+        <v>664</v>
+      </c>
+      <c r="P344" s="16" t="s">
+        <v>1134</v>
+      </c>
+      <c r="Q344" s="9" t="s">
+        <v>469</v>
+      </c>
+      <c r="R344" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="S344" s="17">
+        <f t="shared" si="123"/>
+        <v>165</v>
+      </c>
+      <c r="T344" s="17">
+        <v>0</v>
+      </c>
     </row>
     <row r="345" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A345" s="13"/>
-      <c r="B345" s="9"/>
-      <c r="C345" s="9"/>
-      <c r="D345" s="9"/>
-      <c r="E345" s="9"/>
-      <c r="F345" s="9"/>
-      <c r="G345" s="9"/>
-      <c r="H345" s="9"/>
-      <c r="I345" s="9"/>
-      <c r="J345" s="9"/>
-      <c r="K345" s="9"/>
-      <c r="L345" s="9"/>
-      <c r="M345" s="9"/>
-      <c r="N345" s="9"/>
-      <c r="O345" s="9"/>
-      <c r="P345" s="13"/>
-      <c r="Q345" s="9"/>
-      <c r="R345" s="9"/>
-      <c r="S345" s="17"/>
-      <c r="T345" s="9"/>
+      <c r="A345" s="13" t="s">
+        <v>1135</v>
+      </c>
+      <c r="B345" s="17">
+        <v>2023</v>
+      </c>
+      <c r="C345" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D345" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E345" s="9" t="s">
+        <v>666</v>
+      </c>
+      <c r="F345" s="17">
+        <v>168</v>
+      </c>
+      <c r="G345" s="9" t="s">
+        <v>1133</v>
+      </c>
+      <c r="H345" s="9">
+        <f t="shared" ref="H345" si="171">YEAR(G345)</f>
+        <v>2025</v>
+      </c>
+      <c r="I345" s="9">
+        <f t="shared" ref="I345" si="172">MONTH(G345)</f>
+        <v>5</v>
+      </c>
+      <c r="J345" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="K345" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="L345" s="9" t="s">
+        <v>367</v>
+      </c>
+      <c r="M345" s="17">
+        <v>2</v>
+      </c>
+      <c r="N345" s="17">
+        <v>35.99</v>
+      </c>
+      <c r="O345" s="9" t="s">
+        <v>664</v>
+      </c>
+      <c r="P345" s="13" t="s">
+        <v>1136</v>
+      </c>
+      <c r="Q345" s="9" t="s">
+        <v>1107</v>
+      </c>
+      <c r="R345" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="S345" s="17">
+        <f t="shared" si="123"/>
+        <v>83</v>
+      </c>
+      <c r="T345" s="17">
+        <v>0</v>
+      </c>
     </row>
     <row r="346" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A346" s="13"/>
-      <c r="B346" s="9"/>
-      <c r="C346" s="9"/>
-      <c r="D346" s="9"/>
-      <c r="E346" s="9"/>
-      <c r="F346" s="9"/>
-      <c r="G346" s="9"/>
-      <c r="H346" s="9"/>
-      <c r="I346" s="9"/>
-      <c r="J346" s="9"/>
-      <c r="K346" s="9"/>
-      <c r="L346" s="9"/>
-      <c r="M346" s="9"/>
-      <c r="N346" s="9"/>
-      <c r="O346" s="9"/>
-      <c r="P346" s="13"/>
-      <c r="Q346" s="9"/>
-      <c r="R346" s="9"/>
-      <c r="S346" s="17"/>
-      <c r="T346" s="9"/>
+      <c r="A346" s="13" t="s">
+        <v>1137</v>
+      </c>
+      <c r="B346" s="17">
+        <v>2025</v>
+      </c>
+      <c r="C346" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D346" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E346" s="9" t="s">
+        <v>666</v>
+      </c>
+      <c r="F346" s="17">
+        <v>345</v>
+      </c>
+      <c r="G346" s="9" t="s">
+        <v>1138</v>
+      </c>
+      <c r="H346" s="9">
+        <f t="shared" ref="H346" si="173">YEAR(G346)</f>
+        <v>2025</v>
+      </c>
+      <c r="I346" s="9">
+        <f t="shared" ref="I346" si="174">MONTH(G346)</f>
+        <v>6</v>
+      </c>
+      <c r="J346" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="K346" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="L346" s="9" t="s">
+        <v>1113</v>
+      </c>
+      <c r="M346" s="17">
+        <v>2</v>
+      </c>
+      <c r="N346" s="17">
+        <v>37.950000000000003</v>
+      </c>
+      <c r="O346" s="9" t="s">
+        <v>664</v>
+      </c>
+      <c r="P346" s="13" t="s">
+        <v>1139</v>
+      </c>
+      <c r="Q346" s="9" t="s">
+        <v>1107</v>
+      </c>
+      <c r="R346" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="S346" s="17">
+        <f t="shared" si="123"/>
+        <v>85</v>
+      </c>
+      <c r="T346" s="17">
+        <v>0</v>
+      </c>
     </row>
     <row r="347" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A347" s="9"/>
-      <c r="B347" s="9"/>
-      <c r="C347" s="9"/>
-      <c r="D347" s="9"/>
-      <c r="E347" s="9"/>
-      <c r="F347" s="9"/>
-      <c r="G347" s="9"/>
-      <c r="H347" s="9"/>
-      <c r="I347" s="9"/>
-      <c r="J347" s="9"/>
-      <c r="K347" s="9"/>
-      <c r="L347" s="9"/>
-      <c r="M347" s="9"/>
-      <c r="N347" s="9"/>
-      <c r="O347" s="9"/>
-      <c r="P347" s="9"/>
-      <c r="Q347" s="9"/>
-      <c r="R347" s="9"/>
-      <c r="S347" s="17"/>
-      <c r="T347" s="9"/>
+      <c r="A347" s="13" t="s">
+        <v>1140</v>
+      </c>
+      <c r="B347" s="17">
+        <v>2024</v>
+      </c>
+      <c r="C347" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D347" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E347" s="9" t="s">
+        <v>666</v>
+      </c>
+      <c r="F347" s="17">
+        <v>59</v>
+      </c>
+      <c r="G347" s="9" t="s">
+        <v>1141</v>
+      </c>
+      <c r="H347" s="9">
+        <f t="shared" ref="H347" si="175">YEAR(G347)</f>
+        <v>2025</v>
+      </c>
+      <c r="I347" s="9">
+        <f t="shared" ref="I347" si="176">MONTH(G347)</f>
+        <v>6</v>
+      </c>
+      <c r="J347" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="K347" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="L347" s="9" t="s">
+        <v>602</v>
+      </c>
+      <c r="M347" s="17">
+        <v>3</v>
+      </c>
+      <c r="N347" s="17">
+        <v>49.99</v>
+      </c>
+      <c r="O347" s="9" t="s">
+        <v>664</v>
+      </c>
+      <c r="P347" s="13" t="s">
+        <v>1142</v>
+      </c>
+      <c r="Q347" s="9" t="s">
+        <v>876</v>
+      </c>
+      <c r="R347" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="S347" s="17">
+        <f t="shared" si="123"/>
+        <v>99</v>
+      </c>
+      <c r="T347" s="17">
+        <v>0</v>
+      </c>
     </row>
     <row r="348" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A348" s="9"/>
-      <c r="B348" s="9"/>
-      <c r="C348" s="9"/>
-      <c r="D348" s="9"/>
-      <c r="E348" s="9"/>
-      <c r="F348" s="9"/>
-      <c r="G348" s="9"/>
-      <c r="H348" s="9"/>
-      <c r="I348" s="9"/>
-      <c r="J348" s="9"/>
-      <c r="K348" s="9"/>
-      <c r="L348" s="9"/>
-      <c r="M348" s="9"/>
-      <c r="N348" s="9"/>
-      <c r="O348" s="9"/>
-      <c r="P348" s="9"/>
-      <c r="Q348" s="9"/>
-      <c r="R348" s="9"/>
-      <c r="S348" s="17"/>
-      <c r="T348" s="9"/>
+      <c r="A348" s="13" t="s">
+        <v>1143</v>
+      </c>
+      <c r="B348" s="17">
+        <v>2025</v>
+      </c>
+      <c r="C348" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D348" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E348" s="9" t="s">
+        <v>666</v>
+      </c>
+      <c r="F348" s="17">
+        <v>160</v>
+      </c>
+      <c r="G348" s="9" t="s">
+        <v>1141</v>
+      </c>
+      <c r="H348" s="9">
+        <f t="shared" ref="H348" si="177">YEAR(G348)</f>
+        <v>2025</v>
+      </c>
+      <c r="I348" s="9">
+        <f t="shared" ref="I348" si="178">MONTH(G348)</f>
+        <v>6</v>
+      </c>
+      <c r="J348" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="K348" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="L348" s="9" t="s">
+        <v>1144</v>
+      </c>
+      <c r="M348" s="17">
+        <v>3</v>
+      </c>
+      <c r="N348" s="17">
+        <v>42.99</v>
+      </c>
+      <c r="O348" s="9" t="s">
+        <v>664</v>
+      </c>
+      <c r="P348" s="13" t="s">
+        <v>1145</v>
+      </c>
+      <c r="Q348" s="9" t="s">
+        <v>962</v>
+      </c>
+      <c r="R348" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="S348" s="17">
+        <f t="shared" si="123"/>
+        <v>51</v>
+      </c>
+      <c r="T348" s="17">
+        <v>0</v>
+      </c>
     </row>
     <row r="349" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A349" s="9"/>
+      <c r="A349" s="13"/>
       <c r="B349" s="9"/>
       <c r="C349" s="9"/>
       <c r="D349" s="9"/>
@@ -33643,14 +33952,14 @@
       <c r="M349" s="9"/>
       <c r="N349" s="9"/>
       <c r="O349" s="9"/>
-      <c r="P349" s="9"/>
+      <c r="P349" s="13"/>
       <c r="Q349" s="9"/>
       <c r="R349" s="9"/>
       <c r="S349" s="17"/>
       <c r="T349" s="9"/>
     </row>
     <row r="350" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A350" s="9"/>
+      <c r="A350" s="13"/>
       <c r="B350" s="9"/>
       <c r="C350" s="9"/>
       <c r="D350" s="9"/>
@@ -33665,14 +33974,14 @@
       <c r="M350" s="9"/>
       <c r="N350" s="9"/>
       <c r="O350" s="9"/>
-      <c r="P350" s="9"/>
+      <c r="P350" s="13"/>
       <c r="Q350" s="9"/>
       <c r="R350" s="9"/>
       <c r="S350" s="17"/>
       <c r="T350" s="9"/>
     </row>
     <row r="351" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A351" s="9"/>
+      <c r="A351" s="13"/>
       <c r="B351" s="9"/>
       <c r="C351" s="9"/>
       <c r="D351" s="9"/>
@@ -33687,14 +33996,14 @@
       <c r="M351" s="9"/>
       <c r="N351" s="9"/>
       <c r="O351" s="9"/>
-      <c r="P351" s="9"/>
+      <c r="P351" s="13"/>
       <c r="Q351" s="9"/>
       <c r="R351" s="9"/>
       <c r="S351" s="17"/>
       <c r="T351" s="9"/>
     </row>
     <row r="352" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A352" s="9"/>
+      <c r="A352" s="13"/>
       <c r="B352" s="9"/>
       <c r="C352" s="9"/>
       <c r="D352" s="9"/>
@@ -33709,14 +34018,14 @@
       <c r="M352" s="9"/>
       <c r="N352" s="9"/>
       <c r="O352" s="9"/>
-      <c r="P352" s="9"/>
+      <c r="P352" s="13"/>
       <c r="Q352" s="9"/>
       <c r="R352" s="9"/>
       <c r="S352" s="17"/>
       <c r="T352" s="9"/>
     </row>
     <row r="353" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A353" s="9"/>
+      <c r="A353" s="13"/>
       <c r="B353" s="9"/>
       <c r="C353" s="9"/>
       <c r="D353" s="9"/>
@@ -33731,14 +34040,14 @@
       <c r="M353" s="9"/>
       <c r="N353" s="9"/>
       <c r="O353" s="9"/>
-      <c r="P353" s="9"/>
+      <c r="P353" s="13"/>
       <c r="Q353" s="9"/>
       <c r="R353" s="9"/>
       <c r="S353" s="17"/>
       <c r="T353" s="9"/>
     </row>
     <row r="354" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A354" s="9"/>
+      <c r="A354" s="13"/>
       <c r="B354" s="9"/>
       <c r="C354" s="9"/>
       <c r="D354" s="9"/>
@@ -33753,14 +34062,14 @@
       <c r="M354" s="9"/>
       <c r="N354" s="9"/>
       <c r="O354" s="9"/>
-      <c r="P354" s="9"/>
+      <c r="P354" s="13"/>
       <c r="Q354" s="9"/>
       <c r="R354" s="9"/>
       <c r="S354" s="17"/>
       <c r="T354" s="9"/>
     </row>
     <row r="355" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A355" s="9"/>
+      <c r="A355" s="13"/>
       <c r="B355" s="9"/>
       <c r="C355" s="9"/>
       <c r="D355" s="9"/>
@@ -33775,14 +34084,14 @@
       <c r="M355" s="9"/>
       <c r="N355" s="9"/>
       <c r="O355" s="9"/>
-      <c r="P355" s="9"/>
+      <c r="P355" s="13"/>
       <c r="Q355" s="9"/>
       <c r="R355" s="9"/>
       <c r="S355" s="17"/>
       <c r="T355" s="9"/>
     </row>
     <row r="356" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A356" s="9"/>
+      <c r="A356" s="13"/>
       <c r="B356" s="9"/>
       <c r="C356" s="9"/>
       <c r="D356" s="9"/>
@@ -33797,11 +34106,209 @@
       <c r="M356" s="9"/>
       <c r="N356" s="9"/>
       <c r="O356" s="9"/>
-      <c r="P356" s="9"/>
+      <c r="P356" s="13"/>
       <c r="Q356" s="9"/>
       <c r="R356" s="9"/>
       <c r="S356" s="17"/>
       <c r="T356" s="9"/>
+    </row>
+    <row r="357" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A357" s="9"/>
+      <c r="B357" s="9"/>
+      <c r="C357" s="9"/>
+      <c r="D357" s="9"/>
+      <c r="E357" s="9"/>
+      <c r="F357" s="9"/>
+      <c r="G357" s="9"/>
+      <c r="H357" s="9"/>
+      <c r="I357" s="9"/>
+      <c r="J357" s="9"/>
+      <c r="K357" s="9"/>
+      <c r="L357" s="9"/>
+      <c r="M357" s="9"/>
+      <c r="N357" s="9"/>
+      <c r="O357" s="9"/>
+      <c r="P357" s="9"/>
+      <c r="Q357" s="9"/>
+      <c r="R357" s="9"/>
+      <c r="S357" s="17"/>
+      <c r="T357" s="9"/>
+    </row>
+    <row r="358" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A358" s="9"/>
+      <c r="B358" s="9"/>
+      <c r="C358" s="9"/>
+      <c r="D358" s="9"/>
+      <c r="E358" s="9"/>
+      <c r="F358" s="9"/>
+      <c r="G358" s="9"/>
+      <c r="H358" s="9"/>
+      <c r="I358" s="9"/>
+      <c r="J358" s="9"/>
+      <c r="K358" s="9"/>
+      <c r="L358" s="9"/>
+      <c r="M358" s="9"/>
+      <c r="N358" s="9"/>
+      <c r="O358" s="9"/>
+      <c r="P358" s="9"/>
+      <c r="Q358" s="9"/>
+      <c r="R358" s="9"/>
+      <c r="S358" s="17"/>
+      <c r="T358" s="9"/>
+    </row>
+    <row r="359" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A359" s="9"/>
+      <c r="B359" s="9"/>
+      <c r="C359" s="9"/>
+      <c r="D359" s="9"/>
+      <c r="E359" s="9"/>
+      <c r="F359" s="9"/>
+      <c r="G359" s="9"/>
+      <c r="H359" s="9"/>
+      <c r="I359" s="9"/>
+      <c r="J359" s="9"/>
+      <c r="K359" s="9"/>
+      <c r="L359" s="9"/>
+      <c r="M359" s="9"/>
+      <c r="N359" s="9"/>
+      <c r="O359" s="9"/>
+      <c r="P359" s="9"/>
+      <c r="Q359" s="9"/>
+      <c r="R359" s="9"/>
+      <c r="S359" s="17"/>
+      <c r="T359" s="9"/>
+    </row>
+    <row r="360" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A360" s="9"/>
+      <c r="B360" s="9"/>
+      <c r="C360" s="9"/>
+      <c r="D360" s="9"/>
+      <c r="E360" s="9"/>
+      <c r="F360" s="9"/>
+      <c r="G360" s="9"/>
+      <c r="H360" s="9"/>
+      <c r="I360" s="9"/>
+      <c r="J360" s="9"/>
+      <c r="K360" s="9"/>
+      <c r="L360" s="9"/>
+      <c r="M360" s="9"/>
+      <c r="N360" s="9"/>
+      <c r="O360" s="9"/>
+      <c r="P360" s="9"/>
+      <c r="Q360" s="9"/>
+      <c r="R360" s="9"/>
+      <c r="S360" s="17"/>
+      <c r="T360" s="9"/>
+    </row>
+    <row r="361" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A361" s="9"/>
+      <c r="B361" s="9"/>
+      <c r="C361" s="9"/>
+      <c r="D361" s="9"/>
+      <c r="E361" s="9"/>
+      <c r="F361" s="9"/>
+      <c r="G361" s="9"/>
+      <c r="H361" s="9"/>
+      <c r="I361" s="9"/>
+      <c r="J361" s="9"/>
+      <c r="K361" s="9"/>
+      <c r="L361" s="9"/>
+      <c r="M361" s="9"/>
+      <c r="N361" s="9"/>
+      <c r="O361" s="9"/>
+      <c r="P361" s="9"/>
+      <c r="Q361" s="9"/>
+      <c r="R361" s="9"/>
+      <c r="S361" s="17"/>
+      <c r="T361" s="9"/>
+    </row>
+    <row r="362" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A362" s="9"/>
+      <c r="B362" s="9"/>
+      <c r="C362" s="9"/>
+      <c r="D362" s="9"/>
+      <c r="E362" s="9"/>
+      <c r="F362" s="9"/>
+      <c r="G362" s="9"/>
+      <c r="H362" s="9"/>
+      <c r="I362" s="9"/>
+      <c r="J362" s="9"/>
+      <c r="K362" s="9"/>
+      <c r="L362" s="9"/>
+      <c r="M362" s="9"/>
+      <c r="N362" s="9"/>
+      <c r="O362" s="9"/>
+      <c r="P362" s="9"/>
+      <c r="Q362" s="9"/>
+      <c r="R362" s="9"/>
+      <c r="S362" s="17"/>
+      <c r="T362" s="9"/>
+    </row>
+    <row r="363" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A363" s="9"/>
+      <c r="B363" s="9"/>
+      <c r="C363" s="9"/>
+      <c r="D363" s="9"/>
+      <c r="E363" s="9"/>
+      <c r="F363" s="9"/>
+      <c r="G363" s="9"/>
+      <c r="H363" s="9"/>
+      <c r="I363" s="9"/>
+      <c r="J363" s="9"/>
+      <c r="K363" s="9"/>
+      <c r="L363" s="9"/>
+      <c r="M363" s="9"/>
+      <c r="N363" s="9"/>
+      <c r="O363" s="9"/>
+      <c r="P363" s="9"/>
+      <c r="Q363" s="9"/>
+      <c r="R363" s="9"/>
+      <c r="S363" s="17"/>
+      <c r="T363" s="9"/>
+    </row>
+    <row r="364" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A364" s="9"/>
+      <c r="B364" s="9"/>
+      <c r="C364" s="9"/>
+      <c r="D364" s="9"/>
+      <c r="E364" s="9"/>
+      <c r="F364" s="9"/>
+      <c r="G364" s="9"/>
+      <c r="H364" s="9"/>
+      <c r="I364" s="9"/>
+      <c r="J364" s="9"/>
+      <c r="K364" s="9"/>
+      <c r="L364" s="9"/>
+      <c r="M364" s="9"/>
+      <c r="N364" s="9"/>
+      <c r="O364" s="9"/>
+      <c r="P364" s="9"/>
+      <c r="Q364" s="9"/>
+      <c r="R364" s="9"/>
+      <c r="S364" s="17"/>
+      <c r="T364" s="9"/>
+    </row>
+    <row r="365" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A365" s="9"/>
+      <c r="B365" s="9"/>
+      <c r="C365" s="9"/>
+      <c r="D365" s="9"/>
+      <c r="E365" s="9"/>
+      <c r="F365" s="9"/>
+      <c r="G365" s="9"/>
+      <c r="H365" s="9"/>
+      <c r="I365" s="9"/>
+      <c r="J365" s="9"/>
+      <c r="K365" s="9"/>
+      <c r="L365" s="9"/>
+      <c r="M365" s="9"/>
+      <c r="N365" s="9"/>
+      <c r="O365" s="9"/>
+      <c r="P365" s="9"/>
+      <c r="Q365" s="9"/>
+      <c r="R365" s="9"/>
+      <c r="S365" s="17"/>
+      <c r="T365" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
#47 Reading List: updated to 2025-07-13.
</commit_message>
<xml_diff>
--- a/data/Reading List.xlsx
+++ b/data/Reading List.xlsx
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5382" uniqueCount="1146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5442" uniqueCount="1159">
   <si>
     <t>Format</t>
   </si>
@@ -3479,6 +3479,45 @@
   </si>
   <si>
     <t>Useful. Ok as a Getting Started book for beginners.</t>
+  </si>
+  <si>
+    <t>Safe 5.0 Distilled</t>
+  </si>
+  <si>
+    <t>2025-06-26</t>
+  </si>
+  <si>
+    <t>Useful. Quite repetitive but ok as introductory book.</t>
+  </si>
+  <si>
+    <t>Command Line Handbook</t>
+  </si>
+  <si>
+    <t>2025-06-27</t>
+  </si>
+  <si>
+    <t>Competing With Unicorns</t>
+  </si>
+  <si>
+    <t>Useless. Not a bad book, but mostly for beginners.</t>
+  </si>
+  <si>
+    <t>2025-07-03</t>
+  </si>
+  <si>
+    <t>Developer Experience Unleashed</t>
+  </si>
+  <si>
+    <t>Building LLMs for Production</t>
+  </si>
+  <si>
+    <t>2025-07-11</t>
+  </si>
+  <si>
+    <t>Useless. Well-written but painfully redundant - 80% of the content could be easily removed or summarized without loss of knowledge.</t>
+  </si>
+  <si>
+    <t>Useless. Just a list of concepts and Python modules without any personality. Very boring.</t>
   </si>
 </sst>
 </file>
@@ -31719,7 +31758,7 @@
         <v>159</v>
       </c>
       <c r="S314" s="17">
-        <f t="shared" ref="S314:S348" si="123">LEN(P314)</f>
+        <f t="shared" ref="S314:S353" si="123">LEN(P314)</f>
         <v>35</v>
       </c>
       <c r="T314" s="49">
@@ -33937,114 +33976,329 @@
       </c>
     </row>
     <row r="349" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A349" s="13"/>
-      <c r="B349" s="9"/>
-      <c r="C349" s="9"/>
-      <c r="D349" s="9"/>
-      <c r="E349" s="9"/>
-      <c r="F349" s="9"/>
-      <c r="G349" s="9"/>
-      <c r="H349" s="9"/>
-      <c r="I349" s="9"/>
-      <c r="J349" s="9"/>
-      <c r="K349" s="9"/>
-      <c r="L349" s="9"/>
-      <c r="M349" s="9"/>
-      <c r="N349" s="9"/>
-      <c r="O349" s="9"/>
-      <c r="P349" s="13"/>
-      <c r="Q349" s="9"/>
-      <c r="R349" s="9"/>
-      <c r="S349" s="17"/>
-      <c r="T349" s="9"/>
+      <c r="A349" s="13" t="s">
+        <v>1146</v>
+      </c>
+      <c r="B349" s="17">
+        <v>2020</v>
+      </c>
+      <c r="C349" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D349" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E349" s="9" t="s">
+        <v>666</v>
+      </c>
+      <c r="F349" s="17">
+        <v>321</v>
+      </c>
+      <c r="G349" s="9" t="s">
+        <v>1147</v>
+      </c>
+      <c r="H349" s="9">
+        <f t="shared" ref="H349" si="179">YEAR(G349)</f>
+        <v>2025</v>
+      </c>
+      <c r="I349" s="9">
+        <f t="shared" ref="I349" si="180">MONTH(G349)</f>
+        <v>6</v>
+      </c>
+      <c r="J349" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="K349" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="L349" s="9" t="s">
+        <v>370</v>
+      </c>
+      <c r="M349" s="17">
+        <v>3</v>
+      </c>
+      <c r="N349" s="17">
+        <v>38.58</v>
+      </c>
+      <c r="O349" s="9" t="s">
+        <v>664</v>
+      </c>
+      <c r="P349" s="13" t="s">
+        <v>1148</v>
+      </c>
+      <c r="Q349" s="9" t="s">
+        <v>962</v>
+      </c>
+      <c r="R349" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="S349" s="17">
+        <f t="shared" si="123"/>
+        <v>53</v>
+      </c>
+      <c r="T349" s="17">
+        <v>0</v>
+      </c>
     </row>
     <row r="350" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A350" s="13"/>
-      <c r="B350" s="9"/>
-      <c r="C350" s="9"/>
-      <c r="D350" s="9"/>
-      <c r="E350" s="9"/>
-      <c r="F350" s="9"/>
-      <c r="G350" s="9"/>
-      <c r="H350" s="9"/>
-      <c r="I350" s="9"/>
-      <c r="J350" s="9"/>
-      <c r="K350" s="9"/>
-      <c r="L350" s="9"/>
-      <c r="M350" s="9"/>
-      <c r="N350" s="9"/>
-      <c r="O350" s="9"/>
-      <c r="P350" s="13"/>
-      <c r="Q350" s="9"/>
-      <c r="R350" s="9"/>
-      <c r="S350" s="17"/>
-      <c r="T350" s="9"/>
+      <c r="A350" s="13" t="s">
+        <v>1149</v>
+      </c>
+      <c r="B350" s="17">
+        <v>2025</v>
+      </c>
+      <c r="C350" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D350" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E350" s="9" t="s">
+        <v>666</v>
+      </c>
+      <c r="F350" s="17">
+        <v>123</v>
+      </c>
+      <c r="G350" s="9" t="s">
+        <v>1150</v>
+      </c>
+      <c r="H350" s="9">
+        <f t="shared" ref="H350" si="181">YEAR(G350)</f>
+        <v>2025</v>
+      </c>
+      <c r="I350" s="9">
+        <f t="shared" ref="I350" si="182">MONTH(G350)</f>
+        <v>6</v>
+      </c>
+      <c r="J350" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="K350" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="L350" s="9" t="s">
+        <v>602</v>
+      </c>
+      <c r="M350" s="17">
+        <v>2</v>
+      </c>
+      <c r="N350" s="43">
+        <v>0</v>
+      </c>
+      <c r="O350" s="9" t="s">
+        <v>664</v>
+      </c>
+      <c r="P350" s="13" t="s">
+        <v>1152</v>
+      </c>
+      <c r="Q350" s="9" t="s">
+        <v>501</v>
+      </c>
+      <c r="R350" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="S350" s="17">
+        <f t="shared" si="123"/>
+        <v>50</v>
+      </c>
+      <c r="T350" s="17">
+        <v>0</v>
+      </c>
     </row>
     <row r="351" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A351" s="13"/>
-      <c r="B351" s="9"/>
-      <c r="C351" s="9"/>
-      <c r="D351" s="9"/>
-      <c r="E351" s="9"/>
-      <c r="F351" s="9"/>
-      <c r="G351" s="9"/>
-      <c r="H351" s="9"/>
-      <c r="I351" s="9"/>
-      <c r="J351" s="9"/>
-      <c r="K351" s="9"/>
-      <c r="L351" s="9"/>
-      <c r="M351" s="9"/>
-      <c r="N351" s="9"/>
-      <c r="O351" s="9"/>
-      <c r="P351" s="13"/>
-      <c r="Q351" s="9"/>
-      <c r="R351" s="9"/>
-      <c r="S351" s="17"/>
-      <c r="T351" s="9"/>
+      <c r="A351" s="13" t="s">
+        <v>1151</v>
+      </c>
+      <c r="B351" s="17">
+        <v>2020</v>
+      </c>
+      <c r="C351" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D351" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E351" s="9" t="s">
+        <v>666</v>
+      </c>
+      <c r="F351" s="17">
+        <v>131</v>
+      </c>
+      <c r="G351" s="9" t="s">
+        <v>1153</v>
+      </c>
+      <c r="H351" s="9">
+        <f t="shared" ref="H351" si="183">YEAR(G351)</f>
+        <v>2025</v>
+      </c>
+      <c r="I351" s="9">
+        <f t="shared" ref="I351" si="184">MONTH(G351)</f>
+        <v>7</v>
+      </c>
+      <c r="J351" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="K351" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="L351" s="9" t="s">
+        <v>386</v>
+      </c>
+      <c r="M351" s="17">
+        <v>3</v>
+      </c>
+      <c r="N351" s="17">
+        <v>26.95</v>
+      </c>
+      <c r="O351" s="9" t="s">
+        <v>664</v>
+      </c>
+      <c r="P351" s="13" t="s">
+        <v>674</v>
+      </c>
+      <c r="Q351" s="9" t="s">
+        <v>962</v>
+      </c>
+      <c r="R351" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="S351" s="17">
+        <f t="shared" si="123"/>
+        <v>16</v>
+      </c>
+      <c r="T351" s="17">
+        <v>0</v>
+      </c>
     </row>
     <row r="352" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A352" s="13"/>
-      <c r="B352" s="9"/>
-      <c r="C352" s="9"/>
-      <c r="D352" s="9"/>
-      <c r="E352" s="9"/>
-      <c r="F352" s="9"/>
-      <c r="G352" s="9"/>
-      <c r="H352" s="9"/>
-      <c r="I352" s="9"/>
-      <c r="J352" s="9"/>
-      <c r="K352" s="9"/>
-      <c r="L352" s="9"/>
-      <c r="M352" s="9"/>
-      <c r="N352" s="9"/>
-      <c r="O352" s="9"/>
-      <c r="P352" s="13"/>
-      <c r="Q352" s="9"/>
-      <c r="R352" s="9"/>
-      <c r="S352" s="17"/>
-      <c r="T352" s="9"/>
+      <c r="A352" s="13" t="s">
+        <v>1154</v>
+      </c>
+      <c r="B352" s="17">
+        <v>2025</v>
+      </c>
+      <c r="C352" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D352" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E352" s="9" t="s">
+        <v>666</v>
+      </c>
+      <c r="F352" s="17">
+        <v>485</v>
+      </c>
+      <c r="G352" s="9" t="s">
+        <v>1153</v>
+      </c>
+      <c r="H352" s="9">
+        <f t="shared" ref="H352" si="185">YEAR(G352)</f>
+        <v>2025</v>
+      </c>
+      <c r="I352" s="9">
+        <f t="shared" ref="I352" si="186">MONTH(G352)</f>
+        <v>7</v>
+      </c>
+      <c r="J352" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="K352" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="L352" s="9" t="s">
+        <v>372</v>
+      </c>
+      <c r="M352" s="17">
+        <v>2</v>
+      </c>
+      <c r="N352" s="17">
+        <v>38.89</v>
+      </c>
+      <c r="O352" s="9" t="s">
+        <v>664</v>
+      </c>
+      <c r="P352" s="13" t="s">
+        <v>1157</v>
+      </c>
+      <c r="Q352" s="9" t="s">
+        <v>962</v>
+      </c>
+      <c r="R352" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="S352" s="17">
+        <f t="shared" si="123"/>
+        <v>131</v>
+      </c>
+      <c r="T352" s="17">
+        <v>0</v>
+      </c>
     </row>
     <row r="353" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A353" s="13"/>
-      <c r="B353" s="9"/>
-      <c r="C353" s="9"/>
-      <c r="D353" s="9"/>
-      <c r="E353" s="9"/>
-      <c r="F353" s="9"/>
-      <c r="G353" s="9"/>
-      <c r="H353" s="9"/>
-      <c r="I353" s="9"/>
-      <c r="J353" s="9"/>
-      <c r="K353" s="9"/>
-      <c r="L353" s="9"/>
-      <c r="M353" s="9"/>
-      <c r="N353" s="9"/>
-      <c r="O353" s="9"/>
-      <c r="P353" s="13"/>
-      <c r="Q353" s="9"/>
-      <c r="R353" s="9"/>
-      <c r="S353" s="17"/>
-      <c r="T353" s="9"/>
+      <c r="A353" s="13" t="s">
+        <v>1155</v>
+      </c>
+      <c r="B353" s="17">
+        <v>2024</v>
+      </c>
+      <c r="C353" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D353" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E353" s="9" t="s">
+        <v>666</v>
+      </c>
+      <c r="F353" s="17">
+        <v>569</v>
+      </c>
+      <c r="G353" s="9" t="s">
+        <v>1156</v>
+      </c>
+      <c r="H353" s="9">
+        <f t="shared" ref="H353" si="187">YEAR(G353)</f>
+        <v>2025</v>
+      </c>
+      <c r="I353" s="9">
+        <f t="shared" ref="I353" si="188">MONTH(G353)</f>
+        <v>7</v>
+      </c>
+      <c r="J353" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="K353" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="L353" s="9" t="s">
+        <v>602</v>
+      </c>
+      <c r="M353" s="17">
+        <v>2</v>
+      </c>
+      <c r="N353" s="17">
+        <v>58.99</v>
+      </c>
+      <c r="O353" s="9" t="s">
+        <v>664</v>
+      </c>
+      <c r="P353" s="13" t="s">
+        <v>1158</v>
+      </c>
+      <c r="Q353" s="9" t="s">
+        <v>958</v>
+      </c>
+      <c r="R353" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="S353" s="17">
+        <f t="shared" si="123"/>
+        <v>89</v>
+      </c>
+      <c r="T353" s="17">
+        <v>0</v>
+      </c>
     </row>
     <row r="354" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A354" s="13"/>

</xml_diff>

<commit_message>
#47 Reading List: updated to 2025-08-12.
</commit_message>
<xml_diff>
--- a/data/Reading List.xlsx
+++ b/data/Reading List.xlsx
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5442" uniqueCount="1159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5478" uniqueCount="1167">
   <si>
     <t>Format</t>
   </si>
@@ -3518,6 +3518,30 @@
   </si>
   <si>
     <t>Useless. Just a list of concepts and Python modules without any personality. Very boring.</t>
+  </si>
+  <si>
+    <t>The Art of PostgreSQL (2nd Edition)</t>
+  </si>
+  <si>
+    <t>2025-07-17</t>
+  </si>
+  <si>
+    <t>Useless. A very unstructured book: perhaps there is a logic but it makes sense only in the author's mind. The selection of topics is very random and brings low value to the reader, and some frustration too.</t>
+  </si>
+  <si>
+    <t>The Data Scientist's Toolkit</t>
+  </si>
+  <si>
+    <t>2025-07-18</t>
+  </si>
+  <si>
+    <t>Useful. An excellent showcase of less known Python libraries and techniques to solve several common problems. Very original approach and very concise writing.</t>
+  </si>
+  <si>
+    <t>Clean Architecture with Python</t>
+  </si>
+  <si>
+    <t>2025-08-12</t>
   </si>
 </sst>
 </file>
@@ -3663,7 +3687,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3808,6 +3832,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -31758,7 +31788,7 @@
         <v>159</v>
       </c>
       <c r="S314" s="17">
-        <f t="shared" ref="S314:S353" si="123">LEN(P314)</f>
+        <f t="shared" ref="S314:S356" si="123">LEN(P314)</f>
         <v>35</v>
       </c>
       <c r="T314" s="49">
@@ -34301,70 +34331,199 @@
       </c>
     </row>
     <row r="354" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A354" s="13"/>
-      <c r="B354" s="9"/>
-      <c r="C354" s="9"/>
-      <c r="D354" s="9"/>
-      <c r="E354" s="9"/>
-      <c r="F354" s="9"/>
-      <c r="G354" s="9"/>
-      <c r="H354" s="9"/>
-      <c r="I354" s="9"/>
-      <c r="J354" s="9"/>
-      <c r="K354" s="9"/>
-      <c r="L354" s="9"/>
-      <c r="M354" s="9"/>
-      <c r="N354" s="9"/>
-      <c r="O354" s="9"/>
-      <c r="P354" s="13"/>
-      <c r="Q354" s="9"/>
-      <c r="R354" s="9"/>
-      <c r="S354" s="17"/>
-      <c r="T354" s="9"/>
+      <c r="A354" s="13" t="s">
+        <v>1159</v>
+      </c>
+      <c r="B354" s="17">
+        <v>2024</v>
+      </c>
+      <c r="C354" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D354" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E354" s="9" t="s">
+        <v>666</v>
+      </c>
+      <c r="F354" s="17">
+        <v>236</v>
+      </c>
+      <c r="G354" s="9" t="s">
+        <v>1160</v>
+      </c>
+      <c r="H354" s="9">
+        <f t="shared" ref="H354" si="189">YEAR(G354)</f>
+        <v>2025</v>
+      </c>
+      <c r="I354" s="9">
+        <f t="shared" ref="I354" si="190">MONTH(G354)</f>
+        <v>7</v>
+      </c>
+      <c r="J354" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="K354" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="L354" s="9" t="s">
+        <v>602</v>
+      </c>
+      <c r="M354" s="17">
+        <v>1</v>
+      </c>
+      <c r="N354" s="17">
+        <v>129</v>
+      </c>
+      <c r="O354" s="9" t="s">
+        <v>664</v>
+      </c>
+      <c r="P354" s="16" t="s">
+        <v>1161</v>
+      </c>
+      <c r="Q354" s="9" t="s">
+        <v>903</v>
+      </c>
+      <c r="R354" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="S354" s="17">
+        <f t="shared" si="123"/>
+        <v>206</v>
+      </c>
+      <c r="T354" s="17">
+        <v>0</v>
+      </c>
     </row>
     <row r="355" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A355" s="13"/>
-      <c r="B355" s="9"/>
-      <c r="C355" s="9"/>
-      <c r="D355" s="9"/>
-      <c r="E355" s="9"/>
-      <c r="F355" s="9"/>
-      <c r="G355" s="9"/>
-      <c r="H355" s="9"/>
-      <c r="I355" s="9"/>
-      <c r="J355" s="9"/>
-      <c r="K355" s="9"/>
-      <c r="L355" s="9"/>
-      <c r="M355" s="9"/>
-      <c r="N355" s="9"/>
-      <c r="O355" s="9"/>
-      <c r="P355" s="13"/>
-      <c r="Q355" s="9"/>
-      <c r="R355" s="9"/>
-      <c r="S355" s="17"/>
-      <c r="T355" s="9"/>
+      <c r="A355" s="13" t="s">
+        <v>1162</v>
+      </c>
+      <c r="B355" s="17">
+        <v>2024</v>
+      </c>
+      <c r="C355" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D355" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E355" s="9" t="s">
+        <v>666</v>
+      </c>
+      <c r="F355" s="17">
+        <v>265</v>
+      </c>
+      <c r="G355" s="9" t="s">
+        <v>1163</v>
+      </c>
+      <c r="H355" s="9">
+        <f t="shared" ref="H355:H356" si="191">YEAR(G355)</f>
+        <v>2025</v>
+      </c>
+      <c r="I355" s="9">
+        <f t="shared" ref="I355:I356" si="192">MONTH(G355)</f>
+        <v>7</v>
+      </c>
+      <c r="J355" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="K355" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="L355" s="9" t="s">
+        <v>602</v>
+      </c>
+      <c r="M355" s="17">
+        <v>5</v>
+      </c>
+      <c r="N355" s="43">
+        <v>0</v>
+      </c>
+      <c r="O355" s="9" t="s">
+        <v>664</v>
+      </c>
+      <c r="P355" s="16" t="s">
+        <v>1164</v>
+      </c>
+      <c r="Q355" s="9" t="s">
+        <v>903</v>
+      </c>
+      <c r="R355" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="S355" s="17">
+        <f t="shared" si="123"/>
+        <v>158</v>
+      </c>
+      <c r="T355" s="17">
+        <v>0</v>
+      </c>
     </row>
     <row r="356" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A356" s="13"/>
-      <c r="B356" s="9"/>
-      <c r="C356" s="9"/>
-      <c r="D356" s="9"/>
-      <c r="E356" s="9"/>
-      <c r="F356" s="9"/>
-      <c r="G356" s="9"/>
-      <c r="H356" s="9"/>
-      <c r="I356" s="9"/>
-      <c r="J356" s="9"/>
-      <c r="K356" s="9"/>
-      <c r="L356" s="9"/>
-      <c r="M356" s="9"/>
-      <c r="N356" s="9"/>
-      <c r="O356" s="9"/>
-      <c r="P356" s="13"/>
-      <c r="Q356" s="9"/>
-      <c r="R356" s="9"/>
-      <c r="S356" s="17"/>
-      <c r="T356" s="9"/>
+      <c r="A356" s="13" t="s">
+        <v>1165</v>
+      </c>
+      <c r="B356" s="17">
+        <v>2025</v>
+      </c>
+      <c r="C356" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D356" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E356" s="9" t="s">
+        <v>666</v>
+      </c>
+      <c r="F356" s="17">
+        <v>362</v>
+      </c>
+      <c r="G356" s="53" t="s">
+        <v>1166</v>
+      </c>
+      <c r="H356" s="9">
+        <f t="shared" si="191"/>
+        <v>2025</v>
+      </c>
+      <c r="I356" s="9">
+        <f t="shared" si="192"/>
+        <v>8</v>
+      </c>
+      <c r="J356" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="K356" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="L356" s="9" t="s">
+        <v>365</v>
+      </c>
+      <c r="M356" s="50">
+        <v>3</v>
+      </c>
+      <c r="N356" s="17">
+        <v>44.99</v>
+      </c>
+      <c r="O356" s="9" t="s">
+        <v>664</v>
+      </c>
+      <c r="P356" s="54" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q356" s="9" t="s">
+        <v>569</v>
+      </c>
+      <c r="R356" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="S356" s="17">
+        <f t="shared" si="123"/>
+        <v>8</v>
+      </c>
+      <c r="T356" s="17">
+        <v>0</v>
+      </c>
     </row>
     <row r="357" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A357" s="9"/>

</xml_diff>

<commit_message>
#47 Reading List: updated 08/09/2025.
</commit_message>
<xml_diff>
--- a/data/Reading List.xlsx
+++ b/data/Reading List.xlsx
@@ -15584,7 +15584,7 @@
         <v>143</v>
       </c>
       <c r="T66" s="10">
-        <v>956</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="67" spans="1:20" x14ac:dyDescent="0.2">
@@ -17209,7 +17209,7 @@
         <v>108</v>
       </c>
       <c r="T91" s="10">
-        <v>298</v>
+        <v>300</v>
       </c>
     </row>
     <row r="92" spans="1:20" x14ac:dyDescent="0.2">
@@ -23773,7 +23773,7 @@
         <v>8</v>
       </c>
       <c r="T192" s="10">
-        <v>2016</v>
+        <v>1977</v>
       </c>
     </row>
     <row r="193" spans="1:20" x14ac:dyDescent="0.2">
@@ -23838,7 +23838,7 @@
         <v>21</v>
       </c>
       <c r="T193" s="10">
-        <v>0</v>
+        <v>482</v>
       </c>
     </row>
     <row r="194" spans="1:20" x14ac:dyDescent="0.2">
@@ -23903,7 +23903,7 @@
         <v>24</v>
       </c>
       <c r="T194" s="10">
-        <v>353</v>
+        <v>348</v>
       </c>
     </row>
     <row r="195" spans="1:20" x14ac:dyDescent="0.2">
@@ -23968,7 +23968,7 @@
         <v>155</v>
       </c>
       <c r="T195" s="10">
-        <v>364</v>
+        <v>392</v>
       </c>
     </row>
     <row r="196" spans="1:20" x14ac:dyDescent="0.2">
@@ -24293,7 +24293,7 @@
         <v>16</v>
       </c>
       <c r="T200" s="10">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="201" spans="1:20" x14ac:dyDescent="0.2">
@@ -24618,7 +24618,7 @@
         <v>16</v>
       </c>
       <c r="T205" s="10">
-        <v>155</v>
+        <v>152</v>
       </c>
     </row>
     <row r="206" spans="1:20" x14ac:dyDescent="0.2">
@@ -24748,7 +24748,7 @@
         <v>17</v>
       </c>
       <c r="T207" s="10">
-        <v>1354</v>
+        <v>150</v>
       </c>
     </row>
     <row r="208" spans="1:20" x14ac:dyDescent="0.2">
@@ -25073,7 +25073,7 @@
         <v>149</v>
       </c>
       <c r="T212" s="10">
-        <v>520</v>
+        <v>512</v>
       </c>
     </row>
     <row r="213" spans="1:20" x14ac:dyDescent="0.2">
@@ -25463,7 +25463,7 @@
         <v>77</v>
       </c>
       <c r="T218" s="10">
-        <v>1242</v>
+        <v>1247</v>
       </c>
     </row>
     <row r="219" spans="1:20" x14ac:dyDescent="0.2">
@@ -26048,7 +26048,7 @@
         <v>16</v>
       </c>
       <c r="T227" s="10">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="228" spans="1:20" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
#47 Reading List: updated to 2025-11-10.
</commit_message>
<xml_diff>
--- a/data/Reading List.xlsx
+++ b/data/Reading List.xlsx
@@ -11287,7 +11287,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr codeName="Sheet5" filterMode="1"/>
+  <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:T367"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
   <cols>
@@ -11374,7 +11374,7 @@
         <v>882</v>
       </c>
     </row>
-    <row r="2" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A2" s="7" t="s">
         <v>3</v>
       </c>
@@ -11439,7 +11439,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="3" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A3" s="7" t="s">
         <v>6</v>
       </c>
@@ -11501,10 +11501,10 @@
         <v>7</v>
       </c>
       <c r="T3" s="10">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="4" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="s">
         <v>10</v>
       </c>
@@ -11569,7 +11569,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="5" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
         <v>582</v>
       </c>
@@ -11634,7 +11634,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
         <v>13</v>
       </c>
@@ -11699,7 +11699,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="7" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
         <v>14</v>
       </c>
@@ -11764,7 +11764,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="8" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
         <v>15</v>
       </c>
@@ -11826,10 +11826,10 @@
         <v>115</v>
       </c>
       <c r="T8" s="10">
-        <v>535</v>
-      </c>
-    </row>
-    <row r="9" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A9" s="7" t="s">
         <v>17</v>
       </c>
@@ -11894,7 +11894,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="10" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A10" s="7" t="s">
         <v>19</v>
       </c>
@@ -11959,7 +11959,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="11" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A11" s="7" t="s">
         <v>22</v>
       </c>
@@ -12024,7 +12024,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="12" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A12" s="7" t="s">
         <v>33</v>
       </c>
@@ -12089,7 +12089,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="13" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="s">
         <v>62</v>
       </c>
@@ -12154,7 +12154,7 @@
         <v>2142</v>
       </c>
     </row>
-    <row r="14" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A14" s="7" t="s">
         <v>63</v>
       </c>
@@ -12219,7 +12219,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="15" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A15" s="7" t="s">
         <v>70</v>
       </c>
@@ -12284,7 +12284,7 @@
         <v>1063</v>
       </c>
     </row>
-    <row r="16" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A16" s="7" t="s">
         <v>73</v>
       </c>
@@ -12349,7 +12349,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="17" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A17" s="7" t="s">
         <v>1152</v>
       </c>
@@ -12414,7 +12414,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="18" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A18" s="7" t="s">
         <v>82</v>
       </c>
@@ -12479,7 +12479,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A19" s="7" t="s">
         <v>1153</v>
       </c>
@@ -12544,7 +12544,7 @@
         <v>1373</v>
       </c>
     </row>
-    <row r="20" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A20" s="7" t="s">
         <v>89</v>
       </c>
@@ -12609,7 +12609,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="21" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A21" s="7" t="s">
         <v>97</v>
       </c>
@@ -12674,7 +12674,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="22" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="s">
         <v>100</v>
       </c>
@@ -12739,7 +12739,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="23" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A23" s="7" t="s">
         <v>101</v>
       </c>
@@ -12804,7 +12804,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A24" s="7" t="s">
         <v>103</v>
       </c>
@@ -12869,7 +12869,7 @@
         <v>852</v>
       </c>
     </row>
-    <row r="25" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A25" s="7" t="s">
         <v>105</v>
       </c>
@@ -12934,7 +12934,7 @@
         <v>1545</v>
       </c>
     </row>
-    <row r="26" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A26" s="7" t="s">
         <v>107</v>
       </c>
@@ -12999,7 +12999,7 @@
         <v>2271</v>
       </c>
     </row>
-    <row r="27" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A27" s="7" t="s">
         <v>109</v>
       </c>
@@ -13064,7 +13064,7 @@
         <v>1418</v>
       </c>
     </row>
-    <row r="28" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A28" s="7" t="s">
         <v>115</v>
       </c>
@@ -13129,7 +13129,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="29" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A29" s="7" t="s">
         <v>117</v>
       </c>
@@ -13194,7 +13194,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A30" s="7" t="s">
         <v>119</v>
       </c>
@@ -13259,7 +13259,7 @@
         <v>999</v>
       </c>
     </row>
-    <row r="31" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="s">
         <v>121</v>
       </c>
@@ -13324,7 +13324,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="32" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A32" s="7" t="s">
         <v>123</v>
       </c>
@@ -13389,7 +13389,7 @@
         <v>1547</v>
       </c>
     </row>
-    <row r="33" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A33" s="7" t="s">
         <v>125</v>
       </c>
@@ -13454,7 +13454,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="34" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A34" s="7" t="s">
         <v>126</v>
       </c>
@@ -13519,7 +13519,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="35" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A35" s="7" t="s">
         <v>128</v>
       </c>
@@ -13584,7 +13584,7 @@
         <v>788</v>
       </c>
     </row>
-    <row r="36" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A36" s="7" t="s">
         <v>130</v>
       </c>
@@ -13649,7 +13649,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A37" s="7" t="s">
         <v>1144</v>
       </c>
@@ -13714,7 +13714,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="38" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A38" s="7" t="s">
         <v>132</v>
       </c>
@@ -13779,7 +13779,7 @@
         <v>1361</v>
       </c>
     </row>
-    <row r="39" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A39" s="7" t="s">
         <v>136</v>
       </c>
@@ -13844,7 +13844,7 @@
         <v>2313</v>
       </c>
     </row>
-    <row r="40" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="s">
         <v>138</v>
       </c>
@@ -13909,7 +13909,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="41" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A41" s="7" t="s">
         <v>1154</v>
       </c>
@@ -13974,7 +13974,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="42" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A42" s="7" t="s">
         <v>1155</v>
       </c>
@@ -14039,7 +14039,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="43" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A43" s="7" t="s">
         <v>140</v>
       </c>
@@ -14104,7 +14104,7 @@
         <v>538</v>
       </c>
     </row>
-    <row r="44" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A44" s="7" t="s">
         <v>141</v>
       </c>
@@ -14169,7 +14169,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="45" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A45" s="7" t="s">
         <v>146</v>
       </c>
@@ -14234,7 +14234,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="46" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A46" s="7" t="s">
         <v>148</v>
       </c>
@@ -14299,7 +14299,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="47" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A47" s="7" t="s">
         <v>149</v>
       </c>
@@ -14364,7 +14364,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A48" s="7" t="s">
         <v>150</v>
       </c>
@@ -14429,7 +14429,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="49" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="s">
         <v>151</v>
       </c>
@@ -14494,7 +14494,7 @@
         <v>855</v>
       </c>
     </row>
-    <row r="50" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A50" s="7" t="s">
         <v>1156</v>
       </c>
@@ -14559,7 +14559,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="51" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A51" s="7" t="s">
         <v>361</v>
       </c>
@@ -14689,7 +14689,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="53" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A53" s="7" t="s">
         <v>1145</v>
       </c>
@@ -14754,7 +14754,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="54" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A54" s="7" t="s">
         <v>1157</v>
       </c>
@@ -14819,7 +14819,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="55" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A55" s="7" t="s">
         <v>158</v>
       </c>
@@ -14884,7 +14884,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="56" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A56" s="7" t="s">
         <v>1146</v>
       </c>
@@ -14949,7 +14949,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="57" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A57" s="7" t="s">
         <v>159</v>
       </c>
@@ -15014,7 +15014,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="58" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="s">
         <v>363</v>
       </c>
@@ -15079,7 +15079,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A59" s="7" t="s">
         <v>166</v>
       </c>
@@ -15144,7 +15144,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="60" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A60" s="7" t="s">
         <v>174</v>
       </c>
@@ -15209,7 +15209,7 @@
         <v>1780</v>
       </c>
     </row>
-    <row r="61" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A61" s="7" t="s">
         <v>176</v>
       </c>
@@ -15274,7 +15274,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="62" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A62" s="7" t="s">
         <v>178</v>
       </c>
@@ -15339,7 +15339,7 @@
         <v>1048</v>
       </c>
     </row>
-    <row r="63" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A63" s="7" t="s">
         <v>179</v>
       </c>
@@ -15404,7 +15404,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="64" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A64" s="7" t="s">
         <v>181</v>
       </c>
@@ -15469,7 +15469,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="65" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A65" s="7" t="s">
         <v>182</v>
       </c>
@@ -15534,7 +15534,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="66" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A66" s="7" t="s">
         <v>1147</v>
       </c>
@@ -15599,7 +15599,7 @@
         <v>1340</v>
       </c>
     </row>
-    <row r="67" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="s">
         <v>185</v>
       </c>
@@ -15664,7 +15664,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="68" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A68" s="7" t="s">
         <v>186</v>
       </c>
@@ -15729,7 +15729,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="69" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A69" s="7" t="s">
         <v>187</v>
       </c>
@@ -15859,7 +15859,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="71" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A71" s="7" t="s">
         <v>190</v>
       </c>
@@ -15924,7 +15924,7 @@
         <v>946</v>
       </c>
     </row>
-    <row r="72" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A72" s="7" t="s">
         <v>192</v>
       </c>
@@ -15989,7 +15989,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="73" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A73" s="7" t="s">
         <v>194</v>
       </c>
@@ -16054,7 +16054,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="74" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A74" s="7" t="s">
         <v>197</v>
       </c>
@@ -16119,7 +16119,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="75" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A75" s="7" t="s">
         <v>1159</v>
       </c>
@@ -16184,7 +16184,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="76" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="s">
         <v>217</v>
       </c>
@@ -16249,7 +16249,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="77" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A77" s="7" t="s">
         <v>199</v>
       </c>
@@ -16314,7 +16314,7 @@
         <v>1014</v>
       </c>
     </row>
-    <row r="78" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A78" s="7" t="s">
         <v>200</v>
       </c>
@@ -16379,7 +16379,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="79" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A79" s="7" t="s">
         <v>202</v>
       </c>
@@ -16444,7 +16444,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="80" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A80" s="7" t="s">
         <v>208</v>
       </c>
@@ -16509,7 +16509,7 @@
         <v>1448</v>
       </c>
     </row>
-    <row r="81" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A81" s="7" t="s">
         <v>1148</v>
       </c>
@@ -16574,7 +16574,7 @@
         <v>1004</v>
       </c>
     </row>
-    <row r="82" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A82" s="7" t="s">
         <v>1149</v>
       </c>
@@ -16639,7 +16639,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="83" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A83" s="7" t="s">
         <v>215</v>
       </c>
@@ -16704,7 +16704,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="84" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A84" s="7" t="s">
         <v>1162</v>
       </c>
@@ -16769,7 +16769,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="85" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A85" s="7" t="s">
         <v>816</v>
       </c>
@@ -16834,7 +16834,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="86" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A86" s="7" t="s">
         <v>1160</v>
       </c>
@@ -16899,7 +16899,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="87" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A87" s="7" t="s">
         <v>1161</v>
       </c>
@@ -16964,7 +16964,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="88" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A88" s="7" t="s">
         <v>222</v>
       </c>
@@ -17029,7 +17029,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="89" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A89" s="7" t="s">
         <v>223</v>
       </c>
@@ -17094,7 +17094,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A90" s="7" t="s">
         <v>225</v>
       </c>
@@ -17159,7 +17159,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A91" s="7" t="s">
         <v>227</v>
       </c>
@@ -17224,7 +17224,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="92" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A92" s="7" t="s">
         <v>229</v>
       </c>
@@ -17289,7 +17289,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="93" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A93" s="7" t="s">
         <v>566</v>
       </c>
@@ -17354,7 +17354,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="94" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A94" s="7" t="s">
         <v>231</v>
       </c>
@@ -17419,7 +17419,7 @@
         <v>752</v>
       </c>
     </row>
-    <row r="95" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A95" s="7" t="s">
         <v>233</v>
       </c>
@@ -17484,7 +17484,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="96" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A96" s="7" t="s">
         <v>235</v>
       </c>
@@ -17549,7 +17549,7 @@
         <v>960</v>
       </c>
     </row>
-    <row r="97" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A97" s="7" t="s">
         <v>237</v>
       </c>
@@ -17614,7 +17614,7 @@
         <v>1184</v>
       </c>
     </row>
-    <row r="98" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A98" s="7" t="s">
         <v>239</v>
       </c>
@@ -17679,7 +17679,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="99" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A99" s="7" t="s">
         <v>240</v>
       </c>
@@ -17744,7 +17744,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A100" s="12" t="s">
         <v>1158</v>
       </c>
@@ -17809,7 +17809,7 @@
         <v>1641</v>
       </c>
     </row>
-    <row r="101" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A101" s="7" t="s">
         <v>246</v>
       </c>
@@ -17874,7 +17874,7 @@
         <v>1379</v>
       </c>
     </row>
-    <row r="102" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A102" s="7" t="s">
         <v>248</v>
       </c>
@@ -17939,7 +17939,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="103" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A103" s="7" t="s">
         <v>250</v>
       </c>
@@ -18004,7 +18004,7 @@
         <v>3732</v>
       </c>
     </row>
-    <row r="104" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A104" s="7" t="s">
         <v>252</v>
       </c>
@@ -18069,7 +18069,7 @@
         <v>3272</v>
       </c>
     </row>
-    <row r="105" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A105" s="7" t="s">
         <v>256</v>
       </c>
@@ -18134,7 +18134,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="106" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A106" s="7" t="s">
         <v>254</v>
       </c>
@@ -18199,7 +18199,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A107" s="7" t="s">
         <v>1165</v>
       </c>
@@ -18264,7 +18264,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="108" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A108" s="7" t="s">
         <v>1167</v>
       </c>
@@ -18329,7 +18329,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="109" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A109" s="7" t="s">
         <v>285</v>
       </c>
@@ -18394,7 +18394,7 @@
         <v>864</v>
       </c>
     </row>
-    <row r="110" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A110" s="7" t="s">
         <v>286</v>
       </c>
@@ -18459,7 +18459,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="111" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A111" s="7" t="s">
         <v>289</v>
       </c>
@@ -18524,7 +18524,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="112" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A112" s="7" t="s">
         <v>292</v>
       </c>
@@ -18589,7 +18589,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="113" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A113" s="7" t="s">
         <v>294</v>
       </c>
@@ -18914,7 +18914,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="118" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A118" s="7" t="s">
         <v>302</v>
       </c>
@@ -18979,7 +18979,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="119" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A119" s="7" t="s">
         <v>194</v>
       </c>
@@ -19044,7 +19044,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="120" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A120" s="7" t="s">
         <v>303</v>
       </c>
@@ -19109,7 +19109,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="121" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A121" s="7" t="s">
         <v>305</v>
       </c>
@@ -19174,7 +19174,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="122" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A122" s="7" t="s">
         <v>403</v>
       </c>
@@ -19238,7 +19238,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A123" s="7" t="s">
         <v>324</v>
       </c>
@@ -19303,7 +19303,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="124" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A124" s="7" t="s">
         <v>326</v>
       </c>
@@ -19368,7 +19368,7 @@
         <v>963</v>
       </c>
     </row>
-    <row r="125" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A125" s="7" t="s">
         <v>818</v>
       </c>
@@ -19433,7 +19433,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="126" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A126" s="7" t="s">
         <v>329</v>
       </c>
@@ -19498,7 +19498,7 @@
         <v>932</v>
       </c>
     </row>
-    <row r="127" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A127" s="7" t="s">
         <v>331</v>
       </c>
@@ -19563,7 +19563,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="128" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A128" s="7" t="s">
         <v>332</v>
       </c>
@@ -19628,7 +19628,7 @@
         <v>782</v>
       </c>
     </row>
-    <row r="129" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A129" s="7" t="s">
         <v>320</v>
       </c>
@@ -19693,7 +19693,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="130" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A130" s="7" t="s">
         <v>319</v>
       </c>
@@ -19758,7 +19758,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="131" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A131" s="7" t="s">
         <v>322</v>
       </c>
@@ -19823,7 +19823,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A132" s="7" t="s">
         <v>1168</v>
       </c>
@@ -19888,7 +19888,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="133" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A133" s="7" t="s">
         <v>321</v>
       </c>
@@ -19953,7 +19953,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="134" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A134" s="7" t="s">
         <v>323</v>
       </c>
@@ -20148,7 +20148,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="137" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A137" s="7" t="s">
         <v>315</v>
       </c>
@@ -20213,7 +20213,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="138" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A138" s="7" t="s">
         <v>316</v>
       </c>
@@ -20278,7 +20278,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="139" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A139" s="7" t="s">
         <v>317</v>
       </c>
@@ -20343,7 +20343,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="140" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A140" s="7" t="s">
         <v>313</v>
       </c>
@@ -20408,7 +20408,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="141" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A141" s="7" t="s">
         <v>318</v>
       </c>
@@ -20473,7 +20473,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="142" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A142" s="7" t="s">
         <v>314</v>
       </c>
@@ -20538,7 +20538,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="143" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A143" s="7" t="s">
         <v>379</v>
       </c>
@@ -20603,7 +20603,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="144" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A144" s="7" t="s">
         <v>381</v>
       </c>
@@ -20668,7 +20668,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="145" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A145" s="7" t="s">
         <v>382</v>
       </c>
@@ -20733,7 +20733,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="146" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A146" s="7" t="s">
         <v>384</v>
       </c>
@@ -20798,7 +20798,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="147" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A147" s="7" t="s">
         <v>386</v>
       </c>
@@ -20863,7 +20863,7 @@
         <v>989</v>
       </c>
     </row>
-    <row r="148" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A148" s="7" t="s">
         <v>387</v>
       </c>
@@ -20928,7 +20928,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="149" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A149" s="7" t="s">
         <v>389</v>
       </c>
@@ -20993,7 +20993,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="150" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A150" s="7" t="s">
         <v>391</v>
       </c>
@@ -21058,7 +21058,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="151" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A151" s="7" t="s">
         <v>393</v>
       </c>
@@ -21123,7 +21123,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="152" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A152" s="7" t="s">
         <v>395</v>
       </c>
@@ -21188,7 +21188,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A153" s="7" t="s">
         <v>396</v>
       </c>
@@ -21253,7 +21253,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="154" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A154" s="7" t="s">
         <v>398</v>
       </c>
@@ -21318,7 +21318,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="155" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A155" s="7" t="s">
         <v>399</v>
       </c>
@@ -21383,7 +21383,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="156" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A156" s="7" t="s">
         <v>401</v>
       </c>
@@ -21448,7 +21448,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A157" s="7" t="s">
         <v>405</v>
       </c>
@@ -21513,7 +21513,7 @@
         <v>1028</v>
       </c>
     </row>
-    <row r="158" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A158" s="7" t="s">
         <v>406</v>
       </c>
@@ -21578,7 +21578,7 @@
         <v>2255</v>
       </c>
     </row>
-    <row r="159" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A159" s="7" t="s">
         <v>407</v>
       </c>
@@ -21643,7 +21643,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="160" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A160" s="7" t="s">
         <v>408</v>
       </c>
@@ -21708,7 +21708,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="161" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A161" s="7" t="s">
         <v>409</v>
       </c>
@@ -21773,7 +21773,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="162" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A162" s="7" t="s">
         <v>410</v>
       </c>
@@ -21838,7 +21838,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="163" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A163" s="7" t="s">
         <v>411</v>
       </c>
@@ -21903,7 +21903,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="164" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A164" s="7" t="s">
         <v>412</v>
       </c>
@@ -21968,7 +21968,7 @@
         <v>2320</v>
       </c>
     </row>
-    <row r="165" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A165" s="7" t="s">
         <v>413</v>
       </c>
@@ -22033,7 +22033,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="166" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A166" s="7" t="s">
         <v>414</v>
       </c>
@@ -22098,7 +22098,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="167" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A167" s="7" t="s">
         <v>415</v>
       </c>
@@ -22228,7 +22228,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A169" s="7" t="s">
         <v>417</v>
       </c>
@@ -22293,7 +22293,7 @@
         <v>817</v>
       </c>
     </row>
-    <row r="170" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A170" s="7" t="s">
         <v>418</v>
       </c>
@@ -22358,7 +22358,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="171" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A171" s="7" t="s">
         <v>419</v>
       </c>
@@ -22423,7 +22423,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="172" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A172" s="7" t="s">
         <v>420</v>
       </c>
@@ -22488,7 +22488,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="173" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A173" s="7" t="s">
         <v>421</v>
       </c>
@@ -22553,7 +22553,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A174" s="7" t="s">
         <v>422</v>
       </c>
@@ -22618,7 +22618,7 @@
         <v>1679</v>
       </c>
     </row>
-    <row r="175" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A175" s="7" t="s">
         <v>423</v>
       </c>
@@ -22683,7 +22683,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A176" s="7" t="s">
         <v>424</v>
       </c>
@@ -22748,7 +22748,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="177" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A177" s="7" t="s">
         <v>440</v>
       </c>
@@ -22813,7 +22813,7 @@
         <v>852</v>
       </c>
     </row>
-    <row r="178" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A178" s="7" t="s">
         <v>442</v>
       </c>
@@ -22878,7 +22878,7 @@
         <v>856</v>
       </c>
     </row>
-    <row r="179" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A179" s="7" t="s">
         <v>1151</v>
       </c>
@@ -22943,7 +22943,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="180" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A180" s="7" t="s">
         <v>443</v>
       </c>
@@ -23008,7 +23008,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="181" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A181" s="7" t="s">
         <v>466</v>
       </c>
@@ -23138,7 +23138,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="183" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A183" s="7" t="s">
         <v>468</v>
       </c>
@@ -23203,7 +23203,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A184" s="7" t="s">
         <v>470</v>
       </c>
@@ -23268,7 +23268,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="185" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A185" s="7" t="s">
         <v>471</v>
       </c>
@@ -23333,7 +23333,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="186" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A186" s="7" t="s">
         <v>472</v>
       </c>
@@ -23398,7 +23398,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="187" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A187" s="12" t="s">
         <v>473</v>
       </c>
@@ -23463,7 +23463,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="188" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A188" s="12" t="s">
         <v>475</v>
       </c>
@@ -23528,7 +23528,7 @@
         <v>835</v>
       </c>
     </row>
-    <row r="189" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A189" s="7" t="s">
         <v>476</v>
       </c>
@@ -23593,7 +23593,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="190" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A190" s="7" t="s">
         <v>479</v>
       </c>
@@ -23658,7 +23658,7 @@
         <v>952</v>
       </c>
     </row>
-    <row r="191" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A191" s="7" t="s">
         <v>480</v>
       </c>
@@ -23723,7 +23723,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="192" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A192" s="7" t="s">
         <v>485</v>
       </c>
@@ -23788,7 +23788,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="193" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A193" s="7" t="s">
         <v>486</v>
       </c>
@@ -23853,7 +23853,7 @@
         <v>1352</v>
       </c>
     </row>
-    <row r="194" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A194" s="7" t="s">
         <v>489</v>
       </c>
@@ -23918,7 +23918,7 @@
         <v>1977</v>
       </c>
     </row>
-    <row r="195" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A195" s="7" t="s">
         <v>491</v>
       </c>
@@ -23983,7 +23983,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="196" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A196" s="7" t="s">
         <v>494</v>
       </c>
@@ -24048,7 +24048,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="197" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A197" s="7" t="s">
         <v>496</v>
       </c>
@@ -24113,7 +24113,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="198" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A198" s="7" t="s">
         <v>499</v>
       </c>
@@ -24178,7 +24178,7 @@
         <v>1715</v>
       </c>
     </row>
-    <row r="199" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A199" s="7" t="s">
         <v>533</v>
       </c>
@@ -24243,7 +24243,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="200" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A200" s="7" t="s">
         <v>535</v>
       </c>
@@ -24308,7 +24308,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="201" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A201" s="7" t="s">
         <v>537</v>
       </c>
@@ -24373,7 +24373,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="202" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A202" s="7" t="s">
         <v>540</v>
       </c>
@@ -24438,7 +24438,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="203" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A203" s="7" t="s">
         <v>541</v>
       </c>
@@ -24503,7 +24503,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="204" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A204" s="7" t="s">
         <v>543</v>
       </c>
@@ -24568,7 +24568,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="205" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A205" s="7" t="s">
         <v>544</v>
       </c>
@@ -24633,7 +24633,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="206" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A206" s="7" t="s">
         <v>545</v>
       </c>
@@ -24698,7 +24698,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="207" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A207" s="7" t="s">
         <v>548</v>
       </c>
@@ -24763,7 +24763,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="208" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A208" s="7" t="s">
         <v>553</v>
       </c>
@@ -24828,7 +24828,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="209" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A209" s="7" t="s">
         <v>486</v>
       </c>
@@ -24893,7 +24893,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="210" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A210" s="7" t="s">
         <v>556</v>
       </c>
@@ -24958,7 +24958,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="211" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A211" s="7" t="s">
         <v>557</v>
       </c>
@@ -25023,7 +25023,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="212" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A212" s="7" t="s">
         <v>558</v>
       </c>
@@ -25088,7 +25088,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="213" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A213" s="7" t="s">
         <v>559</v>
       </c>
@@ -25153,7 +25153,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="214" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A214" s="7" t="s">
         <v>560</v>
       </c>
@@ -25218,7 +25218,7 @@
         <v>512</v>
       </c>
     </row>
-    <row r="215" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A215" s="7" t="s">
         <v>561</v>
       </c>
@@ -25283,7 +25283,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="216" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A216" s="7" t="s">
         <v>562</v>
       </c>
@@ -25348,7 +25348,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="217" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A217" s="7" t="s">
         <v>563</v>
       </c>
@@ -25413,7 +25413,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="218" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A218" s="7" t="s">
         <v>564</v>
       </c>
@@ -25478,7 +25478,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="219" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="219" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A219" s="7" t="s">
         <v>565</v>
       </c>
@@ -25543,7 +25543,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="220" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A220" s="7" t="s">
         <v>567</v>
       </c>
@@ -25608,7 +25608,7 @@
         <v>1247</v>
       </c>
     </row>
-    <row r="221" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A221" s="7" t="s">
         <v>588</v>
       </c>
@@ -25673,7 +25673,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="222" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A222" s="7" t="s">
         <v>590</v>
       </c>
@@ -25738,7 +25738,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="223" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A223" s="7" t="s">
         <v>591</v>
       </c>
@@ -25803,7 +25803,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="224" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A224" s="7" t="s">
         <v>593</v>
       </c>
@@ -25868,7 +25868,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="225" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A225" s="7" t="s">
         <v>594</v>
       </c>
@@ -25998,7 +25998,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="227" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A227" s="7" t="s">
         <v>597</v>
       </c>
@@ -26063,7 +26063,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="228" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A228" s="7" t="s">
         <v>599</v>
       </c>
@@ -26128,7 +26128,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="229" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A229" s="7" t="s">
         <v>600</v>
       </c>
@@ -26193,7 +26193,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="230" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A230" s="7" t="s">
         <v>602</v>
       </c>
@@ -26258,7 +26258,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="231" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A231" s="7" t="s">
         <v>603</v>
       </c>
@@ -26323,7 +26323,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="232" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A232" s="7" t="s">
         <v>628</v>
       </c>
@@ -26388,7 +26388,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="233" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A233" s="7" t="s">
         <v>630</v>
       </c>
@@ -26453,7 +26453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="234" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A234" s="7" t="s">
         <v>1170</v>
       </c>
@@ -26518,7 +26518,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="235" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A235" s="7" t="s">
         <v>255</v>
       </c>
@@ -26583,7 +26583,7 @@
         <v>1603</v>
       </c>
     </row>
-    <row r="236" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A236" s="7" t="s">
         <v>632</v>
       </c>
@@ -26648,7 +26648,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="237" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A237" s="7" t="s">
         <v>834</v>
       </c>
@@ -26713,7 +26713,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="238" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A238" s="7" t="s">
         <v>819</v>
       </c>
@@ -26778,7 +26778,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="239" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A239" s="7" t="s">
         <v>822</v>
       </c>
@@ -26843,7 +26843,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="240" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A240" s="7" t="s">
         <v>825</v>
       </c>
@@ -26908,7 +26908,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="241" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A241" s="7" t="s">
         <v>826</v>
       </c>
@@ -26973,7 +26973,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="242" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A242" s="7" t="s">
         <v>827</v>
       </c>
@@ -27038,7 +27038,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="243" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A243" s="7" t="s">
         <v>829</v>
       </c>
@@ -27103,7 +27103,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="244" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A244" s="7" t="s">
         <v>831</v>
       </c>
@@ -27168,7 +27168,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="245" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A245" s="7" t="s">
         <v>838</v>
       </c>
@@ -27233,7 +27233,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="246" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A246" s="7" t="s">
         <v>841</v>
       </c>
@@ -27298,7 +27298,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="247" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A247" s="7" t="s">
         <v>843</v>
       </c>
@@ -27363,7 +27363,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="248" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="248" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A248" s="7" t="s">
         <v>847</v>
       </c>
@@ -27428,7 +27428,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="249" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A249" s="7" t="s">
         <v>855</v>
       </c>
@@ -27493,7 +27493,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="250" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A250" s="7" t="s">
         <v>859</v>
       </c>
@@ -27558,7 +27558,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="251" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="251" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A251" s="7" t="s">
         <v>862</v>
       </c>
@@ -27623,7 +27623,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="252" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A252" s="7" t="s">
         <v>864</v>
       </c>
@@ -27688,7 +27688,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="253" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="253" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A253" s="7" t="s">
         <v>867</v>
       </c>
@@ -27753,7 +27753,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="254" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A254" s="7" t="s">
         <v>869</v>
       </c>
@@ -27818,7 +27818,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="255" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A255" s="7" t="s">
         <v>873</v>
       </c>
@@ -27883,7 +27883,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="256" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="256" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A256" s="7" t="s">
         <v>875</v>
       </c>
@@ -27948,7 +27948,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="257" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="257" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A257" s="7" t="s">
         <v>878</v>
       </c>
@@ -28013,7 +28013,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="258" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="258" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A258" s="7" t="s">
         <v>883</v>
       </c>
@@ -28078,7 +28078,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="259" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="259" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A259" s="7" t="s">
         <v>886</v>
       </c>
@@ -28143,7 +28143,7 @@
         <v>732</v>
       </c>
     </row>
-    <row r="260" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="260" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A260" s="7" t="s">
         <v>898</v>
       </c>
@@ -28208,7 +28208,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="261" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="261" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A261" s="7" t="s">
         <v>897</v>
       </c>
@@ -28273,7 +28273,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="262" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="262" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A262" s="7" t="s">
         <v>892</v>
       </c>
@@ -28338,7 +28338,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="263" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="263" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A263" s="7" t="s">
         <v>895</v>
       </c>
@@ -28403,7 +28403,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="264" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="264" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A264" s="7" t="s">
         <v>899</v>
       </c>
@@ -28468,7 +28468,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="265" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="265" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A265" s="7" t="s">
         <v>902</v>
       </c>
@@ -28533,7 +28533,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="266" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="266" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A266" s="7" t="s">
         <v>904</v>
       </c>
@@ -28598,7 +28598,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="267" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="267" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A267" s="7" t="s">
         <v>1011</v>
       </c>
@@ -28663,7 +28663,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="268" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A268" s="7" t="s">
         <v>907</v>
       </c>
@@ -28728,7 +28728,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="269" spans="1:20" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="269" spans="1:20" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A269" s="7" t="s">
         <v>909</v>
       </c>
@@ -28793,7 +28793,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="270" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="270" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A270" s="7" t="s">
         <v>911</v>
       </c>
@@ -28858,7 +28858,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="271" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A271" s="7" t="s">
         <v>914</v>
       </c>
@@ -28923,7 +28923,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="272" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="272" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A272" s="7" t="s">
         <v>916</v>
       </c>
@@ -28988,7 +28988,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="273" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="273" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A273" s="7" t="s">
         <v>919</v>
       </c>
@@ -29053,7 +29053,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="274" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="274" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A274" s="7" t="s">
         <v>922</v>
       </c>
@@ -29118,7 +29118,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="275" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="275" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A275" s="7" t="s">
         <v>924</v>
       </c>
@@ -29183,7 +29183,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="276" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="276" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A276" s="7" t="s">
         <v>926</v>
       </c>
@@ -29248,7 +29248,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="277" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="277" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A277" s="7" t="s">
         <v>929</v>
       </c>
@@ -29313,7 +29313,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="278" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="278" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A278" s="7" t="s">
         <v>931</v>
       </c>
@@ -29378,7 +29378,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="279" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="279" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A279" s="7" t="s">
         <v>933</v>
       </c>
@@ -29443,7 +29443,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="280" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="280" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A280" s="7" t="s">
         <v>937</v>
       </c>
@@ -29508,7 +29508,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="281" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="281" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A281" s="7" t="s">
         <v>940</v>
       </c>
@@ -29573,7 +29573,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="282" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="282" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A282" s="7" t="s">
         <v>1171</v>
       </c>
@@ -29638,7 +29638,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="283" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="283" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A283" s="7" t="s">
         <v>944</v>
       </c>
@@ -29703,7 +29703,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="284" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="284" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A284" s="7" t="s">
         <v>946</v>
       </c>
@@ -29768,7 +29768,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="285" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="285" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A285" s="7" t="s">
         <v>949</v>
       </c>
@@ -29833,7 +29833,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="286" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="286" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A286" s="7" t="s">
         <v>952</v>
       </c>
@@ -29898,7 +29898,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="287" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="287" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A287" s="7" t="s">
         <v>955</v>
       </c>
@@ -29963,7 +29963,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="288" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="288" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A288" s="7" t="s">
         <v>957</v>
       </c>
@@ -30028,7 +30028,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="289" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="289" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A289" s="7" t="s">
         <v>959</v>
       </c>
@@ -30093,7 +30093,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="290" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="290" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A290" s="7" t="s">
         <v>961</v>
       </c>
@@ -30158,7 +30158,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="291" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="291" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A291" s="7" t="s">
         <v>964</v>
       </c>
@@ -30223,7 +30223,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="292" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="292" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A292" s="7" t="s">
         <v>967</v>
       </c>
@@ -30288,7 +30288,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="293" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="293" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A293" s="7" t="s">
         <v>970</v>
       </c>
@@ -30353,7 +30353,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="294" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="294" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A294" s="7" t="s">
         <v>972</v>
       </c>
@@ -30418,7 +30418,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="295" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="295" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A295" s="7" t="s">
         <v>973</v>
       </c>
@@ -30483,7 +30483,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="296" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="296" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A296" s="7" t="s">
         <v>976</v>
       </c>
@@ -30548,7 +30548,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="297" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="297" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A297" s="7" t="s">
         <v>980</v>
       </c>
@@ -30613,7 +30613,7 @@
         <v>708</v>
       </c>
     </row>
-    <row r="298" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="298" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A298" s="7" t="s">
         <v>983</v>
       </c>
@@ -30678,7 +30678,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="299" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="299" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A299" s="7" t="s">
         <v>986</v>
       </c>
@@ -30743,7 +30743,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="300" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="300" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A300" s="7" t="s">
         <v>989</v>
       </c>
@@ -30808,7 +30808,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="301" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="301" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A301" s="12" t="s">
         <v>991</v>
       </c>
@@ -30873,7 +30873,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="302" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="302" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A302" s="7" t="s">
         <v>993</v>
       </c>
@@ -30938,7 +30938,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="303" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="303" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A303" s="7" t="s">
         <v>996</v>
       </c>
@@ -31003,7 +31003,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="304" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="304" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A304" s="7" t="s">
         <v>998</v>
       </c>
@@ -31068,7 +31068,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="305" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="305" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A305" s="7" t="s">
         <v>1000</v>
       </c>
@@ -31133,7 +31133,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="306" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="306" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A306" s="7" t="s">
         <v>1002</v>
       </c>
@@ -31198,7 +31198,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="307" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="307" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A307" s="7" t="s">
         <v>1004</v>
       </c>
@@ -31263,7 +31263,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="308" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="308" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A308" s="7" t="s">
         <v>1008</v>
       </c>
@@ -31328,7 +31328,7 @@
         <v>1374</v>
       </c>
     </row>
-    <row r="309" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="309" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A309" s="7" t="s">
         <v>1013</v>
       </c>
@@ -31393,7 +31393,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="310" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="310" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A310" s="7" t="s">
         <v>1016</v>
       </c>
@@ -31458,7 +31458,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="311" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="311" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A311" s="7" t="s">
         <v>1019</v>
       </c>
@@ -31523,7 +31523,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="312" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="312" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A312" s="7" t="s">
         <v>1022</v>
       </c>
@@ -31588,7 +31588,7 @@
         <v>868</v>
       </c>
     </row>
-    <row r="313" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="313" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A313" s="7" t="s">
         <v>1026</v>
       </c>
@@ -31653,7 +31653,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="314" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="314" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A314" s="7" t="s">
         <v>1028</v>
       </c>
@@ -31718,7 +31718,7 @@
         <v>846</v>
       </c>
     </row>
-    <row r="315" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="315" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A315" s="7" t="s">
         <v>1030</v>
       </c>
@@ -31783,7 +31783,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="316" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="316" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A316" s="7" t="s">
         <v>1033</v>
       </c>
@@ -31848,7 +31848,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="317" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="317" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A317" s="7" t="s">
         <v>1035</v>
       </c>
@@ -31913,7 +31913,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="318" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="318" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A318" s="7" t="s">
         <v>1038</v>
       </c>
@@ -31978,7 +31978,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="319" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="319" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A319" s="7" t="s">
         <v>1041</v>
       </c>
@@ -32043,7 +32043,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="320" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="320" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A320" s="7" t="s">
         <v>1044</v>
       </c>
@@ -32108,7 +32108,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="321" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="321" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A321" s="7" t="s">
         <v>1046</v>
       </c>
@@ -32173,7 +32173,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="322" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="322" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A322" s="7" t="s">
         <v>1048</v>
       </c>
@@ -32238,7 +32238,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="323" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="323" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A323" s="7" t="s">
         <v>1051</v>
       </c>
@@ -32303,7 +32303,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="324" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="324" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A324" s="7" t="s">
         <v>1053</v>
       </c>
@@ -32368,7 +32368,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="325" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="325" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A325" s="7" t="s">
         <v>1055</v>
       </c>
@@ -32433,7 +32433,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="326" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="326" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A326" s="7" t="s">
         <v>1057</v>
       </c>
@@ -32498,7 +32498,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="327" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="327" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A327" s="7" t="s">
         <v>1060</v>
       </c>
@@ -32563,7 +32563,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="328" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="328" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A328" s="7" t="s">
         <v>1062</v>
       </c>
@@ -32628,7 +32628,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="329" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="329" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A329" s="7" t="s">
         <v>1064</v>
       </c>
@@ -32693,7 +32693,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="330" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="330" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A330" s="7" t="s">
         <v>1067</v>
       </c>
@@ -32758,7 +32758,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="331" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="331" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A331" s="7" t="s">
         <v>1068</v>
       </c>
@@ -32810,7 +32810,7 @@
         <v>1069</v>
       </c>
       <c r="Q331" s="9" t="s">
-        <v>880</v>
+        <v>1172</v>
       </c>
       <c r="R331" s="9" t="s">
         <v>154</v>
@@ -32823,7 +32823,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="332" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="332" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A332" s="7" t="s">
         <v>1071</v>
       </c>
@@ -32875,7 +32875,7 @@
         <v>1073</v>
       </c>
       <c r="Q332" s="9" t="s">
-        <v>880</v>
+        <v>1172</v>
       </c>
       <c r="R332" s="9" t="s">
         <v>154</v>
@@ -32888,7 +32888,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="333" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="333" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A333" s="7" t="s">
         <v>1074</v>
       </c>
@@ -32940,7 +32940,7 @@
         <v>1076</v>
       </c>
       <c r="Q333" s="9" t="s">
-        <v>880</v>
+        <v>1172</v>
       </c>
       <c r="R333" s="9" t="s">
         <v>154</v>
@@ -32953,7 +32953,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="334" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="334" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A334" s="7" t="s">
         <v>1077</v>
       </c>
@@ -33018,7 +33018,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="335" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="335" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A335" s="7" t="s">
         <v>1079</v>
       </c>
@@ -33083,7 +33083,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="336" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="336" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A336" s="7" t="s">
         <v>1082</v>
       </c>
@@ -33148,7 +33148,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="337" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="337" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A337" s="7" t="s">
         <v>1085</v>
       </c>
@@ -33213,7 +33213,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="338" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="338" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A338" s="7" t="s">
         <v>1088</v>
       </c>
@@ -33278,7 +33278,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="339" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="339" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A339" s="7" t="s">
         <v>1090</v>
       </c>
@@ -33343,7 +33343,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="340" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="340" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A340" s="7" t="s">
         <v>1092</v>
       </c>
@@ -33408,7 +33408,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="341" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="341" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A341" s="7" t="s">
         <v>1094</v>
       </c>
@@ -33473,7 +33473,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="342" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="342" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A342" s="7" t="s">
         <v>1097</v>
       </c>
@@ -33538,7 +33538,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="343" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="343" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A343" s="7" t="s">
         <v>1099</v>
       </c>
@@ -33603,7 +33603,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="344" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="344" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A344" s="7" t="s">
         <v>1102</v>
       </c>
@@ -33668,7 +33668,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="345" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="345" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A345" s="7" t="s">
         <v>1105</v>
       </c>
@@ -33733,7 +33733,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="346" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="346" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A346" s="7" t="s">
         <v>1108</v>
       </c>
@@ -33798,7 +33798,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="347" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="347" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A347" s="7" t="s">
         <v>1111</v>
       </c>
@@ -33863,7 +33863,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="348" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="348" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A348" s="7" t="s">
         <v>1113</v>
       </c>
@@ -33928,7 +33928,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="349" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="349" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A349" s="7" t="s">
         <v>1116</v>
       </c>
@@ -33993,7 +33993,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="350" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="350" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A350" s="7" t="s">
         <v>1119</v>
       </c>
@@ -34058,7 +34058,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="351" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="351" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A351" s="7" t="s">
         <v>1122</v>
       </c>
@@ -34123,7 +34123,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="352" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="352" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A352" s="7" t="s">
         <v>1125</v>
       </c>
@@ -34188,7 +34188,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="353" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="353" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A353" s="7" t="s">
         <v>1127</v>
       </c>
@@ -34253,7 +34253,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="354" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="354" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A354" s="7" t="s">
         <v>1130</v>
       </c>
@@ -34318,7 +34318,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="355" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="355" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A355" s="7" t="s">
         <v>1131</v>
       </c>
@@ -34383,7 +34383,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="356" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="356" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A356" s="7" t="s">
         <v>1135</v>
       </c>
@@ -34448,7 +34448,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="357" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="357" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A357" s="7" t="s">
         <v>1138</v>
       </c>
@@ -34513,7 +34513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="358" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="358" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A358" s="7" t="s">
         <v>1141</v>
       </c>
@@ -34777,13 +34777,7 @@
       <c r="T367" s="9"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T358">
-    <filterColumn colId="16">
-      <filters>
-        <filter val="SQL Databases"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:T358"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="8" fitToWidth="0" orientation="landscape" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
#47 Reading List: updated to 2025-11-17 (added latest read books).
</commit_message>
<xml_diff>
--- a/data/Reading List.xlsx
+++ b/data/Reading List.xlsx
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5526" uniqueCount="1175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5622" uniqueCount="1197">
   <si>
     <t>Format</t>
   </si>
@@ -3569,6 +3569,72 @@
   </si>
   <si>
     <t>Using Docker</t>
+  </si>
+  <si>
+    <t>Postgres Succintly</t>
+  </si>
+  <si>
+    <t>2025-08-14</t>
+  </si>
+  <si>
+    <t>Useful. Well-written and straight to the point.</t>
+  </si>
+  <si>
+    <t>Learning PostgreSQL</t>
+  </si>
+  <si>
+    <t>2025-08-21</t>
+  </si>
+  <si>
+    <t>Useful. Ok book, well written, no repetitions.</t>
+  </si>
+  <si>
+    <t>The Design of Everyday Things</t>
+  </si>
+  <si>
+    <t>Basic Books</t>
+  </si>
+  <si>
+    <t>2025-11-13</t>
+  </si>
+  <si>
+    <t>Useless. This is a classic design book but it's mostly a philosophical essay. If you are searching for same actionable advices, this is not the right book.</t>
+  </si>
+  <si>
+    <t>Normal UI</t>
+  </si>
+  <si>
+    <t>Useful. Really original, clear, concise book about UI-related workflows.</t>
+  </si>
+  <si>
+    <t>Retrieval-Augmented Generation</t>
+  </si>
+  <si>
+    <t>2025-11-14</t>
+  </si>
+  <si>
+    <t>Useless. Just a list of types of RAG systems with a short description. A very impersonal book.</t>
+  </si>
+  <si>
+    <t>Rapid Product Development With n8n</t>
+  </si>
+  <si>
+    <t>Useful. A decent introduction to n8n.</t>
+  </si>
+  <si>
+    <t>RAG-Driven Generative AI</t>
+  </si>
+  <si>
+    <t>Useless. Very confusing book structure, continuosly jumping back and forth concepts, zero linearity, usual Packt book published without any editing.</t>
+  </si>
+  <si>
+    <t>RAG With Python Cookbook (Early Release)</t>
+  </si>
+  <si>
+    <t>2025-11-15</t>
+  </si>
+  <si>
+    <t>Useful. Very wellwritten, concise and linear.</t>
   </si>
 </sst>
 </file>
@@ -3708,7 +3774,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3826,6 +3892,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -11294,7 +11363,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet5"/>
-  <dimension ref="A1:T369"/>
+  <dimension ref="A1:T378"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="57.42578125" style="1" customWidth="1"/>
@@ -31977,7 +32046,7 @@
         <v>154</v>
       </c>
       <c r="S318" s="14">
-        <f t="shared" ref="S318:S360" si="125">LEN(P318)</f>
+        <f t="shared" ref="S318:S368" si="125">LEN(P318)</f>
         <v>35</v>
       </c>
       <c r="T318" s="10">
@@ -34715,183 +34784,527 @@
       </c>
     </row>
     <row r="361" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A361" s="9"/>
-      <c r="B361" s="9"/>
-      <c r="C361" s="9"/>
-      <c r="D361" s="9"/>
-      <c r="E361" s="9"/>
-      <c r="F361" s="9"/>
-      <c r="G361" s="9"/>
-      <c r="H361" s="9"/>
-      <c r="I361" s="9"/>
-      <c r="J361" s="9"/>
-      <c r="K361" s="9"/>
-      <c r="L361" s="9"/>
-      <c r="M361" s="9"/>
-      <c r="N361" s="9"/>
-      <c r="O361" s="9"/>
-      <c r="P361" s="9"/>
-      <c r="Q361" s="9"/>
-      <c r="R361" s="9"/>
-      <c r="S361" s="14"/>
-      <c r="T361" s="9"/>
+      <c r="A361" s="7" t="s">
+        <v>1175</v>
+      </c>
+      <c r="B361" s="14">
+        <v>2013</v>
+      </c>
+      <c r="C361" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D361" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E361" s="9" t="s">
+        <v>642</v>
+      </c>
+      <c r="F361" s="43">
+        <v>135</v>
+      </c>
+      <c r="G361" s="9" t="s">
+        <v>1176</v>
+      </c>
+      <c r="H361" s="9">
+        <f t="shared" ref="H361" si="195">YEAR(G361)</f>
+        <v>2025</v>
+      </c>
+      <c r="I361" s="9">
+        <f t="shared" ref="I361" si="196">MONTH(G361)</f>
+        <v>8</v>
+      </c>
+      <c r="J361" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="K361" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="L361" s="9" t="s">
+        <v>354</v>
+      </c>
+      <c r="M361" s="43">
+        <v>4</v>
+      </c>
+      <c r="N361" s="35">
+        <v>0</v>
+      </c>
+      <c r="O361" s="9" t="s">
+        <v>640</v>
+      </c>
+      <c r="P361" s="7" t="s">
+        <v>1177</v>
+      </c>
+      <c r="Q361" s="9" t="s">
+        <v>1169</v>
+      </c>
+      <c r="R361" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="S361" s="14">
+        <f t="shared" si="125"/>
+        <v>47</v>
+      </c>
+      <c r="T361" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="362" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A362" s="9"/>
-      <c r="B362" s="9"/>
-      <c r="C362" s="9"/>
-      <c r="D362" s="9"/>
-      <c r="E362" s="9"/>
-      <c r="F362" s="9"/>
-      <c r="G362" s="9"/>
-      <c r="H362" s="9"/>
-      <c r="I362" s="9"/>
-      <c r="J362" s="9"/>
-      <c r="K362" s="9"/>
-      <c r="L362" s="9"/>
-      <c r="M362" s="9"/>
-      <c r="N362" s="9"/>
-      <c r="O362" s="9"/>
-      <c r="P362" s="9"/>
-      <c r="Q362" s="9"/>
-      <c r="R362" s="9"/>
-      <c r="S362" s="14"/>
-      <c r="T362" s="9"/>
+      <c r="A362" s="7" t="s">
+        <v>1178</v>
+      </c>
+      <c r="B362" s="14">
+        <v>2015</v>
+      </c>
+      <c r="C362" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D362" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E362" s="9" t="s">
+        <v>642</v>
+      </c>
+      <c r="F362" s="43">
+        <v>464</v>
+      </c>
+      <c r="G362" s="9" t="s">
+        <v>1179</v>
+      </c>
+      <c r="H362" s="9">
+        <f t="shared" ref="H362" si="197">YEAR(G362)</f>
+        <v>2025</v>
+      </c>
+      <c r="I362" s="9">
+        <f t="shared" ref="I362" si="198">MONTH(G362)</f>
+        <v>8</v>
+      </c>
+      <c r="J362" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="K362" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="L362" s="9" t="s">
+        <v>345</v>
+      </c>
+      <c r="M362" s="14">
+        <v>3</v>
+      </c>
+      <c r="N362" s="43">
+        <v>60.99</v>
+      </c>
+      <c r="O362" s="9" t="s">
+        <v>640</v>
+      </c>
+      <c r="P362" s="7" t="s">
+        <v>1180</v>
+      </c>
+      <c r="Q362" s="9" t="s">
+        <v>1169</v>
+      </c>
+      <c r="R362" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="S362" s="14">
+        <f t="shared" si="125"/>
+        <v>46</v>
+      </c>
+      <c r="T362" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="363" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A363" s="9"/>
-      <c r="B363" s="9"/>
-      <c r="C363" s="9"/>
-      <c r="D363" s="9"/>
-      <c r="E363" s="9"/>
-      <c r="F363" s="9"/>
-      <c r="G363" s="9"/>
-      <c r="H363" s="9"/>
-      <c r="I363" s="9"/>
-      <c r="J363" s="9"/>
-      <c r="K363" s="9"/>
-      <c r="L363" s="9"/>
-      <c r="M363" s="9"/>
-      <c r="N363" s="9"/>
-      <c r="O363" s="9"/>
-      <c r="P363" s="9"/>
-      <c r="Q363" s="9"/>
-      <c r="R363" s="9"/>
-      <c r="S363" s="14"/>
-      <c r="T363" s="9"/>
+      <c r="A363" s="7" t="s">
+        <v>1181</v>
+      </c>
+      <c r="B363" s="14">
+        <v>2013</v>
+      </c>
+      <c r="C363" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D363" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E363" s="9" t="s">
+        <v>642</v>
+      </c>
+      <c r="F363" s="43">
+        <v>369</v>
+      </c>
+      <c r="G363" s="9" t="s">
+        <v>1183</v>
+      </c>
+      <c r="H363" s="9">
+        <f t="shared" ref="H363" si="199">YEAR(G363)</f>
+        <v>2025</v>
+      </c>
+      <c r="I363" s="9">
+        <f t="shared" ref="I363:I364" si="200">MONTH(G363)</f>
+        <v>11</v>
+      </c>
+      <c r="J363" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="K363" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="L363" s="9" t="s">
+        <v>1182</v>
+      </c>
+      <c r="M363" s="14">
+        <v>2</v>
+      </c>
+      <c r="N363" s="43">
+        <v>19.989999999999998</v>
+      </c>
+      <c r="O363" s="9" t="s">
+        <v>640</v>
+      </c>
+      <c r="P363" s="7" t="s">
+        <v>1184</v>
+      </c>
+      <c r="Q363" s="9" t="s">
+        <v>1080</v>
+      </c>
+      <c r="R363" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="S363" s="14">
+        <f t="shared" si="125"/>
+        <v>155</v>
+      </c>
+      <c r="T363" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="364" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A364" s="9"/>
-      <c r="B364" s="9"/>
-      <c r="C364" s="9"/>
-      <c r="D364" s="9"/>
-      <c r="E364" s="9"/>
-      <c r="F364" s="9"/>
-      <c r="G364" s="9"/>
-      <c r="H364" s="9"/>
-      <c r="I364" s="9"/>
-      <c r="J364" s="9"/>
-      <c r="K364" s="9"/>
-      <c r="L364" s="9"/>
-      <c r="M364" s="9"/>
-      <c r="N364" s="9"/>
-      <c r="O364" s="9"/>
-      <c r="P364" s="9"/>
-      <c r="Q364" s="9"/>
-      <c r="R364" s="9"/>
-      <c r="S364" s="14"/>
-      <c r="T364" s="9"/>
+      <c r="A364" s="7" t="s">
+        <v>1185</v>
+      </c>
+      <c r="B364" s="14">
+        <v>2025</v>
+      </c>
+      <c r="C364" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D364" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E364" s="9" t="s">
+        <v>642</v>
+      </c>
+      <c r="F364" s="43">
+        <v>78</v>
+      </c>
+      <c r="G364" s="9" t="s">
+        <v>1183</v>
+      </c>
+      <c r="H364" s="9">
+        <f t="shared" ref="H364" si="201">YEAR(G364)</f>
+        <v>2025</v>
+      </c>
+      <c r="I364" s="9">
+        <f t="shared" si="200"/>
+        <v>11</v>
+      </c>
+      <c r="J364" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K364" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="L364" s="9" t="s">
+        <v>578</v>
+      </c>
+      <c r="M364" s="43">
+        <v>5</v>
+      </c>
+      <c r="N364" s="35">
+        <v>0</v>
+      </c>
+      <c r="O364" s="9" t="s">
+        <v>640</v>
+      </c>
+      <c r="P364" s="38" t="s">
+        <v>1186</v>
+      </c>
+      <c r="Q364" s="9" t="s">
+        <v>1080</v>
+      </c>
+      <c r="R364" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="S364" s="14">
+        <f t="shared" si="125"/>
+        <v>72</v>
+      </c>
+      <c r="T364" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="365" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A365" s="9"/>
-      <c r="B365" s="9"/>
-      <c r="C365" s="9"/>
-      <c r="D365" s="9"/>
-      <c r="E365" s="9"/>
-      <c r="F365" s="9"/>
-      <c r="G365" s="9"/>
-      <c r="H365" s="9"/>
-      <c r="I365" s="9"/>
-      <c r="J365" s="9"/>
-      <c r="K365" s="9"/>
-      <c r="L365" s="9"/>
-      <c r="M365" s="9"/>
-      <c r="N365" s="9"/>
-      <c r="O365" s="9"/>
-      <c r="P365" s="9"/>
-      <c r="Q365" s="9"/>
-      <c r="R365" s="9"/>
-      <c r="S365" s="14"/>
-      <c r="T365" s="9"/>
+      <c r="A365" s="7" t="s">
+        <v>1187</v>
+      </c>
+      <c r="B365" s="14">
+        <v>2025</v>
+      </c>
+      <c r="C365" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D365" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E365" s="9" t="s">
+        <v>642</v>
+      </c>
+      <c r="F365" s="43">
+        <v>43</v>
+      </c>
+      <c r="G365" s="9" t="s">
+        <v>1188</v>
+      </c>
+      <c r="H365" s="9">
+        <f t="shared" ref="H365" si="202">YEAR(G365)</f>
+        <v>2025</v>
+      </c>
+      <c r="I365" s="9">
+        <f t="shared" ref="I365" si="203">MONTH(G365)</f>
+        <v>11</v>
+      </c>
+      <c r="J365" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="K365" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="L365" s="9" t="s">
+        <v>578</v>
+      </c>
+      <c r="M365" s="14">
+        <v>1</v>
+      </c>
+      <c r="N365" s="35">
+        <v>0</v>
+      </c>
+      <c r="O365" s="9" t="s">
+        <v>640</v>
+      </c>
+      <c r="P365" s="7" t="s">
+        <v>1189</v>
+      </c>
+      <c r="Q365" s="9" t="s">
+        <v>932</v>
+      </c>
+      <c r="R365" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="S365" s="14">
+        <f t="shared" si="125"/>
+        <v>94</v>
+      </c>
+      <c r="T365" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="366" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A366" s="9"/>
-      <c r="B366" s="9"/>
-      <c r="C366" s="9"/>
-      <c r="D366" s="9"/>
-      <c r="E366" s="9"/>
-      <c r="F366" s="9"/>
-      <c r="G366" s="9"/>
-      <c r="H366" s="9"/>
-      <c r="I366" s="9"/>
-      <c r="J366" s="9"/>
-      <c r="K366" s="9"/>
-      <c r="L366" s="9"/>
-      <c r="M366" s="9"/>
-      <c r="N366" s="9"/>
-      <c r="O366" s="9"/>
-      <c r="P366" s="9"/>
-      <c r="Q366" s="9"/>
-      <c r="R366" s="9"/>
-      <c r="S366" s="14"/>
-      <c r="T366" s="9"/>
+      <c r="A366" s="7" t="s">
+        <v>1190</v>
+      </c>
+      <c r="B366" s="43">
+        <v>2022</v>
+      </c>
+      <c r="C366" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D366" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E366" s="9" t="s">
+        <v>642</v>
+      </c>
+      <c r="F366" s="43">
+        <v>236</v>
+      </c>
+      <c r="G366" s="9" t="s">
+        <v>1188</v>
+      </c>
+      <c r="H366" s="9">
+        <f t="shared" ref="H366" si="204">YEAR(G366)</f>
+        <v>2025</v>
+      </c>
+      <c r="I366" s="9">
+        <f t="shared" ref="I366" si="205">MONTH(G366)</f>
+        <v>11</v>
+      </c>
+      <c r="J366" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="K366" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="L366" s="9" t="s">
+        <v>345</v>
+      </c>
+      <c r="M366" s="14">
+        <v>3</v>
+      </c>
+      <c r="N366" s="43">
+        <v>31.99</v>
+      </c>
+      <c r="O366" s="9" t="s">
+        <v>640</v>
+      </c>
+      <c r="P366" s="7" t="s">
+        <v>1191</v>
+      </c>
+      <c r="Q366" s="9" t="s">
+        <v>849</v>
+      </c>
+      <c r="R366" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="S366" s="14">
+        <f t="shared" si="125"/>
+        <v>37</v>
+      </c>
+      <c r="T366" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="367" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A367" s="9"/>
-      <c r="B367" s="9"/>
-      <c r="C367" s="9"/>
-      <c r="D367" s="9"/>
-      <c r="E367" s="9"/>
-      <c r="F367" s="9"/>
-      <c r="G367" s="9"/>
-      <c r="H367" s="9"/>
-      <c r="I367" s="9"/>
-      <c r="J367" s="9"/>
-      <c r="K367" s="9"/>
-      <c r="L367" s="9"/>
-      <c r="M367" s="9"/>
-      <c r="N367" s="9"/>
-      <c r="O367" s="9"/>
-      <c r="P367" s="9"/>
-      <c r="Q367" s="9"/>
-      <c r="R367" s="9"/>
-      <c r="S367" s="14"/>
-      <c r="T367" s="9"/>
+      <c r="A367" s="7" t="s">
+        <v>1192</v>
+      </c>
+      <c r="B367" s="43">
+        <v>2024</v>
+      </c>
+      <c r="C367" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D367" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E367" s="9" t="s">
+        <v>642</v>
+      </c>
+      <c r="F367" s="43">
+        <v>445</v>
+      </c>
+      <c r="G367" s="9" t="s">
+        <v>1188</v>
+      </c>
+      <c r="H367" s="9">
+        <f t="shared" ref="H367" si="206">YEAR(G367)</f>
+        <v>2025</v>
+      </c>
+      <c r="I367" s="9">
+        <f t="shared" ref="I367" si="207">MONTH(G367)</f>
+        <v>11</v>
+      </c>
+      <c r="J367" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="K367" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="L367" s="9" t="s">
+        <v>345</v>
+      </c>
+      <c r="M367" s="14">
+        <v>1</v>
+      </c>
+      <c r="N367" s="43">
+        <v>43.99</v>
+      </c>
+      <c r="O367" s="9" t="s">
+        <v>640</v>
+      </c>
+      <c r="P367" s="7" t="s">
+        <v>1193</v>
+      </c>
+      <c r="Q367" s="9" t="s">
+        <v>932</v>
+      </c>
+      <c r="R367" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="S367" s="14">
+        <f t="shared" si="125"/>
+        <v>148</v>
+      </c>
+      <c r="T367" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="368" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A368" s="9"/>
-      <c r="B368" s="9"/>
-      <c r="C368" s="9"/>
-      <c r="D368" s="9"/>
-      <c r="E368" s="9"/>
-      <c r="F368" s="9"/>
-      <c r="G368" s="9"/>
-      <c r="H368" s="9"/>
-      <c r="I368" s="9"/>
-      <c r="J368" s="9"/>
-      <c r="K368" s="9"/>
-      <c r="L368" s="9"/>
-      <c r="M368" s="9"/>
-      <c r="N368" s="9"/>
-      <c r="O368" s="9"/>
-      <c r="P368" s="9"/>
-      <c r="Q368" s="9"/>
-      <c r="R368" s="9"/>
-      <c r="S368" s="14"/>
-      <c r="T368" s="9"/>
+      <c r="A368" s="7" t="s">
+        <v>1194</v>
+      </c>
+      <c r="B368" s="43">
+        <v>2025</v>
+      </c>
+      <c r="C368" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D368" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E368" s="9" t="s">
+        <v>642</v>
+      </c>
+      <c r="F368" s="43">
+        <v>82</v>
+      </c>
+      <c r="G368" s="9" t="s">
+        <v>1195</v>
+      </c>
+      <c r="H368" s="9">
+        <f t="shared" ref="H368" si="208">YEAR(G368)</f>
+        <v>2025</v>
+      </c>
+      <c r="I368" s="9">
+        <f t="shared" ref="I368" si="209">MONTH(G368)</f>
+        <v>11</v>
+      </c>
+      <c r="J368" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="K368" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L368" s="9" t="s">
+        <v>347</v>
+      </c>
+      <c r="M368" s="43">
+        <v>4</v>
+      </c>
+      <c r="N368" s="43">
+        <v>79.989999999999995</v>
+      </c>
+      <c r="O368" s="9" t="s">
+        <v>640</v>
+      </c>
+      <c r="P368" s="7" t="s">
+        <v>1196</v>
+      </c>
+      <c r="Q368" s="9" t="s">
+        <v>932</v>
+      </c>
+      <c r="R368" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="S368" s="14">
+        <f t="shared" si="125"/>
+        <v>45</v>
+      </c>
+      <c r="T368" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="369" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A369" s="9"/>
+      <c r="A369" s="7"/>
       <c r="B369" s="9"/>
       <c r="C369" s="9"/>
       <c r="D369" s="9"/>
@@ -34906,11 +35319,209 @@
       <c r="M369" s="9"/>
       <c r="N369" s="9"/>
       <c r="O369" s="9"/>
-      <c r="P369" s="9"/>
+      <c r="P369" s="7"/>
       <c r="Q369" s="9"/>
       <c r="R369" s="9"/>
       <c r="S369" s="14"/>
       <c r="T369" s="9"/>
+    </row>
+    <row r="370" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A370" s="9"/>
+      <c r="B370" s="9"/>
+      <c r="C370" s="9"/>
+      <c r="D370" s="9"/>
+      <c r="E370" s="9"/>
+      <c r="F370" s="9"/>
+      <c r="G370" s="9"/>
+      <c r="H370" s="9"/>
+      <c r="I370" s="9"/>
+      <c r="J370" s="9"/>
+      <c r="K370" s="9"/>
+      <c r="L370" s="9"/>
+      <c r="M370" s="9"/>
+      <c r="N370" s="9"/>
+      <c r="O370" s="9"/>
+      <c r="P370" s="9"/>
+      <c r="Q370" s="9"/>
+      <c r="R370" s="9"/>
+      <c r="S370" s="14"/>
+      <c r="T370" s="9"/>
+    </row>
+    <row r="371" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A371" s="9"/>
+      <c r="B371" s="9"/>
+      <c r="C371" s="9"/>
+      <c r="D371" s="9"/>
+      <c r="E371" s="9"/>
+      <c r="F371" s="9"/>
+      <c r="G371" s="9"/>
+      <c r="H371" s="9"/>
+      <c r="I371" s="9"/>
+      <c r="J371" s="9"/>
+      <c r="K371" s="9"/>
+      <c r="L371" s="9"/>
+      <c r="M371" s="9"/>
+      <c r="N371" s="9"/>
+      <c r="O371" s="9"/>
+      <c r="P371" s="9"/>
+      <c r="Q371" s="9"/>
+      <c r="R371" s="9"/>
+      <c r="S371" s="14"/>
+      <c r="T371" s="9"/>
+    </row>
+    <row r="372" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A372" s="9"/>
+      <c r="B372" s="9"/>
+      <c r="C372" s="9"/>
+      <c r="D372" s="9"/>
+      <c r="E372" s="9"/>
+      <c r="F372" s="9"/>
+      <c r="G372" s="9"/>
+      <c r="H372" s="9"/>
+      <c r="I372" s="9"/>
+      <c r="J372" s="9"/>
+      <c r="K372" s="9"/>
+      <c r="L372" s="9"/>
+      <c r="M372" s="9"/>
+      <c r="N372" s="9"/>
+      <c r="O372" s="9"/>
+      <c r="P372" s="9"/>
+      <c r="Q372" s="9"/>
+      <c r="R372" s="9"/>
+      <c r="S372" s="14"/>
+      <c r="T372" s="9"/>
+    </row>
+    <row r="373" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A373" s="9"/>
+      <c r="B373" s="9"/>
+      <c r="C373" s="9"/>
+      <c r="D373" s="9"/>
+      <c r="E373" s="9"/>
+      <c r="F373" s="9"/>
+      <c r="G373" s="9"/>
+      <c r="H373" s="9"/>
+      <c r="I373" s="9"/>
+      <c r="J373" s="9"/>
+      <c r="K373" s="9"/>
+      <c r="L373" s="9"/>
+      <c r="M373" s="9"/>
+      <c r="N373" s="9"/>
+      <c r="O373" s="9"/>
+      <c r="P373" s="9"/>
+      <c r="Q373" s="9"/>
+      <c r="R373" s="9"/>
+      <c r="S373" s="14"/>
+      <c r="T373" s="9"/>
+    </row>
+    <row r="374" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A374" s="9"/>
+      <c r="B374" s="9"/>
+      <c r="C374" s="9"/>
+      <c r="D374" s="9"/>
+      <c r="E374" s="9"/>
+      <c r="F374" s="9"/>
+      <c r="G374" s="9"/>
+      <c r="H374" s="9"/>
+      <c r="I374" s="9"/>
+      <c r="J374" s="9"/>
+      <c r="K374" s="9"/>
+      <c r="L374" s="9"/>
+      <c r="M374" s="9"/>
+      <c r="N374" s="9"/>
+      <c r="O374" s="9"/>
+      <c r="P374" s="9"/>
+      <c r="Q374" s="9"/>
+      <c r="R374" s="9"/>
+      <c r="S374" s="14"/>
+      <c r="T374" s="9"/>
+    </row>
+    <row r="375" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A375" s="9"/>
+      <c r="B375" s="9"/>
+      <c r="C375" s="9"/>
+      <c r="D375" s="9"/>
+      <c r="E375" s="9"/>
+      <c r="F375" s="9"/>
+      <c r="G375" s="9"/>
+      <c r="H375" s="9"/>
+      <c r="I375" s="9"/>
+      <c r="J375" s="9"/>
+      <c r="K375" s="9"/>
+      <c r="L375" s="9"/>
+      <c r="M375" s="9"/>
+      <c r="N375" s="9"/>
+      <c r="O375" s="9"/>
+      <c r="P375" s="9"/>
+      <c r="Q375" s="9"/>
+      <c r="R375" s="9"/>
+      <c r="S375" s="14"/>
+      <c r="T375" s="9"/>
+    </row>
+    <row r="376" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A376" s="9"/>
+      <c r="B376" s="9"/>
+      <c r="C376" s="9"/>
+      <c r="D376" s="9"/>
+      <c r="E376" s="9"/>
+      <c r="F376" s="9"/>
+      <c r="G376" s="9"/>
+      <c r="H376" s="9"/>
+      <c r="I376" s="9"/>
+      <c r="J376" s="9"/>
+      <c r="K376" s="9"/>
+      <c r="L376" s="9"/>
+      <c r="M376" s="9"/>
+      <c r="N376" s="9"/>
+      <c r="O376" s="9"/>
+      <c r="P376" s="9"/>
+      <c r="Q376" s="9"/>
+      <c r="R376" s="9"/>
+      <c r="S376" s="14"/>
+      <c r="T376" s="9"/>
+    </row>
+    <row r="377" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A377" s="9"/>
+      <c r="B377" s="9"/>
+      <c r="C377" s="9"/>
+      <c r="D377" s="9"/>
+      <c r="E377" s="9"/>
+      <c r="F377" s="9"/>
+      <c r="G377" s="9"/>
+      <c r="H377" s="9"/>
+      <c r="I377" s="9"/>
+      <c r="J377" s="9"/>
+      <c r="K377" s="9"/>
+      <c r="L377" s="9"/>
+      <c r="M377" s="9"/>
+      <c r="N377" s="9"/>
+      <c r="O377" s="9"/>
+      <c r="P377" s="9"/>
+      <c r="Q377" s="9"/>
+      <c r="R377" s="9"/>
+      <c r="S377" s="14"/>
+      <c r="T377" s="9"/>
+    </row>
+    <row r="378" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A378" s="9"/>
+      <c r="B378" s="9"/>
+      <c r="C378" s="9"/>
+      <c r="D378" s="9"/>
+      <c r="E378" s="9"/>
+      <c r="F378" s="9"/>
+      <c r="G378" s="9"/>
+      <c r="H378" s="9"/>
+      <c r="I378" s="9"/>
+      <c r="J378" s="9"/>
+      <c r="K378" s="9"/>
+      <c r="L378" s="9"/>
+      <c r="M378" s="9"/>
+      <c r="N378" s="9"/>
+      <c r="O378" s="9"/>
+      <c r="P378" s="9"/>
+      <c r="Q378" s="9"/>
+      <c r="R378" s="9"/>
+      <c r="S378" s="14"/>
+      <c r="T378" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
#47 Added: Hugging Face In Action.
</commit_message>
<xml_diff>
--- a/data/Reading List.xlsx
+++ b/data/Reading List.xlsx
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5622" uniqueCount="1197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5634" uniqueCount="1200">
   <si>
     <t>Format</t>
   </si>
@@ -3635,6 +3635,15 @@
   </si>
   <si>
     <t>Useful. Very wellwritten, concise and linear.</t>
+  </si>
+  <si>
+    <t>Hugging Face In Action</t>
+  </si>
+  <si>
+    <t>2025-11-22</t>
+  </si>
+  <si>
+    <t>Useful. It's very unstructured and repetitive, but it contains also some useful bits of information.</t>
   </si>
 </sst>
 </file>
@@ -3888,13 +3897,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -4209,16 +4218,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="14.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="41">
+      <c r="A1" s="42">
         <v>2016</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
-      <c r="G1" s="41"/>
-      <c r="H1" s="42"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="43"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="18" t="s">
@@ -5664,16 +5673,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="14.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="41">
+      <c r="A1" s="42">
         <v>2017</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
-      <c r="G1" s="41"/>
-      <c r="H1" s="42"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="43"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="18" t="s">
@@ -6615,16 +6624,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="14.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="41">
+      <c r="A1" s="42">
         <v>2018</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
-      <c r="G1" s="41"/>
-      <c r="H1" s="42"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="43"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="18" t="s">
@@ -7566,16 +7575,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="14.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="41">
+      <c r="A1" s="42">
         <v>2019</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
-      <c r="G1" s="41"/>
-      <c r="H1" s="42"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="43"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="18" t="s">
@@ -8517,16 +8526,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="14.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="41">
+      <c r="A1" s="42">
         <v>2020</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
-      <c r="G1" s="41"/>
-      <c r="H1" s="42"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="43"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="18" t="s">
@@ -9468,16 +9477,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="14.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="41">
+      <c r="A1" s="42">
         <v>2021</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
-      <c r="G1" s="41"/>
-      <c r="H1" s="42"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="43"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="18" t="s">
@@ -10419,16 +10428,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="14.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="41">
+      <c r="A1" s="42">
         <v>2022</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
-      <c r="G1" s="41"/>
-      <c r="H1" s="42"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="43"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="18" t="s">
@@ -32046,7 +32055,7 @@
         <v>154</v>
       </c>
       <c r="S318" s="14">
-        <f t="shared" ref="S318:S368" si="125">LEN(P318)</f>
+        <f t="shared" ref="S318:S369" si="125">LEN(P318)</f>
         <v>35</v>
       </c>
       <c r="T318" s="10">
@@ -34799,7 +34808,7 @@
       <c r="E361" s="9" t="s">
         <v>642</v>
       </c>
-      <c r="F361" s="43">
+      <c r="F361" s="41">
         <v>135</v>
       </c>
       <c r="G361" s="9" t="s">
@@ -34822,7 +34831,7 @@
       <c r="L361" s="9" t="s">
         <v>354</v>
       </c>
-      <c r="M361" s="43">
+      <c r="M361" s="41">
         <v>4</v>
       </c>
       <c r="N361" s="35">
@@ -34864,7 +34873,7 @@
       <c r="E362" s="9" t="s">
         <v>642</v>
       </c>
-      <c r="F362" s="43">
+      <c r="F362" s="41">
         <v>464</v>
       </c>
       <c r="G362" s="9" t="s">
@@ -34890,7 +34899,7 @@
       <c r="M362" s="14">
         <v>3</v>
       </c>
-      <c r="N362" s="43">
+      <c r="N362" s="41">
         <v>60.99</v>
       </c>
       <c r="O362" s="9" t="s">
@@ -34929,7 +34938,7 @@
       <c r="E363" s="9" t="s">
         <v>642</v>
       </c>
-      <c r="F363" s="43">
+      <c r="F363" s="41">
         <v>369</v>
       </c>
       <c r="G363" s="9" t="s">
@@ -34955,7 +34964,7 @@
       <c r="M363" s="14">
         <v>2</v>
       </c>
-      <c r="N363" s="43">
+      <c r="N363" s="41">
         <v>19.989999999999998</v>
       </c>
       <c r="O363" s="9" t="s">
@@ -34994,7 +35003,7 @@
       <c r="E364" s="9" t="s">
         <v>642</v>
       </c>
-      <c r="F364" s="43">
+      <c r="F364" s="41">
         <v>78</v>
       </c>
       <c r="G364" s="9" t="s">
@@ -35017,7 +35026,7 @@
       <c r="L364" s="9" t="s">
         <v>578</v>
       </c>
-      <c r="M364" s="43">
+      <c r="M364" s="41">
         <v>5</v>
       </c>
       <c r="N364" s="35">
@@ -35059,7 +35068,7 @@
       <c r="E365" s="9" t="s">
         <v>642</v>
       </c>
-      <c r="F365" s="43">
+      <c r="F365" s="41">
         <v>43</v>
       </c>
       <c r="G365" s="9" t="s">
@@ -35112,7 +35121,7 @@
       <c r="A366" s="7" t="s">
         <v>1190</v>
       </c>
-      <c r="B366" s="43">
+      <c r="B366" s="41">
         <v>2022</v>
       </c>
       <c r="C366" s="9" t="s">
@@ -35124,7 +35133,7 @@
       <c r="E366" s="9" t="s">
         <v>642</v>
       </c>
-      <c r="F366" s="43">
+      <c r="F366" s="41">
         <v>236</v>
       </c>
       <c r="G366" s="9" t="s">
@@ -35150,7 +35159,7 @@
       <c r="M366" s="14">
         <v>3</v>
       </c>
-      <c r="N366" s="43">
+      <c r="N366" s="41">
         <v>31.99</v>
       </c>
       <c r="O366" s="9" t="s">
@@ -35177,7 +35186,7 @@
       <c r="A367" s="7" t="s">
         <v>1192</v>
       </c>
-      <c r="B367" s="43">
+      <c r="B367" s="41">
         <v>2024</v>
       </c>
       <c r="C367" s="9" t="s">
@@ -35189,7 +35198,7 @@
       <c r="E367" s="9" t="s">
         <v>642</v>
       </c>
-      <c r="F367" s="43">
+      <c r="F367" s="41">
         <v>445</v>
       </c>
       <c r="G367" s="9" t="s">
@@ -35215,7 +35224,7 @@
       <c r="M367" s="14">
         <v>1</v>
       </c>
-      <c r="N367" s="43">
+      <c r="N367" s="41">
         <v>43.99</v>
       </c>
       <c r="O367" s="9" t="s">
@@ -35242,7 +35251,7 @@
       <c r="A368" s="7" t="s">
         <v>1194</v>
       </c>
-      <c r="B368" s="43">
+      <c r="B368" s="41">
         <v>2025</v>
       </c>
       <c r="C368" s="9" t="s">
@@ -35254,7 +35263,7 @@
       <c r="E368" s="9" t="s">
         <v>642</v>
       </c>
-      <c r="F368" s="43">
+      <c r="F368" s="41">
         <v>82</v>
       </c>
       <c r="G368" s="9" t="s">
@@ -35277,10 +35286,10 @@
       <c r="L368" s="9" t="s">
         <v>347</v>
       </c>
-      <c r="M368" s="43">
-        <v>4</v>
-      </c>
-      <c r="N368" s="43">
+      <c r="M368" s="41">
+        <v>4</v>
+      </c>
+      <c r="N368" s="41">
         <v>79.989999999999995</v>
       </c>
       <c r="O368" s="9" t="s">
@@ -35304,26 +35313,69 @@
       </c>
     </row>
     <row r="369" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A369" s="7"/>
-      <c r="B369" s="9"/>
-      <c r="C369" s="9"/>
-      <c r="D369" s="9"/>
-      <c r="E369" s="9"/>
-      <c r="F369" s="9"/>
-      <c r="G369" s="9"/>
-      <c r="H369" s="9"/>
-      <c r="I369" s="9"/>
-      <c r="J369" s="9"/>
-      <c r="K369" s="9"/>
-      <c r="L369" s="9"/>
-      <c r="M369" s="9"/>
-      <c r="N369" s="9"/>
-      <c r="O369" s="9"/>
-      <c r="P369" s="7"/>
-      <c r="Q369" s="9"/>
-      <c r="R369" s="9"/>
-      <c r="S369" s="14"/>
-      <c r="T369" s="9"/>
+      <c r="A369" s="7" t="s">
+        <v>1197</v>
+      </c>
+      <c r="B369" s="41">
+        <v>2025</v>
+      </c>
+      <c r="C369" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D369" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E369" s="9" t="s">
+        <v>642</v>
+      </c>
+      <c r="F369" s="41">
+        <v>368</v>
+      </c>
+      <c r="G369" s="9" t="s">
+        <v>1198</v>
+      </c>
+      <c r="H369" s="9">
+        <f t="shared" ref="H369" si="210">YEAR(G369)</f>
+        <v>2025</v>
+      </c>
+      <c r="I369" s="9">
+        <f t="shared" ref="I369" si="211">MONTH(G369)</f>
+        <v>11</v>
+      </c>
+      <c r="J369" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="K369" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="L369" s="9" t="s">
+        <v>349</v>
+      </c>
+      <c r="M369" s="14">
+        <v>3</v>
+      </c>
+      <c r="N369" s="41">
+        <v>49.99</v>
+      </c>
+      <c r="O369" s="9" t="s">
+        <v>640</v>
+      </c>
+      <c r="P369" s="7" t="s">
+        <v>1199</v>
+      </c>
+      <c r="Q369" s="9" t="s">
+        <v>932</v>
+      </c>
+      <c r="R369" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="S369" s="14">
+        <f t="shared" si="125"/>
+        <v>100</v>
+      </c>
+      <c r="T369" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="370" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A370" s="9"/>

</xml_diff>

<commit_message>
#47 Reading List: updated to 2025-11-28 (* -> Self-Growth).
</commit_message>
<xml_diff>
--- a/data/Reading List.xlsx
+++ b/data/Reading List.xlsx
@@ -2587,9 +2587,6 @@
     <t>Development Tools</t>
   </si>
   <si>
-    <t>Entrepreneurship, Learning</t>
-  </si>
-  <si>
     <t>Electronics, IoT</t>
   </si>
   <si>
@@ -3638,6 +3635,9 @@
   </si>
   <si>
     <t>Beginning XSLT And XPath: Transforming XML Documents And Data</t>
+  </si>
+  <si>
+    <t>Self-Growth</t>
   </si>
 </sst>
 </file>
@@ -11449,7 +11449,7 @@
         <v>832</v>
       </c>
       <c r="T1" s="6" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.2">
@@ -12429,7 +12429,7 @@
     </row>
     <row r="17" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A17" s="7" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
       <c r="B17" s="10">
         <v>2015</v>
@@ -12544,7 +12544,7 @@
         <v>60</v>
       </c>
       <c r="Q18" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R18" s="9" t="s">
         <v>153</v>
@@ -12559,7 +12559,7 @@
     </row>
     <row r="19" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A19" s="7" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
       <c r="B19" s="10">
         <v>2014</v>
@@ -12739,7 +12739,7 @@
         <v>669</v>
       </c>
       <c r="Q21" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R21" s="9" t="s">
         <v>153</v>
@@ -13129,7 +13129,7 @@
         <v>672</v>
       </c>
       <c r="Q27" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R27" s="9" t="s">
         <v>153</v>
@@ -13144,7 +13144,7 @@
     </row>
     <row r="28" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A28" s="7" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
       <c r="B28" s="10">
         <v>2009</v>
@@ -13194,7 +13194,7 @@
         <v>673</v>
       </c>
       <c r="Q28" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R28" s="9" t="s">
         <v>153</v>
@@ -13259,7 +13259,7 @@
         <v>642</v>
       </c>
       <c r="Q29" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R29" s="9" t="s">
         <v>153</v>
@@ -13729,7 +13729,7 @@
     </row>
     <row r="37" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A37" s="7" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="B37" s="10">
         <v>2013</v>
@@ -13989,7 +13989,7 @@
     </row>
     <row r="41" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A41" s="7" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="B41" s="10">
         <v>1996</v>
@@ -14054,7 +14054,7 @@
     </row>
     <row r="42" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A42" s="7" t="s">
-        <v>1149</v>
+        <v>1148</v>
       </c>
       <c r="B42" s="10">
         <v>2008</v>
@@ -14219,7 +14219,7 @@
         <v>153</v>
       </c>
       <c r="L44" s="9" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="M44" s="10">
         <v>4</v>
@@ -14299,7 +14299,7 @@
         <v>60</v>
       </c>
       <c r="Q45" s="9" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="R45" s="9" t="s">
         <v>153</v>
@@ -14364,7 +14364,7 @@
         <v>60</v>
       </c>
       <c r="Q46" s="9" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="R46" s="9" t="s">
         <v>153</v>
@@ -14429,7 +14429,7 @@
         <v>649</v>
       </c>
       <c r="Q47" s="9" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="R47" s="9" t="s">
         <v>153</v>
@@ -14574,7 +14574,7 @@
     </row>
     <row r="50" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A50" s="7" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
       <c r="B50" s="10">
         <v>2010</v>
@@ -14674,7 +14674,7 @@
         <v>153</v>
       </c>
       <c r="L51" s="9" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="M51" s="10">
         <v>1</v>
@@ -14754,7 +14754,7 @@
         <v>676</v>
       </c>
       <c r="Q52" s="9" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
       <c r="R52" s="9" t="s">
         <v>153</v>
@@ -14769,7 +14769,7 @@
     </row>
     <row r="53" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A53" s="7" t="s">
-        <v>1139</v>
+        <v>1138</v>
       </c>
       <c r="B53" s="10">
         <v>2015</v>
@@ -14834,7 +14834,7 @@
     </row>
     <row r="54" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A54" s="7" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="B54" s="10">
         <v>2003</v>
@@ -14964,7 +14964,7 @@
     </row>
     <row r="56" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A56" s="7" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="B56" s="10">
         <v>2011</v>
@@ -15209,7 +15209,7 @@
         <v>60</v>
       </c>
       <c r="Q59" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R59" s="9" t="s">
         <v>153</v>
@@ -15614,7 +15614,7 @@
     </row>
     <row r="66" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A66" s="7" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="B66" s="10">
         <v>2013</v>
@@ -15924,7 +15924,7 @@
         <v>690</v>
       </c>
       <c r="Q70" s="9" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
       <c r="R70" s="9" t="s">
         <v>153</v>
@@ -16004,7 +16004,7 @@
     </row>
     <row r="72" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A72" s="7" t="s">
-        <v>1167</v>
+        <v>1166</v>
       </c>
       <c r="B72" s="10">
         <v>2012</v>
@@ -16199,7 +16199,7 @@
     </row>
     <row r="75" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A75" s="7" t="s">
-        <v>1153</v>
+        <v>1152</v>
       </c>
       <c r="B75" s="10">
         <v>2007</v>
@@ -16589,7 +16589,7 @@
     </row>
     <row r="81" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A81" s="7" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="B81" s="10">
         <v>2014</v>
@@ -16654,7 +16654,7 @@
     </row>
     <row r="82" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A82" s="7" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
       <c r="B82" s="10">
         <v>2013</v>
@@ -16784,7 +16784,7 @@
     </row>
     <row r="84" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A84" s="7" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
       <c r="B84" s="10">
         <v>2015</v>
@@ -16914,7 +16914,7 @@
     </row>
     <row r="86" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A86" s="7" t="s">
-        <v>1154</v>
+        <v>1153</v>
       </c>
       <c r="B86" s="10">
         <v>2004</v>
@@ -16979,7 +16979,7 @@
     </row>
     <row r="87" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A87" s="7" t="s">
-        <v>1155</v>
+        <v>1154</v>
       </c>
       <c r="B87" s="8">
         <v>1997</v>
@@ -17224,7 +17224,7 @@
         <v>707</v>
       </c>
       <c r="Q90" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R90" s="9" t="s">
         <v>153</v>
@@ -17416,7 +17416,7 @@
         <v>638</v>
       </c>
       <c r="P93" s="22" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="Q93" s="9" t="s">
         <v>446</v>
@@ -17824,7 +17824,7 @@
     </row>
     <row r="100" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A100" s="12" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
       <c r="B100" s="10">
         <v>2016</v>
@@ -17939,7 +17939,7 @@
         <v>713</v>
       </c>
       <c r="Q101" s="9" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="R101" s="9" t="s">
         <v>153</v>
@@ -18069,7 +18069,7 @@
         <v>715</v>
       </c>
       <c r="Q103" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R103" s="9" t="s">
         <v>153</v>
@@ -18134,7 +18134,7 @@
         <v>716</v>
       </c>
       <c r="Q104" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R104" s="9" t="s">
         <v>153</v>
@@ -18199,7 +18199,7 @@
         <v>717</v>
       </c>
       <c r="Q105" s="9" t="s">
-        <v>847</v>
+        <v>1197</v>
       </c>
       <c r="R105" s="9" t="s">
         <v>153</v>
@@ -18264,7 +18264,7 @@
         <v>718</v>
       </c>
       <c r="Q106" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R106" s="9" t="s">
         <v>153</v>
@@ -18279,7 +18279,7 @@
     </row>
     <row r="107" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A107" s="7" t="s">
-        <v>1159</v>
+        <v>1158</v>
       </c>
       <c r="B107" s="10">
         <v>2017</v>
@@ -18297,7 +18297,7 @@
         <v>253</v>
       </c>
       <c r="G107" s="9" t="s">
-        <v>1158</v>
+        <v>1157</v>
       </c>
       <c r="H107" s="14">
         <f t="shared" si="6"/>
@@ -18326,7 +18326,7 @@
         <v>638</v>
       </c>
       <c r="P107" s="22" t="s">
-        <v>1157</v>
+        <v>1156</v>
       </c>
       <c r="Q107" s="9" t="s">
         <v>447</v>
@@ -18344,7 +18344,7 @@
     </row>
     <row r="108" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A108" s="7" t="s">
-        <v>1161</v>
+        <v>1160</v>
       </c>
       <c r="B108" s="10">
         <v>2007</v>
@@ -18362,7 +18362,7 @@
         <v>315</v>
       </c>
       <c r="G108" s="9" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="H108" s="14">
         <f t="shared" si="6"/>
@@ -18391,7 +18391,7 @@
         <v>638</v>
       </c>
       <c r="P108" s="22" t="s">
-        <v>1157</v>
+        <v>1156</v>
       </c>
       <c r="Q108" s="9" t="s">
         <v>447</v>
@@ -18669,7 +18669,7 @@
     </row>
     <row r="113" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A113" s="7" t="s">
-        <v>1168</v>
+        <v>1167</v>
       </c>
       <c r="B113" s="8">
         <v>2015</v>
@@ -18784,7 +18784,7 @@
         <v>723</v>
       </c>
       <c r="Q114" s="9" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
       <c r="R114" s="9" t="s">
         <v>153</v>
@@ -18849,7 +18849,7 @@
         <v>724</v>
       </c>
       <c r="Q115" s="9" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
       <c r="R115" s="9" t="s">
         <v>153</v>
@@ -18914,7 +18914,7 @@
         <v>725</v>
       </c>
       <c r="Q116" s="9" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
       <c r="R116" s="9" t="s">
         <v>153</v>
@@ -18979,7 +18979,7 @@
         <v>726</v>
       </c>
       <c r="Q117" s="9" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
       <c r="R117" s="9" t="s">
         <v>153</v>
@@ -19059,7 +19059,7 @@
     </row>
     <row r="119" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A119" s="7" t="s">
-        <v>1169</v>
+        <v>1168</v>
       </c>
       <c r="B119" s="10">
         <v>2016</v>
@@ -19124,7 +19124,7 @@
     </row>
     <row r="120" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A120" s="7" t="s">
-        <v>1170</v>
+        <v>1169</v>
       </c>
       <c r="B120" s="10">
         <v>2016</v>
@@ -19189,7 +19189,7 @@
     </row>
     <row r="121" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A121" s="7" t="s">
-        <v>1171</v>
+        <v>1170</v>
       </c>
       <c r="B121" s="10">
         <v>2016</v>
@@ -19498,7 +19498,7 @@
         <v>730</v>
       </c>
       <c r="Q125" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R125" s="9" t="s">
         <v>153</v>
@@ -19823,7 +19823,7 @@
         <v>735</v>
       </c>
       <c r="Q130" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R130" s="9" t="s">
         <v>153</v>
@@ -19888,7 +19888,7 @@
         <v>736</v>
       </c>
       <c r="Q131" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R131" s="9" t="s">
         <v>153</v>
@@ -20033,7 +20033,7 @@
     </row>
     <row r="134" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A134" s="7" t="s">
-        <v>1162</v>
+        <v>1161</v>
       </c>
       <c r="B134" s="10">
         <v>2018</v>
@@ -20148,7 +20148,7 @@
         <v>740</v>
       </c>
       <c r="Q135" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R135" s="9" t="s">
         <v>153</v>
@@ -20278,7 +20278,7 @@
         <v>742</v>
       </c>
       <c r="Q137" s="9" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
       <c r="R137" s="9" t="s">
         <v>153</v>
@@ -20343,7 +20343,7 @@
         <v>743</v>
       </c>
       <c r="Q138" s="9" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
       <c r="R138" s="9" t="s">
         <v>153</v>
@@ -20603,7 +20603,7 @@
         <v>747</v>
       </c>
       <c r="Q142" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R142" s="9" t="s">
         <v>153</v>
@@ -20668,7 +20668,7 @@
         <v>748</v>
       </c>
       <c r="Q143" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R143" s="9" t="s">
         <v>153</v>
@@ -21058,7 +21058,7 @@
         <v>752</v>
       </c>
       <c r="Q149" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R149" s="9" t="s">
         <v>153</v>
@@ -21123,7 +21123,7 @@
         <v>648</v>
       </c>
       <c r="Q150" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R150" s="9" t="s">
         <v>153</v>
@@ -21708,7 +21708,7 @@
         <v>759</v>
       </c>
       <c r="Q159" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R159" s="9" t="s">
         <v>152</v>
@@ -22423,7 +22423,7 @@
         <v>768</v>
       </c>
       <c r="Q170" s="9" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
       <c r="R170" s="9" t="s">
         <v>153</v>
@@ -22748,7 +22748,7 @@
         <v>772</v>
       </c>
       <c r="Q175" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R175" s="9" t="s">
         <v>152</v>
@@ -23088,7 +23088,7 @@
     </row>
     <row r="181" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A181" s="7" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="B181" s="10">
         <v>2013</v>
@@ -23333,7 +23333,7 @@
         <v>648</v>
       </c>
       <c r="Q184" s="9" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
       <c r="R184" s="9" t="s">
         <v>153</v>
@@ -23658,7 +23658,7 @@
         <v>779</v>
       </c>
       <c r="Q189" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R189" s="9" t="s">
         <v>152</v>
@@ -23723,7 +23723,7 @@
         <v>780</v>
       </c>
       <c r="Q190" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R190" s="9" t="s">
         <v>152</v>
@@ -23853,7 +23853,7 @@
         <v>648</v>
       </c>
       <c r="Q192" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R192" s="9" t="s">
         <v>153</v>
@@ -25218,7 +25218,7 @@
         <v>793</v>
       </c>
       <c r="Q213" s="9" t="s">
-        <v>847</v>
+        <v>1197</v>
       </c>
       <c r="R213" s="9" t="s">
         <v>153</v>
@@ -25283,7 +25283,7 @@
         <v>794</v>
       </c>
       <c r="Q214" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R214" s="9" t="s">
         <v>153</v>
@@ -25348,7 +25348,7 @@
         <v>795</v>
       </c>
       <c r="Q215" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R215" s="9" t="s">
         <v>153</v>
@@ -25478,7 +25478,7 @@
         <v>797</v>
       </c>
       <c r="Q217" s="9" t="s">
-        <v>847</v>
+        <v>1197</v>
       </c>
       <c r="R217" s="9" t="s">
         <v>153</v>
@@ -25543,7 +25543,7 @@
         <v>798</v>
       </c>
       <c r="Q218" s="9" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="R218" s="9" t="s">
         <v>153</v>
@@ -25673,7 +25673,7 @@
         <v>800</v>
       </c>
       <c r="Q220" s="9" t="s">
-        <v>847</v>
+        <v>1197</v>
       </c>
       <c r="R220" s="9" t="s">
         <v>153</v>
@@ -25738,7 +25738,7 @@
         <v>648</v>
       </c>
       <c r="Q221" s="9" t="s">
-        <v>847</v>
+        <v>1197</v>
       </c>
       <c r="R221" s="9" t="s">
         <v>153</v>
@@ -26193,7 +26193,7 @@
         <v>60</v>
       </c>
       <c r="Q228" s="9" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
       <c r="R228" s="9" t="s">
         <v>153</v>
@@ -26663,7 +26663,7 @@
     </row>
     <row r="236" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A236" s="7" t="s">
-        <v>1164</v>
+        <v>1163</v>
       </c>
       <c r="B236" s="10">
         <v>2009</v>
@@ -26681,7 +26681,7 @@
         <v>206</v>
       </c>
       <c r="G236" s="9" t="s">
-        <v>1163</v>
+        <v>1162</v>
       </c>
       <c r="H236" s="9">
         <f t="shared" si="32"/>
@@ -26710,7 +26710,7 @@
         <v>638</v>
       </c>
       <c r="P236" s="22" t="s">
-        <v>1157</v>
+        <v>1156</v>
       </c>
       <c r="Q236" s="9" t="s">
         <v>447</v>
@@ -26778,7 +26778,7 @@
         <v>809</v>
       </c>
       <c r="Q237" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R237" s="9" t="s">
         <v>153</v>
@@ -26908,7 +26908,7 @@
         <v>831</v>
       </c>
       <c r="Q239" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R239" s="9" t="s">
         <v>153</v>
@@ -27038,7 +27038,7 @@
         <v>819</v>
       </c>
       <c r="Q241" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R241" s="9" t="s">
         <v>153</v>
@@ -27168,7 +27168,7 @@
         <v>58</v>
       </c>
       <c r="Q243" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R243" s="9" t="s">
         <v>153</v>
@@ -27233,7 +27233,7 @@
         <v>648</v>
       </c>
       <c r="Q244" s="9" t="s">
-        <v>847</v>
+        <v>1197</v>
       </c>
       <c r="R244" s="9" t="s">
         <v>153</v>
@@ -27558,7 +27558,7 @@
         <v>841</v>
       </c>
       <c r="Q249" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R249" s="9" t="s">
         <v>153</v>
@@ -27638,7 +27638,7 @@
     </row>
     <row r="251" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A251" s="7" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="B251" s="14">
         <v>2023</v>
@@ -27656,7 +27656,7 @@
         <v>280</v>
       </c>
       <c r="G251" s="9" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="H251" s="14">
         <f t="shared" si="32"/>
@@ -27673,7 +27673,7 @@
         <v>153</v>
       </c>
       <c r="L251" s="11" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="M251" s="8">
         <v>2</v>
@@ -27685,7 +27685,7 @@
         <v>638</v>
       </c>
       <c r="P251" s="12" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="Q251" s="9" t="s">
         <v>544</v>
@@ -27703,7 +27703,7 @@
     </row>
     <row r="252" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A252" s="7" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="B252" s="14">
         <v>2021</v>
@@ -27721,7 +27721,7 @@
         <v>391</v>
       </c>
       <c r="G252" s="9" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="H252" s="14">
         <f t="shared" si="32"/>
@@ -27750,7 +27750,7 @@
         <v>638</v>
       </c>
       <c r="P252" s="12" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="Q252" s="9" t="s">
         <v>544</v>
@@ -27768,7 +27768,7 @@
     </row>
     <row r="253" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A253" s="7" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="B253" s="14">
         <v>2020</v>
@@ -27786,7 +27786,7 @@
         <v>177</v>
       </c>
       <c r="G253" s="9" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="H253" s="14">
         <f t="shared" si="32"/>
@@ -27815,7 +27815,7 @@
         <v>638</v>
       </c>
       <c r="P253" s="12" t="s">
-        <v>1012</v>
+        <v>1011</v>
       </c>
       <c r="Q253" s="9" t="s">
         <v>544</v>
@@ -27833,7 +27833,7 @@
     </row>
     <row r="254" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A254" s="7" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="B254" s="14">
         <v>2018</v>
@@ -27851,7 +27851,7 @@
         <v>105</v>
       </c>
       <c r="G254" s="9" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="H254" s="14">
         <f t="shared" si="32"/>
@@ -27880,10 +27880,10 @@
         <v>638</v>
       </c>
       <c r="P254" s="38" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="Q254" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R254" s="9" t="s">
         <v>153</v>
@@ -27898,7 +27898,7 @@
     </row>
     <row r="255" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A255" s="7" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="B255" s="14">
         <v>2023</v>
@@ -27916,7 +27916,7 @@
         <v>240</v>
       </c>
       <c r="G255" s="9" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="H255" s="14">
         <f t="shared" si="32"/>
@@ -27945,7 +27945,7 @@
         <v>638</v>
       </c>
       <c r="P255" s="7" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="Q255" s="9" t="s">
         <v>447</v>
@@ -27963,7 +27963,7 @@
     </row>
     <row r="256" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A256" s="7" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="B256" s="14">
         <v>2023</v>
@@ -27981,7 +27981,7 @@
         <v>51</v>
       </c>
       <c r="G256" s="9" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="H256" s="14">
         <f t="shared" si="32"/>
@@ -27998,7 +27998,7 @@
         <v>153</v>
       </c>
       <c r="L256" s="9" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="M256" s="10">
         <v>2</v>
@@ -28010,7 +28010,7 @@
         <v>638</v>
       </c>
       <c r="P256" s="7" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="Q256" s="9" t="s">
         <v>544</v>
@@ -28028,7 +28028,7 @@
     </row>
     <row r="257" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A257" s="7" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="B257" s="14">
         <v>2023</v>
@@ -28046,7 +28046,7 @@
         <v>184</v>
       </c>
       <c r="G257" s="9" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="H257" s="14">
         <f t="shared" si="32"/>
@@ -28075,10 +28075,10 @@
         <v>638</v>
       </c>
       <c r="P257" s="12" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="Q257" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R257" s="9" t="s">
         <v>153</v>
@@ -28093,7 +28093,7 @@
     </row>
     <row r="258" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A258" s="7" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="B258" s="14">
         <v>2023</v>
@@ -28111,7 +28111,7 @@
         <v>203</v>
       </c>
       <c r="G258" s="9" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="H258" s="14">
         <f t="shared" si="32"/>
@@ -28140,7 +28140,7 @@
         <v>638</v>
       </c>
       <c r="P258" s="9" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="Q258" s="9" t="s">
         <v>447</v>
@@ -28158,7 +28158,7 @@
     </row>
     <row r="259" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A259" s="7" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="B259" s="14">
         <v>2021</v>
@@ -28176,7 +28176,7 @@
         <v>338</v>
       </c>
       <c r="G259" s="9" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="H259" s="14">
         <f t="shared" si="32"/>
@@ -28205,7 +28205,7 @@
         <v>638</v>
       </c>
       <c r="P259" s="7" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="Q259" s="9" t="s">
         <v>544</v>
@@ -28223,7 +28223,7 @@
     </row>
     <row r="260" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A260" s="7" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="B260" s="14">
         <v>2018</v>
@@ -28241,7 +28241,7 @@
         <v>229</v>
       </c>
       <c r="G260" s="9" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="H260" s="14">
         <f t="shared" si="32"/>
@@ -28270,7 +28270,7 @@
         <v>638</v>
       </c>
       <c r="P260" s="7" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="Q260" s="9" t="s">
         <v>846</v>
@@ -28288,7 +28288,7 @@
     </row>
     <row r="261" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A261" s="7" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="B261" s="14">
         <v>2022</v>
@@ -28306,7 +28306,7 @@
         <v>94</v>
       </c>
       <c r="G261" s="9" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="H261" s="14">
         <f t="shared" ref="H261:H263" si="35">YEAR(G261)</f>
@@ -28335,7 +28335,7 @@
         <v>638</v>
       </c>
       <c r="P261" s="7" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="Q261" s="9" t="s">
         <v>544</v>
@@ -28353,7 +28353,7 @@
     </row>
     <row r="262" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A262" s="7" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="B262" s="14">
         <v>2022</v>
@@ -28371,7 +28371,7 @@
         <v>265</v>
       </c>
       <c r="G262" s="9" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="H262" s="14">
         <f t="shared" si="35"/>
@@ -28400,7 +28400,7 @@
         <v>638</v>
       </c>
       <c r="P262" s="12" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="Q262" s="9" t="s">
         <v>544</v>
@@ -28418,7 +28418,7 @@
     </row>
     <row r="263" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A263" s="7" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="B263" s="14">
         <v>2023</v>
@@ -28436,7 +28436,7 @@
         <v>288</v>
       </c>
       <c r="G263" s="9" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="H263" s="9">
         <f t="shared" si="35"/>
@@ -28465,7 +28465,7 @@
         <v>638</v>
       </c>
       <c r="P263" s="12" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="Q263" s="9" t="s">
         <v>544</v>
@@ -28483,7 +28483,7 @@
     </row>
     <row r="264" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A264" s="7" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="B264" s="14">
         <v>2023</v>
@@ -28501,7 +28501,7 @@
         <v>151</v>
       </c>
       <c r="G264" s="9" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="H264" s="9">
         <f t="shared" ref="H264" si="37">YEAR(G264)</f>
@@ -28530,7 +28530,7 @@
         <v>638</v>
       </c>
       <c r="P264" s="7" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="Q264" s="9" t="s">
         <v>447</v>
@@ -28548,7 +28548,7 @@
     </row>
     <row r="265" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A265" s="7" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="B265" s="14">
         <v>2022</v>
@@ -28566,7 +28566,7 @@
         <v>416</v>
       </c>
       <c r="G265" s="9" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="H265" s="9">
         <f t="shared" ref="H265:H267" si="39">YEAR(G265)</f>
@@ -28595,7 +28595,7 @@
         <v>638</v>
       </c>
       <c r="P265" s="7" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="Q265" s="9" t="s">
         <v>447</v>
@@ -28613,7 +28613,7 @@
     </row>
     <row r="266" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A266" s="7" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="B266" s="14">
         <v>2022</v>
@@ -28631,7 +28631,7 @@
         <v>535</v>
       </c>
       <c r="G266" s="9" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="H266" s="9">
         <f t="shared" si="39"/>
@@ -28660,7 +28660,7 @@
         <v>638</v>
       </c>
       <c r="P266" s="7" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="Q266" s="9" t="s">
         <v>846</v>
@@ -28678,7 +28678,7 @@
     </row>
     <row r="267" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A267" s="7" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="B267" s="14">
         <v>2018</v>
@@ -28696,7 +28696,7 @@
         <v>429</v>
       </c>
       <c r="G267" s="9" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="H267" s="9">
         <f t="shared" si="39"/>
@@ -28725,7 +28725,7 @@
         <v>638</v>
       </c>
       <c r="P267" s="12" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="Q267" s="9" t="s">
         <v>447</v>
@@ -28743,7 +28743,7 @@
     </row>
     <row r="268" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A268" s="7" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="B268" s="14">
         <v>2023</v>
@@ -28761,7 +28761,7 @@
         <v>455</v>
       </c>
       <c r="G268" s="9" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="H268" s="9">
         <f t="shared" ref="H268:H269" si="41">YEAR(G268)</f>
@@ -28790,7 +28790,7 @@
         <v>638</v>
       </c>
       <c r="P268" s="39" t="s">
-        <v>1006</v>
+        <v>1005</v>
       </c>
       <c r="Q268" s="9" t="s">
         <v>544</v>
@@ -28808,7 +28808,7 @@
     </row>
     <row r="269" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A269" s="7" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="B269" s="14">
         <v>2023</v>
@@ -28826,7 +28826,7 @@
         <v>268</v>
       </c>
       <c r="G269" s="9" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="H269" s="9">
         <f t="shared" si="41"/>
@@ -28855,7 +28855,7 @@
         <v>638</v>
       </c>
       <c r="P269" s="12" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="Q269" s="9" t="s">
         <v>544</v>
@@ -28873,7 +28873,7 @@
     </row>
     <row r="270" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A270" s="7" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="B270" s="14">
         <v>2022</v>
@@ -28891,7 +28891,7 @@
         <v>205</v>
       </c>
       <c r="G270" s="9" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="H270" s="9">
         <f t="shared" ref="H270" si="43">YEAR(G270)</f>
@@ -28920,7 +28920,7 @@
         <v>638</v>
       </c>
       <c r="P270" s="12" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="Q270" s="9" t="s">
         <v>544</v>
@@ -28938,7 +28938,7 @@
     </row>
     <row r="271" spans="1:20" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A271" s="7" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="B271" s="14">
         <v>2022</v>
@@ -28956,7 +28956,7 @@
         <v>94</v>
       </c>
       <c r="G271" s="9" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="H271" s="9">
         <f t="shared" ref="H271" si="45">YEAR(G271)</f>
@@ -28985,7 +28985,7 @@
         <v>638</v>
       </c>
       <c r="P271" s="7" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="Q271" s="9" t="s">
         <v>544</v>
@@ -29003,7 +29003,7 @@
     </row>
     <row r="272" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A272" s="7" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="B272" s="14">
         <v>2020</v>
@@ -29021,7 +29021,7 @@
         <v>132</v>
       </c>
       <c r="G272" s="9" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="H272" s="9">
         <f t="shared" ref="H272:H273" si="47">YEAR(G272)</f>
@@ -29050,7 +29050,7 @@
         <v>638</v>
       </c>
       <c r="P272" s="7" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="Q272" s="9" t="s">
         <v>544</v>
@@ -29068,7 +29068,7 @@
     </row>
     <row r="273" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A273" s="7" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="B273" s="14">
         <v>2021</v>
@@ -29086,7 +29086,7 @@
         <v>715</v>
       </c>
       <c r="G273" s="9" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="H273" s="9">
         <f t="shared" si="47"/>
@@ -29115,7 +29115,7 @@
         <v>638</v>
       </c>
       <c r="P273" s="7" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="Q273" s="9" t="s">
         <v>544</v>
@@ -29133,7 +29133,7 @@
     </row>
     <row r="274" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A274" s="7" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="B274" s="14">
         <v>2023</v>
@@ -29151,7 +29151,7 @@
         <v>192</v>
       </c>
       <c r="G274" s="9" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="H274" s="9">
         <f t="shared" ref="H274" si="49">YEAR(G274)</f>
@@ -29168,7 +29168,7 @@
         <v>153</v>
       </c>
       <c r="L274" s="9" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="M274" s="14">
         <v>1</v>
@@ -29180,7 +29180,7 @@
         <v>638</v>
       </c>
       <c r="P274" s="7" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="Q274" s="9" t="s">
         <v>544</v>
@@ -29198,7 +29198,7 @@
     </row>
     <row r="275" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A275" s="7" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="B275" s="14">
         <v>2024</v>
@@ -29216,7 +29216,7 @@
         <v>139</v>
       </c>
       <c r="G275" s="9" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="H275" s="9">
         <f t="shared" ref="H275" si="51">YEAR(G275)</f>
@@ -29233,7 +29233,7 @@
         <v>153</v>
       </c>
       <c r="L275" s="9" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="M275" s="14">
         <v>1</v>
@@ -29245,7 +29245,7 @@
         <v>638</v>
       </c>
       <c r="P275" s="7" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="Q275" s="9" t="s">
         <v>544</v>
@@ -29263,7 +29263,7 @@
     </row>
     <row r="276" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A276" s="7" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="B276" s="14">
         <v>2023</v>
@@ -29281,7 +29281,7 @@
         <v>963</v>
       </c>
       <c r="G276" s="9" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="H276" s="9">
         <f t="shared" ref="H276" si="53">YEAR(G276)</f>
@@ -29310,7 +29310,7 @@
         <v>638</v>
       </c>
       <c r="P276" s="7" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="Q276" s="9" t="s">
         <v>544</v>
@@ -29328,7 +29328,7 @@
     </row>
     <row r="277" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A277" s="7" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
       <c r="B277" s="14">
         <v>2024</v>
@@ -29346,7 +29346,7 @@
         <v>229</v>
       </c>
       <c r="G277" s="9" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="H277" s="9">
         <f t="shared" ref="H277:H278" si="55">YEAR(G277)</f>
@@ -29363,7 +29363,7 @@
         <v>152</v>
       </c>
       <c r="L277" s="9" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="M277" s="14">
         <v>2</v>
@@ -29375,7 +29375,7 @@
         <v>638</v>
       </c>
       <c r="P277" s="7" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="Q277" s="9" t="s">
         <v>544</v>
@@ -29393,7 +29393,7 @@
     </row>
     <row r="278" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A278" s="7" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="B278" s="14">
         <v>2018</v>
@@ -29411,7 +29411,7 @@
         <v>978</v>
       </c>
       <c r="G278" s="9" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="H278" s="9">
         <f t="shared" si="55"/>
@@ -29440,7 +29440,7 @@
         <v>638</v>
       </c>
       <c r="P278" s="7" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="Q278" s="9" t="s">
         <v>544</v>
@@ -29458,7 +29458,7 @@
     </row>
     <row r="279" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A279" s="7" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="B279" s="14">
         <v>2022</v>
@@ -29476,7 +29476,7 @@
         <v>264</v>
       </c>
       <c r="G279" s="9" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="H279" s="9">
         <f t="shared" ref="H279" si="57">YEAR(G279)</f>
@@ -29505,7 +29505,7 @@
         <v>638</v>
       </c>
       <c r="P279" s="7" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="Q279" s="9" t="s">
         <v>544</v>
@@ -29523,7 +29523,7 @@
     </row>
     <row r="280" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A280" s="7" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="B280" s="14">
         <v>2022</v>
@@ -29541,7 +29541,7 @@
         <v>243</v>
       </c>
       <c r="G280" s="9" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="H280" s="9">
         <f t="shared" ref="H280:H283" si="59">YEAR(G280)</f>
@@ -29558,7 +29558,7 @@
         <v>153</v>
       </c>
       <c r="L280" s="9" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="M280" s="14">
         <v>4</v>
@@ -29570,7 +29570,7 @@
         <v>638</v>
       </c>
       <c r="P280" s="7" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="Q280" s="9" t="s">
         <v>544</v>
@@ -29588,7 +29588,7 @@
     </row>
     <row r="281" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A281" s="7" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="B281" s="14">
         <v>2024</v>
@@ -29606,7 +29606,7 @@
         <v>337</v>
       </c>
       <c r="G281" s="9" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="H281" s="9">
         <f t="shared" si="59"/>
@@ -29635,10 +29635,10 @@
         <v>638</v>
       </c>
       <c r="P281" s="7" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="Q281" s="9" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="R281" s="9" t="s">
         <v>153</v>
@@ -29653,7 +29653,7 @@
     </row>
     <row r="282" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A282" s="7" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="B282" s="14">
         <v>2024</v>
@@ -29671,7 +29671,7 @@
         <v>253</v>
       </c>
       <c r="G282" s="9" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="H282" s="9">
         <f t="shared" si="59"/>
@@ -29700,10 +29700,10 @@
         <v>638</v>
       </c>
       <c r="P282" s="7" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
       <c r="Q282" s="9" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="R282" s="9" t="s">
         <v>153</v>
@@ -29718,7 +29718,7 @@
     </row>
     <row r="283" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A283" s="7" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="B283" s="14">
         <v>2024</v>
@@ -29736,7 +29736,7 @@
         <v>316</v>
       </c>
       <c r="G283" s="9" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="H283" s="9">
         <f t="shared" si="59"/>
@@ -29765,10 +29765,10 @@
         <v>638</v>
       </c>
       <c r="P283" s="7" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="Q283" s="9" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="R283" s="9" t="s">
         <v>153</v>
@@ -29783,7 +29783,7 @@
     </row>
     <row r="284" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A284" s="7" t="s">
-        <v>1165</v>
+        <v>1164</v>
       </c>
       <c r="B284" s="14">
         <v>2024</v>
@@ -29801,7 +29801,7 @@
         <v>112</v>
       </c>
       <c r="G284" s="9" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="H284" s="9">
         <f t="shared" ref="H284" si="62">YEAR(G284)</f>
@@ -29818,7 +29818,7 @@
         <v>153</v>
       </c>
       <c r="L284" s="9" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
       <c r="M284" s="14">
         <v>3</v>
@@ -29830,10 +29830,10 @@
         <v>638</v>
       </c>
       <c r="P284" s="7" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="Q284" s="9" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="R284" s="9" t="s">
         <v>153</v>
@@ -29848,7 +29848,7 @@
     </row>
     <row r="285" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A285" s="7" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="B285" s="14">
         <v>2024</v>
@@ -29866,7 +29866,7 @@
         <v>1779</v>
       </c>
       <c r="G285" s="9" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="H285" s="9">
         <f t="shared" ref="H285:H287" si="63">YEAR(G285)</f>
@@ -29895,10 +29895,10 @@
         <v>638</v>
       </c>
       <c r="P285" s="7" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="Q285" s="9" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="R285" s="9" t="s">
         <v>153</v>
@@ -29913,7 +29913,7 @@
     </row>
     <row r="286" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A286" s="7" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="B286" s="14">
         <v>2022</v>
@@ -29931,7 +29931,7 @@
         <v>365</v>
       </c>
       <c r="G286" s="9" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="H286" s="9">
         <f t="shared" si="63"/>
@@ -29960,10 +29960,10 @@
         <v>638</v>
       </c>
       <c r="P286" s="12" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="Q286" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R286" s="9" t="s">
         <v>153</v>
@@ -29978,7 +29978,7 @@
     </row>
     <row r="287" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A287" s="7" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="B287" s="14">
         <v>2023</v>
@@ -29996,7 +29996,7 @@
         <v>340</v>
       </c>
       <c r="G287" s="9" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="H287" s="9">
         <f t="shared" si="63"/>
@@ -30025,7 +30025,7 @@
         <v>638</v>
       </c>
       <c r="P287" s="7" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="Q287" s="9" t="s">
         <v>447</v>
@@ -30043,7 +30043,7 @@
     </row>
     <row r="288" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A288" s="7" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="B288" s="14">
         <v>2023</v>
@@ -30061,7 +30061,7 @@
         <v>600</v>
       </c>
       <c r="G288" s="9" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="H288" s="9">
         <f t="shared" ref="H288" si="64">YEAR(G288)</f>
@@ -30090,7 +30090,7 @@
         <v>638</v>
       </c>
       <c r="P288" s="7" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
       <c r="Q288" s="9" t="s">
         <v>447</v>
@@ -30108,7 +30108,7 @@
     </row>
     <row r="289" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A289" s="7" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
       <c r="B289" s="14">
         <v>2024</v>
@@ -30126,7 +30126,7 @@
         <v>289</v>
       </c>
       <c r="G289" s="9" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="H289" s="9">
         <f t="shared" ref="H289" si="66">YEAR(G289)</f>
@@ -30155,7 +30155,7 @@
         <v>638</v>
       </c>
       <c r="P289" s="7" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="Q289" s="9" t="s">
         <v>544</v>
@@ -30173,7 +30173,7 @@
     </row>
     <row r="290" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A290" s="7" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="B290" s="14">
         <v>2024</v>
@@ -30191,7 +30191,7 @@
         <v>198</v>
       </c>
       <c r="G290" s="9" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="H290" s="9">
         <f t="shared" ref="H290" si="68">YEAR(G290)</f>
@@ -30220,10 +30220,10 @@
         <v>638</v>
       </c>
       <c r="P290" s="12" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="Q290" s="9" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="R290" s="9" t="s">
         <v>153</v>
@@ -30238,7 +30238,7 @@
     </row>
     <row r="291" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A291" s="7" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="B291" s="14">
         <v>2024</v>
@@ -30256,7 +30256,7 @@
         <v>224</v>
       </c>
       <c r="G291" s="9" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="H291" s="9">
         <f t="shared" ref="H291" si="70">YEAR(G291)</f>
@@ -30285,10 +30285,10 @@
         <v>638</v>
       </c>
       <c r="P291" s="12" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="Q291" s="9" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="R291" s="9" t="s">
         <v>153</v>
@@ -30303,7 +30303,7 @@
     </row>
     <row r="292" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A292" s="7" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
       <c r="B292" s="14">
         <v>2022</v>
@@ -30321,7 +30321,7 @@
         <v>296</v>
       </c>
       <c r="G292" s="9" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="H292" s="9">
         <f t="shared" ref="H292" si="72">YEAR(G292)</f>
@@ -30350,10 +30350,10 @@
         <v>638</v>
       </c>
       <c r="P292" s="12" t="s">
-        <v>957</v>
+        <v>956</v>
       </c>
       <c r="Q292" s="9" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="R292" s="9" t="s">
         <v>153</v>
@@ -30368,7 +30368,7 @@
     </row>
     <row r="293" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A293" s="7" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
       <c r="B293" s="14">
         <v>2023</v>
@@ -30386,7 +30386,7 @@
         <v>200</v>
       </c>
       <c r="G293" s="9" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
       <c r="H293" s="9">
         <f t="shared" ref="H293" si="75">YEAR(G293)</f>
@@ -30415,10 +30415,10 @@
         <v>638</v>
       </c>
       <c r="P293" s="12" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="Q293" s="9" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="R293" s="9" t="s">
         <v>153</v>
@@ -30433,7 +30433,7 @@
     </row>
     <row r="294" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A294" s="7" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
       <c r="B294" s="14">
         <v>2023</v>
@@ -30451,7 +30451,7 @@
         <v>255</v>
       </c>
       <c r="G294" s="9" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
       <c r="H294" s="9">
         <f t="shared" ref="H294" si="78">YEAR(G294)</f>
@@ -30480,7 +30480,7 @@
         <v>638</v>
       </c>
       <c r="P294" s="12" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
       <c r="Q294" s="9" t="s">
         <v>447</v>
@@ -30498,7 +30498,7 @@
     </row>
     <row r="295" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A295" s="7" t="s">
-        <v>964</v>
+        <v>963</v>
       </c>
       <c r="B295" s="14">
         <v>2023</v>
@@ -30516,7 +30516,7 @@
         <v>192</v>
       </c>
       <c r="G295" s="9" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
       <c r="H295" s="9">
         <f t="shared" ref="H295" si="81">YEAR(G295)</f>
@@ -30545,10 +30545,10 @@
         <v>638</v>
       </c>
       <c r="P295" s="12" t="s">
-        <v>965</v>
+        <v>964</v>
       </c>
       <c r="Q295" s="9" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="R295" s="9" t="s">
         <v>153</v>
@@ -30563,7 +30563,7 @@
     </row>
     <row r="296" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A296" s="7" t="s">
-        <v>966</v>
+        <v>965</v>
       </c>
       <c r="B296" s="14">
         <v>2015</v>
@@ -30581,7 +30581,7 @@
         <v>96</v>
       </c>
       <c r="G296" s="9" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
       <c r="H296" s="9">
         <f t="shared" ref="H296" si="84">YEAR(G296)</f>
@@ -30598,7 +30598,7 @@
         <v>153</v>
       </c>
       <c r="L296" s="9" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
       <c r="M296" s="14">
         <v>3</v>
@@ -30613,7 +30613,7 @@
         <v>681</v>
       </c>
       <c r="Q296" s="9" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="R296" s="9" t="s">
         <v>153</v>
@@ -30628,7 +30628,7 @@
     </row>
     <row r="297" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A297" s="7" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="B297" s="14">
         <v>2022</v>
@@ -30646,7 +30646,7 @@
         <v>194</v>
       </c>
       <c r="G297" s="9" t="s">
-        <v>968</v>
+        <v>967</v>
       </c>
       <c r="H297" s="9">
         <f t="shared" ref="H297" si="86">YEAR(G297)</f>
@@ -30663,7 +30663,7 @@
         <v>153</v>
       </c>
       <c r="L297" s="9" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
       <c r="M297" s="14">
         <v>3</v>
@@ -30675,10 +30675,10 @@
         <v>638</v>
       </c>
       <c r="P297" s="22" t="s">
-        <v>969</v>
+        <v>968</v>
       </c>
       <c r="Q297" s="9" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="R297" s="9" t="s">
         <v>153</v>
@@ -30693,7 +30693,7 @@
     </row>
     <row r="298" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A298" s="7" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
       <c r="B298" s="14">
         <v>2018</v>
@@ -30711,7 +30711,7 @@
         <v>188</v>
       </c>
       <c r="G298" s="9" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
       <c r="H298" s="9">
         <f t="shared" ref="H298:H300" si="88">YEAR(G298)</f>
@@ -30728,7 +30728,7 @@
         <v>153</v>
       </c>
       <c r="L298" s="9" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
       <c r="M298" s="14">
         <v>4</v>
@@ -30740,7 +30740,7 @@
         <v>638</v>
       </c>
       <c r="P298" s="12" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
       <c r="Q298" s="9" t="s">
         <v>447</v>
@@ -30758,7 +30758,7 @@
     </row>
     <row r="299" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A299" s="7" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
       <c r="B299" s="14">
         <v>2021</v>
@@ -30776,7 +30776,7 @@
         <v>631</v>
       </c>
       <c r="G299" s="9" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
       <c r="H299" s="9">
         <f t="shared" si="88"/>
@@ -30805,7 +30805,7 @@
         <v>638</v>
       </c>
       <c r="P299" s="12" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="Q299" s="9" t="s">
         <v>544</v>
@@ -30823,7 +30823,7 @@
     </row>
     <row r="300" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A300" s="7" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
       <c r="B300" s="14">
         <v>2023</v>
@@ -30841,7 +30841,7 @@
         <v>318</v>
       </c>
       <c r="G300" s="9" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="H300" s="9">
         <f t="shared" si="88"/>
@@ -30870,7 +30870,7 @@
         <v>638</v>
       </c>
       <c r="P300" s="12" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
       <c r="Q300" s="9" t="s">
         <v>845</v>
@@ -30888,7 +30888,7 @@
     </row>
     <row r="301" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A301" s="7" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="B301" s="14">
         <v>2023</v>
@@ -30906,7 +30906,7 @@
         <v>298</v>
       </c>
       <c r="G301" s="9" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="H301" s="9">
         <f t="shared" ref="H301" si="90">YEAR(G301)</f>
@@ -30935,7 +30935,7 @@
         <v>638</v>
       </c>
       <c r="P301" s="12" t="s">
-        <v>982</v>
+        <v>981</v>
       </c>
       <c r="Q301" s="9" t="s">
         <v>845</v>
@@ -30953,7 +30953,7 @@
     </row>
     <row r="302" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A302" s="7" t="s">
-        <v>983</v>
+        <v>982</v>
       </c>
       <c r="B302" s="14">
         <v>2023</v>
@@ -30971,7 +30971,7 @@
         <v>636</v>
       </c>
       <c r="G302" s="9" t="s">
-        <v>984</v>
+        <v>983</v>
       </c>
       <c r="H302" s="9">
         <f t="shared" ref="H302" si="92">YEAR(G302)</f>
@@ -31000,7 +31000,7 @@
         <v>638</v>
       </c>
       <c r="P302" s="12" t="s">
-        <v>982</v>
+        <v>981</v>
       </c>
       <c r="Q302" s="9" t="s">
         <v>544</v>
@@ -31018,7 +31018,7 @@
     </row>
     <row r="303" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A303" s="12" t="s">
-        <v>985</v>
+        <v>984</v>
       </c>
       <c r="B303" s="14">
         <v>2023</v>
@@ -31036,7 +31036,7 @@
         <v>218</v>
       </c>
       <c r="G303" s="9" t="s">
-        <v>984</v>
+        <v>983</v>
       </c>
       <c r="H303" s="9">
         <f t="shared" ref="H303" si="94">YEAR(G303)</f>
@@ -31065,7 +31065,7 @@
         <v>638</v>
       </c>
       <c r="P303" s="12" t="s">
-        <v>986</v>
+        <v>985</v>
       </c>
       <c r="Q303" s="9" t="s">
         <v>544</v>
@@ -31083,7 +31083,7 @@
     </row>
     <row r="304" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A304" s="7" t="s">
-        <v>987</v>
+        <v>986</v>
       </c>
       <c r="B304" s="14">
         <v>2022</v>
@@ -31101,7 +31101,7 @@
         <v>464</v>
       </c>
       <c r="G304" s="9" t="s">
-        <v>988</v>
+        <v>987</v>
       </c>
       <c r="H304" s="9">
         <f t="shared" ref="H304" si="96">YEAR(G304)</f>
@@ -31118,7 +31118,7 @@
         <v>152</v>
       </c>
       <c r="L304" s="9" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="M304" s="14">
         <v>3</v>
@@ -31130,7 +31130,7 @@
         <v>638</v>
       </c>
       <c r="P304" s="12" t="s">
-        <v>989</v>
+        <v>988</v>
       </c>
       <c r="Q304" s="9" t="s">
         <v>544</v>
@@ -31148,7 +31148,7 @@
     </row>
     <row r="305" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A305" s="7" t="s">
-        <v>990</v>
+        <v>989</v>
       </c>
       <c r="B305" s="14">
         <v>2023</v>
@@ -31166,7 +31166,7 @@
         <v>58</v>
       </c>
       <c r="G305" s="9" t="s">
-        <v>988</v>
+        <v>987</v>
       </c>
       <c r="H305" s="9">
         <f t="shared" ref="H305" si="98">YEAR(G305)</f>
@@ -31195,10 +31195,10 @@
         <v>638</v>
       </c>
       <c r="P305" s="22" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
       <c r="Q305" s="9" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="R305" s="9" t="s">
         <v>153</v>
@@ -31213,7 +31213,7 @@
     </row>
     <row r="306" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A306" s="7" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
       <c r="B306" s="14">
         <v>2023</v>
@@ -31231,7 +31231,7 @@
         <v>161</v>
       </c>
       <c r="G306" s="9" t="s">
-        <v>988</v>
+        <v>987</v>
       </c>
       <c r="H306" s="9">
         <f t="shared" ref="H306" si="100">YEAR(G306)</f>
@@ -31260,10 +31260,10 @@
         <v>638</v>
       </c>
       <c r="P306" s="7" t="s">
-        <v>993</v>
+        <v>992</v>
       </c>
       <c r="Q306" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R306" s="9" t="s">
         <v>153</v>
@@ -31278,7 +31278,7 @@
     </row>
     <row r="307" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A307" s="7" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="B307" s="14">
         <v>2023</v>
@@ -31296,7 +31296,7 @@
         <v>331</v>
       </c>
       <c r="G307" s="9" t="s">
-        <v>988</v>
+        <v>987</v>
       </c>
       <c r="H307" s="9">
         <f t="shared" ref="H307" si="102">YEAR(G307)</f>
@@ -31325,7 +31325,7 @@
         <v>638</v>
       </c>
       <c r="P307" s="12" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="Q307" s="9" t="s">
         <v>447</v>
@@ -31343,7 +31343,7 @@
     </row>
     <row r="308" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A308" s="7" t="s">
-        <v>996</v>
+        <v>995</v>
       </c>
       <c r="B308" s="14">
         <v>2024</v>
@@ -31361,7 +31361,7 @@
         <v>179</v>
       </c>
       <c r="G308" s="9" t="s">
-        <v>999</v>
+        <v>998</v>
       </c>
       <c r="H308" s="9">
         <f t="shared" ref="H308" si="104">YEAR(G308)</f>
@@ -31390,7 +31390,7 @@
         <v>638</v>
       </c>
       <c r="P308" s="7" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
       <c r="Q308" s="9" t="s">
         <v>476</v>
@@ -31408,7 +31408,7 @@
     </row>
     <row r="309" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A309" s="7" t="s">
-        <v>998</v>
+        <v>997</v>
       </c>
       <c r="B309" s="14">
         <v>2024</v>
@@ -31426,7 +31426,7 @@
         <v>123</v>
       </c>
       <c r="G309" s="9" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="H309" s="9">
         <f t="shared" ref="H309" si="106">YEAR(G309)</f>
@@ -31455,7 +31455,7 @@
         <v>638</v>
       </c>
       <c r="P309" s="7" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
       <c r="Q309" s="9" t="s">
         <v>476</v>
@@ -31473,7 +31473,7 @@
     </row>
     <row r="310" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A310" s="7" t="s">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="B310" s="14">
         <v>2024</v>
@@ -31491,7 +31491,7 @@
         <v>368</v>
       </c>
       <c r="G310" s="9" t="s">
-        <v>1003</v>
+        <v>1002</v>
       </c>
       <c r="H310" s="9">
         <f t="shared" ref="H310" si="109">YEAR(G310)</f>
@@ -31520,10 +31520,10 @@
         <v>638</v>
       </c>
       <c r="P310" s="7" t="s">
-        <v>1004</v>
+        <v>1003</v>
       </c>
       <c r="Q310" s="9" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="R310" s="9" t="s">
         <v>153</v>
@@ -31538,7 +31538,7 @@
     </row>
     <row r="311" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A311" s="7" t="s">
-        <v>1007</v>
+        <v>1006</v>
       </c>
       <c r="B311" s="14">
         <v>2021</v>
@@ -31556,7 +31556,7 @@
         <v>323</v>
       </c>
       <c r="G311" s="9" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
       <c r="H311" s="9">
         <f t="shared" ref="H311" si="111">YEAR(G311)</f>
@@ -31585,7 +31585,7 @@
         <v>638</v>
       </c>
       <c r="P311" s="7" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
       <c r="Q311" s="9" t="s">
         <v>544</v>
@@ -31603,7 +31603,7 @@
     </row>
     <row r="312" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A312" s="7" t="s">
-        <v>1010</v>
+        <v>1009</v>
       </c>
       <c r="B312" s="14">
         <v>2022</v>
@@ -31621,7 +31621,7 @@
         <v>426</v>
       </c>
       <c r="G312" s="9" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
       <c r="H312" s="9">
         <f t="shared" ref="H312:H313" si="113">YEAR(G312)</f>
@@ -31650,7 +31650,7 @@
         <v>638</v>
       </c>
       <c r="P312" s="7" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
       <c r="Q312" s="9" t="s">
         <v>447</v>
@@ -31668,7 +31668,7 @@
     </row>
     <row r="313" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A313" s="7" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
       <c r="B313" s="14">
         <v>2024</v>
@@ -31686,7 +31686,7 @@
         <v>296</v>
       </c>
       <c r="G313" s="9" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
       <c r="H313" s="9">
         <f t="shared" si="113"/>
@@ -31715,7 +31715,7 @@
         <v>638</v>
       </c>
       <c r="P313" s="12" t="s">
-        <v>1015</v>
+        <v>1014</v>
       </c>
       <c r="Q313" s="9" t="s">
         <v>544</v>
@@ -31733,7 +31733,7 @@
     </row>
     <row r="314" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A314" s="7" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
       <c r="B314" s="14">
         <v>2022</v>
@@ -31751,7 +31751,7 @@
         <v>363</v>
       </c>
       <c r="G314" s="9" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
       <c r="H314" s="9">
         <f t="shared" ref="H314" si="115">YEAR(G314)</f>
@@ -31780,10 +31780,10 @@
         <v>638</v>
       </c>
       <c r="P314" s="7" t="s">
+        <v>1017</v>
+      </c>
+      <c r="Q314" s="9" t="s">
         <v>1018</v>
-      </c>
-      <c r="Q314" s="9" t="s">
-        <v>1019</v>
       </c>
       <c r="R314" s="9" t="s">
         <v>153</v>
@@ -31798,7 +31798,7 @@
     </row>
     <row r="315" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A315" s="7" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
       <c r="B315" s="14">
         <v>2023</v>
@@ -31816,7 +31816,7 @@
         <v>434</v>
       </c>
       <c r="G315" s="9" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
       <c r="H315" s="9">
         <f t="shared" ref="H315" si="117">YEAR(G315)</f>
@@ -31845,7 +31845,7 @@
         <v>638</v>
       </c>
       <c r="P315" s="12" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
       <c r="Q315" s="9" t="s">
         <v>447</v>
@@ -31863,7 +31863,7 @@
     </row>
     <row r="316" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A316" s="7" t="s">
-        <v>1022</v>
+        <v>1021</v>
       </c>
       <c r="B316" s="14">
         <v>2024</v>
@@ -31881,7 +31881,7 @@
         <v>490</v>
       </c>
       <c r="G316" s="9" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="H316" s="9">
         <f t="shared" ref="H316" si="119">YEAR(G316)</f>
@@ -31910,7 +31910,7 @@
         <v>638</v>
       </c>
       <c r="P316" s="12" t="s">
-        <v>1023</v>
+        <v>1022</v>
       </c>
       <c r="Q316" s="9" t="s">
         <v>447</v>
@@ -31928,7 +31928,7 @@
     </row>
     <row r="317" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A317" s="7" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
       <c r="B317" s="14">
         <v>2023</v>
@@ -31946,7 +31946,7 @@
         <v>195</v>
       </c>
       <c r="G317" s="9" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="H317" s="9">
         <f t="shared" ref="H317" si="121">YEAR(G317)</f>
@@ -31963,7 +31963,7 @@
         <v>153</v>
       </c>
       <c r="L317" s="9" t="s">
-        <v>1025</v>
+        <v>1024</v>
       </c>
       <c r="M317" s="14">
         <v>1</v>
@@ -31975,7 +31975,7 @@
         <v>638</v>
       </c>
       <c r="P317" s="7" t="s">
-        <v>1026</v>
+        <v>1025</v>
       </c>
       <c r="Q317" s="9" t="s">
         <v>846</v>
@@ -31993,7 +31993,7 @@
     </row>
     <row r="318" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A318" s="7" t="s">
-        <v>1027</v>
+        <v>1026</v>
       </c>
       <c r="B318" s="14">
         <v>2024</v>
@@ -32011,7 +32011,7 @@
         <v>280</v>
       </c>
       <c r="G318" s="9" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="H318" s="9">
         <f t="shared" ref="H318" si="123">YEAR(G318)</f>
@@ -32040,7 +32040,7 @@
         <v>638</v>
       </c>
       <c r="P318" s="7" t="s">
-        <v>1028</v>
+        <v>1027</v>
       </c>
       <c r="Q318" s="9" t="s">
         <v>846</v>
@@ -32058,7 +32058,7 @@
     </row>
     <row r="319" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A319" s="7" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="B319" s="14">
         <v>2023</v>
@@ -32076,7 +32076,7 @@
         <v>472</v>
       </c>
       <c r="G319" s="9" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="H319" s="9">
         <f t="shared" ref="H319" si="126">YEAR(G319)</f>
@@ -32105,7 +32105,7 @@
         <v>638</v>
       </c>
       <c r="P319" s="7" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="Q319" s="9" t="s">
         <v>846</v>
@@ -32123,7 +32123,7 @@
     </row>
     <row r="320" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A320" s="7" t="s">
-        <v>1032</v>
+        <v>1031</v>
       </c>
       <c r="B320" s="14">
         <v>2016</v>
@@ -32141,7 +32141,7 @@
         <v>68</v>
       </c>
       <c r="G320" s="9" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
       <c r="H320" s="9">
         <f t="shared" ref="H320:H321" si="128">YEAR(G320)</f>
@@ -32170,10 +32170,10 @@
         <v>638</v>
       </c>
       <c r="P320" s="12" t="s">
-        <v>1034</v>
+        <v>1033</v>
       </c>
       <c r="Q320" s="9" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="R320" s="9" t="s">
         <v>153</v>
@@ -32188,7 +32188,7 @@
     </row>
     <row r="321" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A321" s="7" t="s">
-        <v>1035</v>
+        <v>1034</v>
       </c>
       <c r="B321" s="14">
         <v>2023</v>
@@ -32206,7 +32206,7 @@
         <v>512</v>
       </c>
       <c r="G321" s="9" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
       <c r="H321" s="9">
         <f t="shared" si="128"/>
@@ -32235,7 +32235,7 @@
         <v>638</v>
       </c>
       <c r="P321" s="7" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
       <c r="Q321" s="9" t="s">
         <v>544</v>
@@ -32253,7 +32253,7 @@
     </row>
     <row r="322" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A322" s="7" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="B322" s="14">
         <v>2024</v>
@@ -32271,7 +32271,7 @@
         <v>442</v>
       </c>
       <c r="G322" s="9" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
       <c r="H322" s="9">
         <f t="shared" ref="H322" si="130">YEAR(G322)</f>
@@ -32300,7 +32300,7 @@
         <v>638</v>
       </c>
       <c r="P322" s="7" t="s">
-        <v>1039</v>
+        <v>1038</v>
       </c>
       <c r="Q322" s="9" t="s">
         <v>544</v>
@@ -32318,7 +32318,7 @@
     </row>
     <row r="323" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A323" s="7" t="s">
-        <v>1040</v>
+        <v>1039</v>
       </c>
       <c r="B323" s="14">
         <v>2024</v>
@@ -32336,7 +32336,7 @@
         <v>265</v>
       </c>
       <c r="G323" s="9" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
       <c r="H323" s="9">
         <f t="shared" ref="H323" si="132">YEAR(G323)</f>
@@ -32365,7 +32365,7 @@
         <v>638</v>
       </c>
       <c r="P323" s="7" t="s">
-        <v>1041</v>
+        <v>1040</v>
       </c>
       <c r="Q323" s="9" t="s">
         <v>544</v>
@@ -32383,7 +32383,7 @@
     </row>
     <row r="324" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A324" s="7" t="s">
-        <v>1042</v>
+        <v>1041</v>
       </c>
       <c r="B324" s="14">
         <v>2024</v>
@@ -32401,7 +32401,7 @@
         <v>333</v>
       </c>
       <c r="G324" s="9" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
       <c r="H324" s="9">
         <f t="shared" ref="H324" si="134">YEAR(G324)</f>
@@ -32418,7 +32418,7 @@
         <v>153</v>
       </c>
       <c r="L324" s="9" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
       <c r="M324" s="14">
         <v>1</v>
@@ -32430,7 +32430,7 @@
         <v>638</v>
       </c>
       <c r="P324" s="7" t="s">
-        <v>1044</v>
+        <v>1043</v>
       </c>
       <c r="Q324" s="9" t="s">
         <v>544</v>
@@ -32448,7 +32448,7 @@
     </row>
     <row r="325" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A325" s="7" t="s">
-        <v>1045</v>
+        <v>1044</v>
       </c>
       <c r="B325" s="14">
         <v>2024</v>
@@ -32466,7 +32466,7 @@
         <v>386</v>
       </c>
       <c r="G325" s="9" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
       <c r="H325" s="9">
         <f t="shared" ref="H325" si="136">YEAR(G325)</f>
@@ -32495,7 +32495,7 @@
         <v>638</v>
       </c>
       <c r="P325" s="7" t="s">
-        <v>1046</v>
+        <v>1045</v>
       </c>
       <c r="Q325" s="9" t="s">
         <v>544</v>
@@ -32513,7 +32513,7 @@
     </row>
     <row r="326" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A326" s="7" t="s">
-        <v>1047</v>
+        <v>1046</v>
       </c>
       <c r="B326" s="14">
         <v>2020</v>
@@ -32531,7 +32531,7 @@
         <v>213</v>
       </c>
       <c r="G326" s="9" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
       <c r="H326" s="9">
         <f t="shared" ref="H326" si="138">YEAR(G326)</f>
@@ -32560,7 +32560,7 @@
         <v>638</v>
       </c>
       <c r="P326" s="12" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="Q326" s="9" t="s">
         <v>544</v>
@@ -32578,7 +32578,7 @@
     </row>
     <row r="327" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A327" s="7" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
       <c r="B327" s="14">
         <v>2024</v>
@@ -32596,7 +32596,7 @@
         <v>277</v>
       </c>
       <c r="G327" s="9" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
       <c r="H327" s="9">
         <f t="shared" ref="H327" si="140">YEAR(G327)</f>
@@ -32625,7 +32625,7 @@
         <v>638</v>
       </c>
       <c r="P327" s="7" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
       <c r="Q327" s="9" t="s">
         <v>447</v>
@@ -32643,7 +32643,7 @@
     </row>
     <row r="328" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A328" s="7" t="s">
-        <v>1051</v>
+        <v>1050</v>
       </c>
       <c r="B328" s="14">
         <v>2024</v>
@@ -32661,7 +32661,7 @@
         <v>132</v>
       </c>
       <c r="G328" s="9" t="s">
-        <v>1052</v>
+        <v>1051</v>
       </c>
       <c r="H328" s="9">
         <f t="shared" ref="H328" si="142">YEAR(G328)</f>
@@ -32690,7 +32690,7 @@
         <v>638</v>
       </c>
       <c r="P328" s="12" t="s">
-        <v>1053</v>
+        <v>1052</v>
       </c>
       <c r="Q328" s="9" t="s">
         <v>447</v>
@@ -32708,7 +32708,7 @@
     </row>
     <row r="329" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A329" s="7" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
       <c r="B329" s="14">
         <v>2023</v>
@@ -32726,7 +32726,7 @@
         <v>289</v>
       </c>
       <c r="G329" s="9" t="s">
-        <v>1052</v>
+        <v>1051</v>
       </c>
       <c r="H329" s="9">
         <f t="shared" ref="H329" si="144">YEAR(G329)</f>
@@ -32755,7 +32755,7 @@
         <v>638</v>
       </c>
       <c r="P329" s="7" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="Q329" s="9" t="s">
         <v>447</v>
@@ -32773,7 +32773,7 @@
     </row>
     <row r="330" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A330" s="7" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
       <c r="B330" s="14">
         <v>2024</v>
@@ -32791,7 +32791,7 @@
         <v>257</v>
       </c>
       <c r="G330" s="9" t="s">
-        <v>1052</v>
+        <v>1051</v>
       </c>
       <c r="H330" s="9">
         <f t="shared" ref="H330" si="146">YEAR(G330)</f>
@@ -32820,7 +32820,7 @@
         <v>638</v>
       </c>
       <c r="P330" s="7" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="Q330" s="9" t="s">
         <v>846</v>
@@ -32838,7 +32838,7 @@
     </row>
     <row r="331" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A331" s="7" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="B331" s="14">
         <v>2023</v>
@@ -32856,7 +32856,7 @@
         <v>573</v>
       </c>
       <c r="G331" s="9" t="s">
-        <v>1059</v>
+        <v>1058</v>
       </c>
       <c r="H331" s="9">
         <f t="shared" ref="H331" si="148">YEAR(G331)</f>
@@ -32885,7 +32885,7 @@
         <v>638</v>
       </c>
       <c r="P331" s="7" t="s">
-        <v>1060</v>
+        <v>1059</v>
       </c>
       <c r="Q331" s="9" t="s">
         <v>846</v>
@@ -32903,7 +32903,7 @@
     </row>
     <row r="332" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A332" s="7" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
       <c r="B332" s="14">
         <v>2009</v>
@@ -32921,7 +32921,7 @@
         <v>220</v>
       </c>
       <c r="G332" s="9" t="s">
-        <v>1059</v>
+        <v>1058</v>
       </c>
       <c r="H332" s="9">
         <f t="shared" ref="H332:H333" si="150">YEAR(G332)</f>
@@ -32953,7 +32953,7 @@
         <v>648</v>
       </c>
       <c r="Q332" s="9" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
       <c r="R332" s="9" t="s">
         <v>153</v>
@@ -32968,7 +32968,7 @@
     </row>
     <row r="333" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A333" s="7" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="B333" s="14">
         <v>2024</v>
@@ -32986,7 +32986,7 @@
         <v>314</v>
       </c>
       <c r="G333" s="9" t="s">
-        <v>1064</v>
+        <v>1063</v>
       </c>
       <c r="H333" s="9">
         <f t="shared" si="150"/>
@@ -33015,10 +33015,10 @@
         <v>638</v>
       </c>
       <c r="P333" s="7" t="s">
-        <v>1063</v>
+        <v>1062</v>
       </c>
       <c r="Q333" s="9" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
       <c r="R333" s="9" t="s">
         <v>153</v>
@@ -33033,7 +33033,7 @@
     </row>
     <row r="334" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A334" s="7" t="s">
-        <v>1065</v>
+        <v>1064</v>
       </c>
       <c r="B334" s="14">
         <v>2025</v>
@@ -33051,7 +33051,7 @@
         <v>308</v>
       </c>
       <c r="G334" s="9" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="H334" s="9">
         <f t="shared" ref="H334:H335" si="152">YEAR(G334)</f>
@@ -33080,10 +33080,10 @@
         <v>638</v>
       </c>
       <c r="P334" s="7" t="s">
-        <v>1067</v>
+        <v>1066</v>
       </c>
       <c r="Q334" s="9" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
       <c r="R334" s="9" t="s">
         <v>153</v>
@@ -33098,7 +33098,7 @@
     </row>
     <row r="335" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A335" s="7" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="B335" s="14">
         <v>2024</v>
@@ -33116,7 +33116,7 @@
         <v>382</v>
       </c>
       <c r="G335" s="9" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="H335" s="9">
         <f t="shared" si="152"/>
@@ -33145,10 +33145,10 @@
         <v>638</v>
       </c>
       <c r="P335" s="12" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="Q335" s="9" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
       <c r="R335" s="9" t="s">
         <v>153</v>
@@ -33163,7 +33163,7 @@
     </row>
     <row r="336" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A336" s="7" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
       <c r="B336" s="14">
         <v>2023</v>
@@ -33181,7 +33181,7 @@
         <v>469</v>
       </c>
       <c r="G336" s="9" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="H336" s="9">
         <f t="shared" ref="H336" si="154">YEAR(G336)</f>
@@ -33210,7 +33210,7 @@
         <v>638</v>
       </c>
       <c r="P336" s="12" t="s">
-        <v>1072</v>
+        <v>1071</v>
       </c>
       <c r="Q336" s="9" t="s">
         <v>447</v>
@@ -33228,7 +33228,7 @@
     </row>
     <row r="337" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A337" s="7" t="s">
-        <v>1073</v>
+        <v>1072</v>
       </c>
       <c r="B337" s="14">
         <v>2012</v>
@@ -33246,7 +33246,7 @@
         <v>135</v>
       </c>
       <c r="G337" s="9" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
       <c r="H337" s="9">
         <f t="shared" ref="H337" si="156">YEAR(G337)</f>
@@ -33275,7 +33275,7 @@
         <v>638</v>
       </c>
       <c r="P337" s="7" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
       <c r="Q337" s="9" t="s">
         <v>447</v>
@@ -33293,7 +33293,7 @@
     </row>
     <row r="338" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A338" s="7" t="s">
-        <v>1076</v>
+        <v>1075</v>
       </c>
       <c r="B338" s="14">
         <v>2024</v>
@@ -33311,7 +33311,7 @@
         <v>373</v>
       </c>
       <c r="G338" s="9" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
       <c r="H338" s="9">
         <f t="shared" ref="H338:H339" si="158">YEAR(G338)</f>
@@ -33340,10 +33340,10 @@
         <v>638</v>
       </c>
       <c r="P338" s="12" t="s">
-        <v>1078</v>
+        <v>1077</v>
       </c>
       <c r="Q338" s="9" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
       <c r="R338" s="9" t="s">
         <v>153</v>
@@ -33358,7 +33358,7 @@
     </row>
     <row r="339" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A339" s="7" t="s">
-        <v>1079</v>
+        <v>1078</v>
       </c>
       <c r="B339" s="14">
         <v>2024</v>
@@ -33376,7 +33376,7 @@
         <v>286</v>
       </c>
       <c r="G339" s="9" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
       <c r="H339" s="9">
         <f t="shared" si="158"/>
@@ -33405,7 +33405,7 @@
         <v>638</v>
       </c>
       <c r="P339" s="7" t="s">
-        <v>1081</v>
+        <v>1080</v>
       </c>
       <c r="Q339" s="9" t="s">
         <v>447</v>
@@ -33423,7 +33423,7 @@
     </row>
     <row r="340" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A340" s="7" t="s">
-        <v>1082</v>
+        <v>1081</v>
       </c>
       <c r="B340" s="14">
         <v>2024</v>
@@ -33441,7 +33441,7 @@
         <v>418</v>
       </c>
       <c r="G340" s="9" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
       <c r="H340" s="9">
         <f t="shared" ref="H340" si="160">YEAR(G340)</f>
@@ -33458,7 +33458,7 @@
         <v>153</v>
       </c>
       <c r="L340" s="9" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="M340" s="14">
         <v>2</v>
@@ -33470,7 +33470,7 @@
         <v>638</v>
       </c>
       <c r="P340" s="7" t="s">
-        <v>1081</v>
+        <v>1080</v>
       </c>
       <c r="Q340" s="9" t="s">
         <v>447</v>
@@ -33488,7 +33488,7 @@
     </row>
     <row r="341" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A341" s="7" t="s">
-        <v>1084</v>
+        <v>1083</v>
       </c>
       <c r="B341" s="14">
         <v>2024</v>
@@ -33506,7 +33506,7 @@
         <v>611</v>
       </c>
       <c r="G341" s="9" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
       <c r="H341" s="9">
         <f t="shared" ref="H341" si="161">YEAR(G341)</f>
@@ -33523,7 +33523,7 @@
         <v>153</v>
       </c>
       <c r="L341" s="9" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="M341" s="14">
         <v>2</v>
@@ -33535,7 +33535,7 @@
         <v>638</v>
       </c>
       <c r="P341" s="7" t="s">
-        <v>1085</v>
+        <v>1084</v>
       </c>
       <c r="Q341" s="9" t="s">
         <v>447</v>
@@ -33553,7 +33553,7 @@
     </row>
     <row r="342" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A342" s="7" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="B342" s="14">
         <v>2024</v>
@@ -33571,7 +33571,7 @@
         <v>55</v>
       </c>
       <c r="G342" s="9" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
       <c r="H342" s="9">
         <f t="shared" ref="H342" si="162">YEAR(G342)</f>
@@ -33600,10 +33600,10 @@
         <v>638</v>
       </c>
       <c r="P342" s="7" t="s">
-        <v>1087</v>
+        <v>1086</v>
       </c>
       <c r="Q342" s="9" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="R342" s="9" t="s">
         <v>153</v>
@@ -33618,7 +33618,7 @@
     </row>
     <row r="343" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A343" s="7" t="s">
-        <v>1088</v>
+        <v>1087</v>
       </c>
       <c r="B343" s="14">
         <v>2020</v>
@@ -33636,7 +33636,7 @@
         <v>602</v>
       </c>
       <c r="G343" s="9" t="s">
-        <v>1089</v>
+        <v>1088</v>
       </c>
       <c r="H343" s="9">
         <f t="shared" ref="H343" si="163">YEAR(G343)</f>
@@ -33665,7 +33665,7 @@
         <v>638</v>
       </c>
       <c r="P343" s="7" t="s">
-        <v>1090</v>
+        <v>1089</v>
       </c>
       <c r="Q343" s="9" t="s">
         <v>447</v>
@@ -33683,7 +33683,7 @@
     </row>
     <row r="344" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A344" s="7" t="s">
-        <v>1091</v>
+        <v>1090</v>
       </c>
       <c r="B344" s="14">
         <v>2009</v>
@@ -33701,7 +33701,7 @@
         <v>388</v>
       </c>
       <c r="G344" s="9" t="s">
-        <v>1089</v>
+        <v>1088</v>
       </c>
       <c r="H344" s="9">
         <f t="shared" ref="H344" si="164">YEAR(G344)</f>
@@ -33730,7 +33730,7 @@
         <v>638</v>
       </c>
       <c r="P344" s="7" t="s">
-        <v>1092</v>
+        <v>1091</v>
       </c>
       <c r="Q344" s="9" t="s">
         <v>447</v>
@@ -33748,7 +33748,7 @@
     </row>
     <row r="345" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A345" s="7" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
       <c r="B345" s="14">
         <v>2023</v>
@@ -33766,7 +33766,7 @@
         <v>63</v>
       </c>
       <c r="G345" s="9" t="s">
-        <v>1094</v>
+        <v>1093</v>
       </c>
       <c r="H345" s="9">
         <f t="shared" ref="H345" si="165">YEAR(G345)</f>
@@ -33795,10 +33795,10 @@
         <v>638</v>
       </c>
       <c r="P345" s="7" t="s">
-        <v>1095</v>
+        <v>1094</v>
       </c>
       <c r="Q345" s="9" t="s">
-        <v>847</v>
+        <v>1197</v>
       </c>
       <c r="R345" s="9" t="s">
         <v>153</v>
@@ -33813,7 +33813,7 @@
     </row>
     <row r="346" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A346" s="7" t="s">
-        <v>1096</v>
+        <v>1095</v>
       </c>
       <c r="B346" s="14">
         <v>2024</v>
@@ -33831,7 +33831,7 @@
         <v>350</v>
       </c>
       <c r="G346" s="9" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="H346" s="9">
         <f t="shared" ref="H346" si="167">YEAR(G346)</f>
@@ -33860,7 +33860,7 @@
         <v>638</v>
       </c>
       <c r="P346" s="12" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
       <c r="Q346" s="9" t="s">
         <v>544</v>
@@ -33878,7 +33878,7 @@
     </row>
     <row r="347" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A347" s="7" t="s">
-        <v>1099</v>
+        <v>1098</v>
       </c>
       <c r="B347" s="14">
         <v>2018</v>
@@ -33896,7 +33896,7 @@
         <v>331</v>
       </c>
       <c r="G347" s="9" t="s">
-        <v>1100</v>
+        <v>1099</v>
       </c>
       <c r="H347" s="9">
         <f t="shared" ref="H347" si="169">YEAR(G347)</f>
@@ -33925,10 +33925,10 @@
         <v>638</v>
       </c>
       <c r="P347" s="12" t="s">
-        <v>1101</v>
+        <v>1100</v>
       </c>
       <c r="Q347" s="9" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
       <c r="R347" s="9" t="s">
         <v>153</v>
@@ -33943,7 +33943,7 @@
     </row>
     <row r="348" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A348" s="7" t="s">
-        <v>1102</v>
+        <v>1101</v>
       </c>
       <c r="B348" s="14">
         <v>2025</v>
@@ -33961,7 +33961,7 @@
         <v>433</v>
       </c>
       <c r="G348" s="9" t="s">
-        <v>1103</v>
+        <v>1102</v>
       </c>
       <c r="H348" s="9">
         <f t="shared" ref="H348" si="171">YEAR(G348)</f>
@@ -33978,7 +33978,7 @@
         <v>153</v>
       </c>
       <c r="L348" s="9" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="M348" s="14">
         <v>2</v>
@@ -33990,7 +33990,7 @@
         <v>638</v>
       </c>
       <c r="P348" s="12" t="s">
-        <v>1104</v>
+        <v>1103</v>
       </c>
       <c r="Q348" s="9" t="s">
         <v>447</v>
@@ -34008,7 +34008,7 @@
     </row>
     <row r="349" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A349" s="7" t="s">
-        <v>1105</v>
+        <v>1104</v>
       </c>
       <c r="B349" s="14">
         <v>2023</v>
@@ -34026,7 +34026,7 @@
         <v>168</v>
       </c>
       <c r="G349" s="9" t="s">
-        <v>1103</v>
+        <v>1102</v>
       </c>
       <c r="H349" s="9">
         <f t="shared" ref="H349" si="173">YEAR(G349)</f>
@@ -34055,10 +34055,10 @@
         <v>638</v>
       </c>
       <c r="P349" s="7" t="s">
-        <v>1106</v>
+        <v>1105</v>
       </c>
       <c r="Q349" s="9" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
       <c r="R349" s="9" t="s">
         <v>153</v>
@@ -34073,7 +34073,7 @@
     </row>
     <row r="350" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A350" s="7" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="B350" s="14">
         <v>2025</v>
@@ -34091,7 +34091,7 @@
         <v>345</v>
       </c>
       <c r="G350" s="9" t="s">
-        <v>1108</v>
+        <v>1107</v>
       </c>
       <c r="H350" s="9">
         <f t="shared" ref="H350" si="175">YEAR(G350)</f>
@@ -34108,7 +34108,7 @@
         <v>153</v>
       </c>
       <c r="L350" s="9" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="M350" s="14">
         <v>2</v>
@@ -34120,10 +34120,10 @@
         <v>638</v>
       </c>
       <c r="P350" s="7" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="Q350" s="9" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
       <c r="R350" s="9" t="s">
         <v>153</v>
@@ -34138,7 +34138,7 @@
     </row>
     <row r="351" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A351" s="7" t="s">
-        <v>1110</v>
+        <v>1109</v>
       </c>
       <c r="B351" s="14">
         <v>2024</v>
@@ -34156,7 +34156,7 @@
         <v>59</v>
       </c>
       <c r="G351" s="9" t="s">
-        <v>1111</v>
+        <v>1110</v>
       </c>
       <c r="H351" s="9">
         <f t="shared" ref="H351" si="177">YEAR(G351)</f>
@@ -34185,10 +34185,10 @@
         <v>638</v>
       </c>
       <c r="P351" s="7" t="s">
-        <v>1112</v>
+        <v>1111</v>
       </c>
       <c r="Q351" s="9" t="s">
-        <v>847</v>
+        <v>1197</v>
       </c>
       <c r="R351" s="9" t="s">
         <v>153</v>
@@ -34203,7 +34203,7 @@
     </row>
     <row r="352" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A352" s="7" t="s">
-        <v>1113</v>
+        <v>1112</v>
       </c>
       <c r="B352" s="14">
         <v>2025</v>
@@ -34221,7 +34221,7 @@
         <v>160</v>
       </c>
       <c r="G352" s="9" t="s">
-        <v>1111</v>
+        <v>1110</v>
       </c>
       <c r="H352" s="9">
         <f t="shared" ref="H352" si="179">YEAR(G352)</f>
@@ -34238,7 +34238,7 @@
         <v>153</v>
       </c>
       <c r="L352" s="9" t="s">
-        <v>1114</v>
+        <v>1113</v>
       </c>
       <c r="M352" s="14">
         <v>3</v>
@@ -34250,10 +34250,10 @@
         <v>638</v>
       </c>
       <c r="P352" s="7" t="s">
-        <v>1115</v>
+        <v>1114</v>
       </c>
       <c r="Q352" s="9" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="R352" s="9" t="s">
         <v>153</v>
@@ -34268,7 +34268,7 @@
     </row>
     <row r="353" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A353" s="7" t="s">
-        <v>1116</v>
+        <v>1115</v>
       </c>
       <c r="B353" s="14">
         <v>2020</v>
@@ -34286,7 +34286,7 @@
         <v>321</v>
       </c>
       <c r="G353" s="9" t="s">
-        <v>1117</v>
+        <v>1116</v>
       </c>
       <c r="H353" s="9">
         <f t="shared" ref="H353" si="181">YEAR(G353)</f>
@@ -34315,10 +34315,10 @@
         <v>638</v>
       </c>
       <c r="P353" s="7" t="s">
-        <v>1118</v>
+        <v>1117</v>
       </c>
       <c r="Q353" s="9" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="R353" s="9" t="s">
         <v>153</v>
@@ -34333,7 +34333,7 @@
     </row>
     <row r="354" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A354" s="7" t="s">
-        <v>1119</v>
+        <v>1118</v>
       </c>
       <c r="B354" s="14">
         <v>2025</v>
@@ -34351,7 +34351,7 @@
         <v>123</v>
       </c>
       <c r="G354" s="9" t="s">
-        <v>1120</v>
+        <v>1119</v>
       </c>
       <c r="H354" s="9">
         <f t="shared" ref="H354" si="183">YEAR(G354)</f>
@@ -34380,7 +34380,7 @@
         <v>638</v>
       </c>
       <c r="P354" s="7" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
       <c r="Q354" s="9" t="s">
         <v>476</v>
@@ -34398,7 +34398,7 @@
     </row>
     <row r="355" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A355" s="7" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
       <c r="B355" s="14">
         <v>2020</v>
@@ -34416,7 +34416,7 @@
         <v>131</v>
       </c>
       <c r="G355" s="9" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
       <c r="H355" s="9">
         <f t="shared" ref="H355" si="185">YEAR(G355)</f>
@@ -34448,7 +34448,7 @@
         <v>648</v>
       </c>
       <c r="Q355" s="9" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="R355" s="9" t="s">
         <v>153</v>
@@ -34463,7 +34463,7 @@
     </row>
     <row r="356" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A356" s="7" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
       <c r="B356" s="14">
         <v>2025</v>
@@ -34481,7 +34481,7 @@
         <v>485</v>
       </c>
       <c r="G356" s="9" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
       <c r="H356" s="9">
         <f t="shared" ref="H356" si="187">YEAR(G356)</f>
@@ -34510,10 +34510,10 @@
         <v>638</v>
       </c>
       <c r="P356" s="7" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
       <c r="Q356" s="9" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="R356" s="9" t="s">
         <v>153</v>
@@ -34528,7 +34528,7 @@
     </row>
     <row r="357" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A357" s="7" t="s">
-        <v>1125</v>
+        <v>1124</v>
       </c>
       <c r="B357" s="14">
         <v>2024</v>
@@ -34546,7 +34546,7 @@
         <v>569</v>
       </c>
       <c r="G357" s="9" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
       <c r="H357" s="9">
         <f t="shared" ref="H357" si="189">YEAR(G357)</f>
@@ -34575,10 +34575,10 @@
         <v>638</v>
       </c>
       <c r="P357" s="7" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
       <c r="Q357" s="9" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="R357" s="9" t="s">
         <v>153</v>
@@ -34593,7 +34593,7 @@
     </row>
     <row r="358" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A358" s="7" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
       <c r="B358" s="14">
         <v>2024</v>
@@ -34611,7 +34611,7 @@
         <v>236</v>
       </c>
       <c r="G358" s="9" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
       <c r="H358" s="9">
         <f t="shared" ref="H358" si="191">YEAR(G358)</f>
@@ -34640,10 +34640,10 @@
         <v>638</v>
       </c>
       <c r="P358" s="12" t="s">
-        <v>1131</v>
+        <v>1130</v>
       </c>
       <c r="Q358" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R358" s="9" t="s">
         <v>153</v>
@@ -34658,7 +34658,7 @@
     </row>
     <row r="359" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A359" s="7" t="s">
-        <v>1132</v>
+        <v>1131</v>
       </c>
       <c r="B359" s="14">
         <v>2024</v>
@@ -34676,7 +34676,7 @@
         <v>265</v>
       </c>
       <c r="G359" s="9" t="s">
-        <v>1133</v>
+        <v>1132</v>
       </c>
       <c r="H359" s="9">
         <f t="shared" ref="H359:H360" si="193">YEAR(G359)</f>
@@ -34705,10 +34705,10 @@
         <v>638</v>
       </c>
       <c r="P359" s="12" t="s">
-        <v>1134</v>
+        <v>1133</v>
       </c>
       <c r="Q359" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R359" s="9" t="s">
         <v>153</v>
@@ -34723,7 +34723,7 @@
     </row>
     <row r="360" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A360" s="7" t="s">
-        <v>1135</v>
+        <v>1134</v>
       </c>
       <c r="B360" s="14">
         <v>2025</v>
@@ -34741,7 +34741,7 @@
         <v>362</v>
       </c>
       <c r="G360" s="9" t="s">
-        <v>1136</v>
+        <v>1135</v>
       </c>
       <c r="H360" s="9">
         <f t="shared" si="193"/>
@@ -34770,7 +34770,7 @@
         <v>638</v>
       </c>
       <c r="P360" s="7" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="Q360" s="9" t="s">
         <v>544</v>
@@ -34788,7 +34788,7 @@
     </row>
     <row r="361" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A361" s="7" t="s">
-        <v>1172</v>
+        <v>1171</v>
       </c>
       <c r="B361" s="14">
         <v>2013</v>
@@ -34806,7 +34806,7 @@
         <v>135</v>
       </c>
       <c r="G361" s="9" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="H361" s="9">
         <f t="shared" ref="H361" si="195">YEAR(G361)</f>
@@ -34835,10 +34835,10 @@
         <v>638</v>
       </c>
       <c r="P361" s="7" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="Q361" s="9" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
       <c r="R361" s="9" t="s">
         <v>153</v>
@@ -34853,7 +34853,7 @@
     </row>
     <row r="362" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A362" s="7" t="s">
-        <v>1175</v>
+        <v>1174</v>
       </c>
       <c r="B362" s="14">
         <v>2015</v>
@@ -34871,7 +34871,7 @@
         <v>464</v>
       </c>
       <c r="G362" s="9" t="s">
-        <v>1176</v>
+        <v>1175</v>
       </c>
       <c r="H362" s="9">
         <f t="shared" ref="H362" si="197">YEAR(G362)</f>
@@ -34900,10 +34900,10 @@
         <v>638</v>
       </c>
       <c r="P362" s="7" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="Q362" s="9" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
       <c r="R362" s="9" t="s">
         <v>153</v>
@@ -34918,7 +34918,7 @@
     </row>
     <row r="363" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A363" s="7" t="s">
-        <v>1178</v>
+        <v>1177</v>
       </c>
       <c r="B363" s="14">
         <v>2013</v>
@@ -34936,7 +34936,7 @@
         <v>369</v>
       </c>
       <c r="G363" s="9" t="s">
-        <v>1180</v>
+        <v>1179</v>
       </c>
       <c r="H363" s="9">
         <f t="shared" ref="H363" si="199">YEAR(G363)</f>
@@ -34953,7 +34953,7 @@
         <v>153</v>
       </c>
       <c r="L363" s="9" t="s">
-        <v>1179</v>
+        <v>1178</v>
       </c>
       <c r="M363" s="14">
         <v>2</v>
@@ -34965,10 +34965,10 @@
         <v>638</v>
       </c>
       <c r="P363" s="7" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
       <c r="Q363" s="9" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
       <c r="R363" s="9" t="s">
         <v>153</v>
@@ -34983,7 +34983,7 @@
     </row>
     <row r="364" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A364" s="7" t="s">
-        <v>1182</v>
+        <v>1181</v>
       </c>
       <c r="B364" s="14">
         <v>2025</v>
@@ -35001,7 +35001,7 @@
         <v>78</v>
       </c>
       <c r="G364" s="9" t="s">
-        <v>1180</v>
+        <v>1179</v>
       </c>
       <c r="H364" s="9">
         <f t="shared" ref="H364" si="201">YEAR(G364)</f>
@@ -35030,10 +35030,10 @@
         <v>638</v>
       </c>
       <c r="P364" s="38" t="s">
-        <v>1183</v>
+        <v>1182</v>
       </c>
       <c r="Q364" s="9" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
       <c r="R364" s="9" t="s">
         <v>153</v>
@@ -35048,7 +35048,7 @@
     </row>
     <row r="365" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A365" s="7" t="s">
-        <v>1184</v>
+        <v>1183</v>
       </c>
       <c r="B365" s="14">
         <v>2025</v>
@@ -35066,7 +35066,7 @@
         <v>43</v>
       </c>
       <c r="G365" s="9" t="s">
-        <v>1185</v>
+        <v>1184</v>
       </c>
       <c r="H365" s="9">
         <f t="shared" ref="H365" si="202">YEAR(G365)</f>
@@ -35095,10 +35095,10 @@
         <v>638</v>
       </c>
       <c r="P365" s="7" t="s">
-        <v>1186</v>
+        <v>1185</v>
       </c>
       <c r="Q365" s="9" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="R365" s="9" t="s">
         <v>153</v>
@@ -35113,7 +35113,7 @@
     </row>
     <row r="366" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A366" s="7" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
       <c r="B366" s="41">
         <v>2022</v>
@@ -35131,7 +35131,7 @@
         <v>236</v>
       </c>
       <c r="G366" s="9" t="s">
-        <v>1185</v>
+        <v>1184</v>
       </c>
       <c r="H366" s="9">
         <f t="shared" ref="H366" si="204">YEAR(G366)</f>
@@ -35160,7 +35160,7 @@
         <v>638</v>
       </c>
       <c r="P366" s="7" t="s">
-        <v>1188</v>
+        <v>1187</v>
       </c>
       <c r="Q366" s="9" t="s">
         <v>846</v>
@@ -35178,7 +35178,7 @@
     </row>
     <row r="367" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A367" s="7" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="B367" s="41">
         <v>2024</v>
@@ -35196,7 +35196,7 @@
         <v>445</v>
       </c>
       <c r="G367" s="9" t="s">
-        <v>1185</v>
+        <v>1184</v>
       </c>
       <c r="H367" s="9">
         <f t="shared" ref="H367" si="206">YEAR(G367)</f>
@@ -35225,10 +35225,10 @@
         <v>638</v>
       </c>
       <c r="P367" s="7" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
       <c r="Q367" s="9" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="R367" s="9" t="s">
         <v>153</v>
@@ -35243,7 +35243,7 @@
     </row>
     <row r="368" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A368" s="7" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
       <c r="B368" s="41">
         <v>2025</v>
@@ -35261,7 +35261,7 @@
         <v>82</v>
       </c>
       <c r="G368" s="9" t="s">
-        <v>1192</v>
+        <v>1191</v>
       </c>
       <c r="H368" s="9">
         <f t="shared" ref="H368" si="208">YEAR(G368)</f>
@@ -35290,10 +35290,10 @@
         <v>638</v>
       </c>
       <c r="P368" s="7" t="s">
-        <v>1193</v>
+        <v>1192</v>
       </c>
       <c r="Q368" s="9" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="R368" s="9" t="s">
         <v>153</v>
@@ -35308,7 +35308,7 @@
     </row>
     <row r="369" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A369" s="7" t="s">
-        <v>1194</v>
+        <v>1193</v>
       </c>
       <c r="B369" s="41">
         <v>2025</v>
@@ -35326,7 +35326,7 @@
         <v>368</v>
       </c>
       <c r="G369" s="9" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
       <c r="H369" s="9">
         <f t="shared" ref="H369" si="210">YEAR(G369)</f>
@@ -35355,10 +35355,10 @@
         <v>638</v>
       </c>
       <c r="P369" s="7" t="s">
-        <v>1196</v>
+        <v>1195</v>
       </c>
       <c r="Q369" s="9" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="R369" s="9" t="s">
         <v>153</v>

</xml_diff>

<commit_message>
#47 Reading List: updated to 2025-11-30 (Linux books).
</commit_message>
<xml_diff>
--- a/data/Reading List.xlsx
+++ b/data/Reading List.xlsx
@@ -23928,7 +23928,7 @@
         <v>186</v>
       </c>
       <c r="T193" s="10">
-        <v>894</v>
+        <v>874</v>
       </c>
     </row>
     <row r="194" spans="1:20" x14ac:dyDescent="0.2">
@@ -31403,7 +31403,7 @@
         <v>218</v>
       </c>
       <c r="T308" s="10">
-        <v>499</v>
+        <v>496</v>
       </c>
     </row>
     <row r="309" spans="1:20" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
#47 Reading List: updated to 2025-12-02 (mix updates).
</commit_message>
<xml_diff>
--- a/data/Reading List.xlsx
+++ b/data/Reading List.xlsx
@@ -21188,7 +21188,7 @@
         <v>647</v>
       </c>
       <c r="Q151" s="9" t="s">
-        <v>446</v>
+        <v>1163</v>
       </c>
       <c r="R151" s="9" t="s">
         <v>153</v>
@@ -21198,7 +21198,7 @@
         <v>16</v>
       </c>
       <c r="T151" s="10">
-        <v>475</v>
+        <v>478</v>
       </c>
     </row>
     <row r="152" spans="1:20" x14ac:dyDescent="0.2">
@@ -23333,7 +23333,7 @@
         <v>647</v>
       </c>
       <c r="Q184" s="9" t="s">
-        <v>1163</v>
+        <v>844</v>
       </c>
       <c r="R184" s="9" t="s">
         <v>153</v>
@@ -23343,7 +23343,7 @@
         <v>16</v>
       </c>
       <c r="T184" s="10">
-        <v>717</v>
+        <v>716</v>
       </c>
     </row>
     <row r="185" spans="1:20" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
#47 Reading List: updated to 2025-12-04 (UML -> nwkbsoftwareengineering).
</commit_message>
<xml_diff>
--- a/data/Reading List.xlsx
+++ b/data/Reading List.xlsx
@@ -3637,13 +3637,13 @@
     <t>Useful. Very good introductive book about experience marketing.</t>
   </si>
   <si>
-    <t>Unsorted</t>
-  </si>
-  <si>
     <t xml:space="preserve">Make: Electronics (2nd Edition) </t>
   </si>
   <si>
     <t>Maker Media Inc.</t>
+  </si>
+  <si>
+    <t>Uncategorized</t>
   </si>
 </sst>
 </file>
@@ -12361,7 +12361,7 @@
         <v>1196</v>
       </c>
       <c r="Q15" s="9" t="s">
-        <v>1197</v>
+        <v>1199</v>
       </c>
       <c r="R15" s="9" t="s">
         <v>153</v>
@@ -12761,7 +12761,7 @@
         <v>91</v>
       </c>
       <c r="T21" s="10">
-        <v>455</v>
+        <v>522</v>
       </c>
     </row>
     <row r="22" spans="1:20" x14ac:dyDescent="0.2">
@@ -14376,7 +14376,7 @@
         <v>60</v>
       </c>
       <c r="Q46" s="9" t="s">
-        <v>1197</v>
+        <v>1199</v>
       </c>
       <c r="R46" s="9" t="s">
         <v>153</v>
@@ -14441,7 +14441,7 @@
         <v>60</v>
       </c>
       <c r="Q47" s="9" t="s">
-        <v>1197</v>
+        <v>1199</v>
       </c>
       <c r="R47" s="9" t="s">
         <v>153</v>
@@ -14506,7 +14506,7 @@
         <v>645</v>
       </c>
       <c r="Q48" s="9" t="s">
-        <v>1197</v>
+        <v>1199</v>
       </c>
       <c r="R48" s="9" t="s">
         <v>153</v>
@@ -16661,7 +16661,7 @@
         <v>67</v>
       </c>
       <c r="T81" s="10">
-        <v>1448</v>
+        <v>1468</v>
       </c>
     </row>
     <row r="82" spans="1:20" x14ac:dyDescent="0.2">
@@ -17756,7 +17756,7 @@
         <v>641</v>
       </c>
       <c r="Q98" s="9" t="s">
-        <v>1197</v>
+        <v>1199</v>
       </c>
       <c r="R98" s="9" t="s">
         <v>153</v>
@@ -17821,7 +17821,7 @@
         <v>644</v>
       </c>
       <c r="Q99" s="9" t="s">
-        <v>1197</v>
+        <v>1199</v>
       </c>
       <c r="R99" s="9" t="s">
         <v>153</v>
@@ -17966,7 +17966,7 @@
     </row>
     <row r="102" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A102" s="7" t="s">
-        <v>1198</v>
+        <v>1197</v>
       </c>
       <c r="B102" s="10">
         <v>2015</v>
@@ -18001,7 +18001,7 @@
         <v>152</v>
       </c>
       <c r="L102" s="9" t="s">
-        <v>1199</v>
+        <v>1198</v>
       </c>
       <c r="M102" s="10">
         <v>4</v>
@@ -18016,7 +18016,7 @@
         <v>709</v>
       </c>
       <c r="Q102" s="9" t="s">
-        <v>1197</v>
+        <v>1199</v>
       </c>
       <c r="R102" s="9" t="s">
         <v>153</v>

</xml_diff>

<commit_message>
#47 Reading List: updated to 2025-12-08 (nwkbpowershell migrated).
</commit_message>
<xml_diff>
--- a/data/Reading List.xlsx
+++ b/data/Reading List.xlsx
@@ -16271,7 +16271,7 @@
         <v>57</v>
       </c>
       <c r="T75" s="10">
-        <v>255</v>
+        <v>276</v>
       </c>
     </row>
     <row r="76" spans="1:20" x14ac:dyDescent="0.2">
@@ -24525,7 +24525,7 @@
         <v>254</v>
       </c>
       <c r="T202" s="10">
-        <v>308</v>
+        <v>316</v>
       </c>
     </row>
     <row r="203" spans="1:20" x14ac:dyDescent="0.2">
@@ -24590,7 +24590,7 @@
         <v>280</v>
       </c>
       <c r="T203" s="10">
-        <v>48</v>
+        <v>43</v>
       </c>
     </row>
     <row r="204" spans="1:20" x14ac:dyDescent="0.2">
@@ -24655,7 +24655,7 @@
         <v>232</v>
       </c>
       <c r="T204" s="10">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="205" spans="1:20" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
#47 Reading List: updated to 2025-12-15 (added all  missing KBSize values).
</commit_message>
<xml_diff>
--- a/data/Reading List.xlsx
+++ b/data/Reading List.xlsx
@@ -3364,9 +3364,6 @@
     <t>Useful. Ok as a Getting Started book for beginners.</t>
   </si>
   <si>
-    <t>Safe 5.0 Distilled</t>
-  </si>
-  <si>
     <t>2025-06-26</t>
   </si>
   <si>
@@ -3653,6 +3650,9 @@
   </si>
   <si>
     <t>Data Science At The Command Line</t>
+  </si>
+  <si>
+    <t>SAFe 5.0 Distilled</t>
   </si>
 </sst>
 </file>
@@ -12320,7 +12320,7 @@
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A15" s="7" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
       <c r="B15" s="43">
         <v>2014</v>
@@ -12338,7 +12338,7 @@
         <v>272</v>
       </c>
       <c r="G15" s="42" t="s">
-        <v>1192</v>
+        <v>1191</v>
       </c>
       <c r="H15" s="14">
         <f>YEAR(G15)</f>
@@ -12367,10 +12367,10 @@
         <v>632</v>
       </c>
       <c r="P15" s="22" t="s">
-        <v>1193</v>
+        <v>1192</v>
       </c>
       <c r="Q15" s="9" t="s">
-        <v>1196</v>
+        <v>1195</v>
       </c>
       <c r="R15" s="9" t="s">
         <v>153</v>
@@ -12515,7 +12515,7 @@
     </row>
     <row r="18" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A18" s="7" t="s">
-        <v>1136</v>
+        <v>1135</v>
       </c>
       <c r="B18" s="10">
         <v>2015</v>
@@ -12630,7 +12630,7 @@
         <v>60</v>
       </c>
       <c r="Q19" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R19" s="9" t="s">
         <v>153</v>
@@ -12645,7 +12645,7 @@
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A20" s="7" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="B20" s="10">
         <v>2014</v>
@@ -12825,7 +12825,7 @@
         <v>663</v>
       </c>
       <c r="Q22" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R22" s="9" t="s">
         <v>153</v>
@@ -13215,7 +13215,7 @@
         <v>666</v>
       </c>
       <c r="Q28" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R28" s="9" t="s">
         <v>153</v>
@@ -13230,7 +13230,7 @@
     </row>
     <row r="29" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A29" s="7" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
       <c r="B29" s="10">
         <v>2009</v>
@@ -13280,7 +13280,7 @@
         <v>667</v>
       </c>
       <c r="Q29" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R29" s="9" t="s">
         <v>153</v>
@@ -13345,7 +13345,7 @@
         <v>636</v>
       </c>
       <c r="Q30" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R30" s="9" t="s">
         <v>153</v>
@@ -13815,7 +13815,7 @@
     </row>
     <row r="38" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A38" s="7" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
       <c r="B38" s="10">
         <v>2013</v>
@@ -14075,7 +14075,7 @@
     </row>
     <row r="42" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A42" s="7" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="B42" s="10">
         <v>1996</v>
@@ -14140,7 +14140,7 @@
     </row>
     <row r="43" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A43" s="7" t="s">
-        <v>1139</v>
+        <v>1138</v>
       </c>
       <c r="B43" s="10">
         <v>2008</v>
@@ -14385,7 +14385,7 @@
         <v>60</v>
       </c>
       <c r="Q46" s="9" t="s">
-        <v>1196</v>
+        <v>1195</v>
       </c>
       <c r="R46" s="9" t="s">
         <v>153</v>
@@ -14450,7 +14450,7 @@
         <v>60</v>
       </c>
       <c r="Q47" s="9" t="s">
-        <v>1196</v>
+        <v>1195</v>
       </c>
       <c r="R47" s="9" t="s">
         <v>153</v>
@@ -14515,7 +14515,7 @@
         <v>643</v>
       </c>
       <c r="Q48" s="9" t="s">
-        <v>1196</v>
+        <v>1195</v>
       </c>
       <c r="R48" s="9" t="s">
         <v>153</v>
@@ -14660,7 +14660,7 @@
     </row>
     <row r="51" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A51" s="7" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="B51" s="10">
         <v>2010</v>
@@ -14840,7 +14840,7 @@
         <v>670</v>
       </c>
       <c r="Q53" s="9" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
       <c r="R53" s="9" t="s">
         <v>153</v>
@@ -14855,7 +14855,7 @@
     </row>
     <row r="54" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A54" s="7" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
       <c r="B54" s="10">
         <v>2015</v>
@@ -14920,7 +14920,7 @@
     </row>
     <row r="55" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A55" s="7" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="B55" s="10">
         <v>2003</v>
@@ -15050,7 +15050,7 @@
     </row>
     <row r="57" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A57" s="7" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
       <c r="B57" s="10">
         <v>2011</v>
@@ -15295,7 +15295,7 @@
         <v>60</v>
       </c>
       <c r="Q60" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R60" s="9" t="s">
         <v>153</v>
@@ -15700,7 +15700,7 @@
     </row>
     <row r="67" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="s">
-        <v>1131</v>
+        <v>1130</v>
       </c>
       <c r="B67" s="10">
         <v>2013</v>
@@ -16010,7 +16010,7 @@
         <v>684</v>
       </c>
       <c r="Q71" s="9" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
       <c r="R71" s="9" t="s">
         <v>153</v>
@@ -16090,7 +16090,7 @@
     </row>
     <row r="73" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A73" s="7" t="s">
-        <v>1157</v>
+        <v>1156</v>
       </c>
       <c r="B73" s="10">
         <v>2012</v>
@@ -16285,7 +16285,7 @@
     </row>
     <row r="76" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
       <c r="B76" s="10">
         <v>2007</v>
@@ -16675,7 +16675,7 @@
     </row>
     <row r="82" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A82" s="7" t="s">
-        <v>1132</v>
+        <v>1131</v>
       </c>
       <c r="B82" s="10">
         <v>2014</v>
@@ -16740,7 +16740,7 @@
     </row>
     <row r="83" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A83" s="7" t="s">
-        <v>1133</v>
+        <v>1132</v>
       </c>
       <c r="B83" s="10">
         <v>2013</v>
@@ -16870,7 +16870,7 @@
     </row>
     <row r="85" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A85" s="7" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
       <c r="B85" s="10">
         <v>2015</v>
@@ -17000,7 +17000,7 @@
     </row>
     <row r="87" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A87" s="7" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="B87" s="10">
         <v>2004</v>
@@ -17065,7 +17065,7 @@
     </row>
     <row r="88" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A88" s="7" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="B88" s="8">
         <v>1997</v>
@@ -17310,7 +17310,7 @@
         <v>701</v>
       </c>
       <c r="Q91" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R91" s="9" t="s">
         <v>153</v>
@@ -17502,7 +17502,7 @@
         <v>632</v>
       </c>
       <c r="P94" s="22" t="s">
-        <v>1134</v>
+        <v>1133</v>
       </c>
       <c r="Q94" s="9" t="s">
         <v>441</v>
@@ -17765,7 +17765,7 @@
         <v>639</v>
       </c>
       <c r="Q98" s="9" t="s">
-        <v>1196</v>
+        <v>1195</v>
       </c>
       <c r="R98" s="9" t="s">
         <v>153</v>
@@ -17830,7 +17830,7 @@
         <v>642</v>
       </c>
       <c r="Q99" s="9" t="s">
-        <v>1196</v>
+        <v>1195</v>
       </c>
       <c r="R99" s="9" t="s">
         <v>153</v>
@@ -17910,7 +17910,7 @@
     </row>
     <row r="101" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A101" s="12" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="B101" s="10">
         <v>2016</v>
@@ -17975,7 +17975,7 @@
     </row>
     <row r="102" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A102" s="7" t="s">
-        <v>1194</v>
+        <v>1193</v>
       </c>
       <c r="B102" s="10">
         <v>2015</v>
@@ -18010,7 +18010,7 @@
         <v>152</v>
       </c>
       <c r="L102" s="9" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
       <c r="M102" s="10">
         <v>4</v>
@@ -18025,7 +18025,7 @@
         <v>707</v>
       </c>
       <c r="Q102" s="9" t="s">
-        <v>1196</v>
+        <v>1195</v>
       </c>
       <c r="R102" s="9" t="s">
         <v>153</v>
@@ -18090,7 +18090,7 @@
         <v>708</v>
       </c>
       <c r="Q103" s="9" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="R103" s="9" t="s">
         <v>153</v>
@@ -18155,7 +18155,7 @@
         <v>709</v>
       </c>
       <c r="Q104" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R104" s="9" t="s">
         <v>153</v>
@@ -18220,7 +18220,7 @@
         <v>710</v>
       </c>
       <c r="Q105" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R105" s="9" t="s">
         <v>153</v>
@@ -18285,7 +18285,7 @@
         <v>711</v>
       </c>
       <c r="Q106" s="9" t="s">
-        <v>1188</v>
+        <v>1187</v>
       </c>
       <c r="R106" s="9" t="s">
         <v>153</v>
@@ -18350,7 +18350,7 @@
         <v>712</v>
       </c>
       <c r="Q107" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R107" s="9" t="s">
         <v>153</v>
@@ -18365,7 +18365,7 @@
     </row>
     <row r="108" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A108" s="7" t="s">
-        <v>1149</v>
+        <v>1148</v>
       </c>
       <c r="B108" s="10">
         <v>2017</v>
@@ -18383,7 +18383,7 @@
         <v>253</v>
       </c>
       <c r="G108" s="9" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="H108" s="14">
         <f t="shared" si="6"/>
@@ -18412,7 +18412,7 @@
         <v>632</v>
       </c>
       <c r="P108" s="22" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
       <c r="Q108" s="9" t="s">
         <v>442</v>
@@ -18430,7 +18430,7 @@
     </row>
     <row r="109" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A109" s="7" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="B109" s="10">
         <v>2007</v>
@@ -18448,7 +18448,7 @@
         <v>315</v>
       </c>
       <c r="G109" s="9" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
       <c r="H109" s="14">
         <f t="shared" si="6"/>
@@ -18477,7 +18477,7 @@
         <v>632</v>
       </c>
       <c r="P109" s="22" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
       <c r="Q109" s="9" t="s">
         <v>442</v>
@@ -18755,7 +18755,7 @@
     </row>
     <row r="114" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A114" s="7" t="s">
-        <v>1158</v>
+        <v>1157</v>
       </c>
       <c r="B114" s="8">
         <v>2015</v>
@@ -18870,7 +18870,7 @@
         <v>717</v>
       </c>
       <c r="Q115" s="9" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
       <c r="R115" s="9" t="s">
         <v>153</v>
@@ -18935,7 +18935,7 @@
         <v>718</v>
       </c>
       <c r="Q116" s="9" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
       <c r="R116" s="9" t="s">
         <v>153</v>
@@ -19000,7 +19000,7 @@
         <v>719</v>
       </c>
       <c r="Q117" s="9" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
       <c r="R117" s="9" t="s">
         <v>153</v>
@@ -19065,7 +19065,7 @@
         <v>720</v>
       </c>
       <c r="Q118" s="9" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
       <c r="R118" s="9" t="s">
         <v>153</v>
@@ -19145,7 +19145,7 @@
     </row>
     <row r="120" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A120" s="7" t="s">
-        <v>1159</v>
+        <v>1158</v>
       </c>
       <c r="B120" s="10">
         <v>2016</v>
@@ -19210,7 +19210,7 @@
     </row>
     <row r="121" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A121" s="7" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="B121" s="10">
         <v>2016</v>
@@ -19275,7 +19275,7 @@
     </row>
     <row r="122" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A122" s="7" t="s">
-        <v>1161</v>
+        <v>1160</v>
       </c>
       <c r="B122" s="10">
         <v>2016</v>
@@ -19470,7 +19470,7 @@
     </row>
     <row r="125" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A125" s="7" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
       <c r="B125" s="8">
         <v>2018</v>
@@ -19488,7 +19488,7 @@
         <v>339</v>
       </c>
       <c r="G125" s="9" t="s">
-        <v>1198</v>
+        <v>1197</v>
       </c>
       <c r="H125" s="14">
         <f t="shared" ref="H125" si="11">YEAR(G125)</f>
@@ -19505,7 +19505,7 @@
         <v>153</v>
       </c>
       <c r="L125" s="11" t="s">
-        <v>1199</v>
+        <v>1198</v>
       </c>
       <c r="M125" s="8">
         <v>2</v>
@@ -19520,7 +19520,7 @@
         <v>60</v>
       </c>
       <c r="Q125" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R125" s="9" t="s">
         <v>153</v>
@@ -19649,7 +19649,7 @@
         <v>724</v>
       </c>
       <c r="Q127" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R127" s="9" t="s">
         <v>153</v>
@@ -19844,7 +19844,7 @@
         <v>727</v>
       </c>
       <c r="Q130" s="9" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="R130" s="9" t="s">
         <v>153</v>
@@ -19909,7 +19909,7 @@
         <v>728</v>
       </c>
       <c r="Q131" s="9" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="R131" s="9" t="s">
         <v>153</v>
@@ -19974,7 +19974,7 @@
         <v>729</v>
       </c>
       <c r="Q132" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R132" s="9" t="s">
         <v>153</v>
@@ -20039,7 +20039,7 @@
         <v>730</v>
       </c>
       <c r="Q133" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R133" s="9" t="s">
         <v>153</v>
@@ -20104,7 +20104,7 @@
         <v>731</v>
       </c>
       <c r="Q134" s="9" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="R134" s="9" t="s">
         <v>153</v>
@@ -20184,7 +20184,7 @@
     </row>
     <row r="136" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A136" s="7" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
       <c r="B136" s="10">
         <v>2018</v>
@@ -20299,7 +20299,7 @@
         <v>734</v>
       </c>
       <c r="Q137" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R137" s="9" t="s">
         <v>153</v>
@@ -20429,7 +20429,7 @@
         <v>736</v>
       </c>
       <c r="Q139" s="9" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
       <c r="R139" s="9" t="s">
         <v>153</v>
@@ -20494,7 +20494,7 @@
         <v>737</v>
       </c>
       <c r="Q140" s="9" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="R140" s="9" t="s">
         <v>153</v>
@@ -20559,7 +20559,7 @@
         <v>738</v>
       </c>
       <c r="Q141" s="9" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="R141" s="9" t="s">
         <v>153</v>
@@ -20704,7 +20704,7 @@
     </row>
     <row r="144" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A144" s="7" t="s">
-        <v>1201</v>
+        <v>1200</v>
       </c>
       <c r="B144" s="10">
         <v>2018</v>
@@ -20754,7 +20754,7 @@
         <v>741</v>
       </c>
       <c r="Q144" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R144" s="9" t="s">
         <v>153</v>
@@ -20769,7 +20769,7 @@
     </row>
     <row r="145" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A145" s="7" t="s">
-        <v>1202</v>
+        <v>1201</v>
       </c>
       <c r="B145" s="10">
         <v>2015</v>
@@ -20819,7 +20819,7 @@
         <v>742</v>
       </c>
       <c r="Q145" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R145" s="9" t="s">
         <v>153</v>
@@ -20884,7 +20884,7 @@
         <v>642</v>
       </c>
       <c r="Q146" s="9" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="R146" s="9" t="s">
         <v>153</v>
@@ -20949,7 +20949,7 @@
         <v>743</v>
       </c>
       <c r="Q147" s="9" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="R147" s="9" t="s">
         <v>153</v>
@@ -21014,7 +21014,7 @@
         <v>744</v>
       </c>
       <c r="Q148" s="9" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="R148" s="9" t="s">
         <v>153</v>
@@ -21079,7 +21079,7 @@
         <v>642</v>
       </c>
       <c r="Q149" s="9" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="R149" s="9" t="s">
         <v>153</v>
@@ -21209,7 +21209,7 @@
         <v>746</v>
       </c>
       <c r="Q151" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R151" s="9" t="s">
         <v>153</v>
@@ -21274,7 +21274,7 @@
         <v>642</v>
       </c>
       <c r="Q152" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R152" s="9" t="s">
         <v>153</v>
@@ -21339,7 +21339,7 @@
         <v>642</v>
       </c>
       <c r="Q153" s="9" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
       <c r="R153" s="9" t="s">
         <v>153</v>
@@ -21794,7 +21794,7 @@
         <v>752</v>
       </c>
       <c r="Q160" s="9" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="R160" s="9" t="s">
         <v>153</v>
@@ -21859,7 +21859,7 @@
         <v>753</v>
       </c>
       <c r="Q161" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R161" s="9" t="s">
         <v>152</v>
@@ -21989,7 +21989,7 @@
         <v>755</v>
       </c>
       <c r="Q163" s="9" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="R163" s="9" t="s">
         <v>153</v>
@@ -22054,7 +22054,7 @@
         <v>756</v>
       </c>
       <c r="Q164" s="9" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="R164" s="9" t="s">
         <v>152</v>
@@ -22119,7 +22119,7 @@
         <v>757</v>
       </c>
       <c r="Q165" s="9" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="R165" s="9" t="s">
         <v>152</v>
@@ -22184,7 +22184,7 @@
         <v>758</v>
       </c>
       <c r="Q166" s="9" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="R166" s="9" t="s">
         <v>153</v>
@@ -22249,7 +22249,7 @@
         <v>759</v>
       </c>
       <c r="Q167" s="9" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="R167" s="9" t="s">
         <v>153</v>
@@ -22314,7 +22314,7 @@
         <v>760</v>
       </c>
       <c r="Q168" s="9" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="R168" s="9" t="s">
         <v>153</v>
@@ -22574,7 +22574,7 @@
         <v>762</v>
       </c>
       <c r="Q172" s="9" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
       <c r="R172" s="9" t="s">
         <v>153</v>
@@ -22639,7 +22639,7 @@
         <v>657</v>
       </c>
       <c r="Q173" s="9" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="R173" s="9" t="s">
         <v>153</v>
@@ -22704,7 +22704,7 @@
         <v>763</v>
       </c>
       <c r="Q174" s="9" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="R174" s="9" t="s">
         <v>153</v>
@@ -22899,7 +22899,7 @@
         <v>766</v>
       </c>
       <c r="Q177" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R177" s="9" t="s">
         <v>152</v>
@@ -22964,7 +22964,7 @@
         <v>767</v>
       </c>
       <c r="Q178" s="9" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="R178" s="9" t="s">
         <v>152</v>
@@ -23029,7 +23029,7 @@
         <v>768</v>
       </c>
       <c r="Q179" s="9" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="R179" s="9" t="s">
         <v>153</v>
@@ -23239,7 +23239,7 @@
     </row>
     <row r="183" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A183" s="7" t="s">
-        <v>1135</v>
+        <v>1134</v>
       </c>
       <c r="B183" s="10">
         <v>2013</v>
@@ -23549,7 +23549,7 @@
         <v>720</v>
       </c>
       <c r="Q187" s="9" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="R187" s="9" t="s">
         <v>153</v>
@@ -23809,7 +23809,7 @@
         <v>773</v>
       </c>
       <c r="Q191" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R191" s="9" t="s">
         <v>152</v>
@@ -23874,7 +23874,7 @@
         <v>774</v>
       </c>
       <c r="Q192" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R192" s="9" t="s">
         <v>152</v>
@@ -24004,7 +24004,7 @@
         <v>642</v>
       </c>
       <c r="Q194" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R194" s="9" t="s">
         <v>153</v>
@@ -25369,7 +25369,7 @@
         <v>787</v>
       </c>
       <c r="Q215" s="9" t="s">
-        <v>1188</v>
+        <v>1187</v>
       </c>
       <c r="R215" s="9" t="s">
         <v>153</v>
@@ -25434,7 +25434,7 @@
         <v>788</v>
       </c>
       <c r="Q216" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R216" s="9" t="s">
         <v>153</v>
@@ -25499,7 +25499,7 @@
         <v>789</v>
       </c>
       <c r="Q217" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R217" s="9" t="s">
         <v>153</v>
@@ -25629,7 +25629,7 @@
         <v>791</v>
       </c>
       <c r="Q219" s="9" t="s">
-        <v>1188</v>
+        <v>1187</v>
       </c>
       <c r="R219" s="9" t="s">
         <v>153</v>
@@ -25824,7 +25824,7 @@
         <v>794</v>
       </c>
       <c r="Q222" s="9" t="s">
-        <v>1188</v>
+        <v>1187</v>
       </c>
       <c r="R222" s="9" t="s">
         <v>153</v>
@@ -25889,7 +25889,7 @@
         <v>642</v>
       </c>
       <c r="Q223" s="9" t="s">
-        <v>1188</v>
+        <v>1187</v>
       </c>
       <c r="R223" s="9" t="s">
         <v>153</v>
@@ -26344,7 +26344,7 @@
         <v>60</v>
       </c>
       <c r="Q230" s="9" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
       <c r="R230" s="9" t="s">
         <v>153</v>
@@ -26359,7 +26359,7 @@
     </row>
     <row r="231" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A231" s="7" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
       <c r="B231" s="10">
         <v>2019</v>
@@ -26409,7 +26409,7 @@
         <v>786</v>
       </c>
       <c r="Q231" s="9" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="R231" s="9" t="s">
         <v>153</v>
@@ -26879,7 +26879,7 @@
     </row>
     <row r="239" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A239" s="7" t="s">
-        <v>1154</v>
+        <v>1153</v>
       </c>
       <c r="B239" s="10">
         <v>2009</v>
@@ -26897,7 +26897,7 @@
         <v>206</v>
       </c>
       <c r="G239" s="9" t="s">
-        <v>1153</v>
+        <v>1152</v>
       </c>
       <c r="H239" s="9">
         <f t="shared" si="36"/>
@@ -26926,7 +26926,7 @@
         <v>632</v>
       </c>
       <c r="P239" s="22" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
       <c r="Q239" s="9" t="s">
         <v>442</v>
@@ -26994,7 +26994,7 @@
         <v>803</v>
       </c>
       <c r="Q240" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R240" s="9" t="s">
         <v>153</v>
@@ -27124,7 +27124,7 @@
         <v>825</v>
       </c>
       <c r="Q242" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R242" s="9" t="s">
         <v>153</v>
@@ -27254,7 +27254,7 @@
         <v>813</v>
       </c>
       <c r="Q244" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R244" s="9" t="s">
         <v>153</v>
@@ -27384,7 +27384,7 @@
         <v>58</v>
       </c>
       <c r="Q246" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R246" s="9" t="s">
         <v>153</v>
@@ -27449,7 +27449,7 @@
         <v>642</v>
       </c>
       <c r="Q247" s="9" t="s">
-        <v>1188</v>
+        <v>1187</v>
       </c>
       <c r="R247" s="9" t="s">
         <v>153</v>
@@ -27774,7 +27774,7 @@
         <v>835</v>
       </c>
       <c r="Q252" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R252" s="9" t="s">
         <v>153</v>
@@ -28099,7 +28099,7 @@
         <v>851</v>
       </c>
       <c r="Q257" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R257" s="9" t="s">
         <v>153</v>
@@ -28294,7 +28294,7 @@
         <v>859</v>
       </c>
       <c r="Q260" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R260" s="9" t="s">
         <v>153</v>
@@ -29999,7 +29999,7 @@
     </row>
     <row r="287" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A287" s="7" t="s">
-        <v>1155</v>
+        <v>1154</v>
       </c>
       <c r="B287" s="14">
         <v>2024</v>
@@ -30179,7 +30179,7 @@
         <v>932</v>
       </c>
       <c r="Q289" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R289" s="9" t="s">
         <v>153</v>
@@ -31089,7 +31089,7 @@
         <v>969</v>
       </c>
       <c r="Q303" s="9" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="R303" s="9" t="s">
         <v>153</v>
@@ -31154,7 +31154,7 @@
         <v>972</v>
       </c>
       <c r="Q304" s="9" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="R304" s="9" t="s">
         <v>153</v>
@@ -31479,7 +31479,7 @@
         <v>983</v>
       </c>
       <c r="Q309" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R309" s="9" t="s">
         <v>153</v>
@@ -33234,7 +33234,7 @@
         <v>1053</v>
       </c>
       <c r="Q336" s="9" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
       <c r="R336" s="9" t="s">
         <v>153</v>
@@ -33299,7 +33299,7 @@
         <v>1057</v>
       </c>
       <c r="Q337" s="9" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
       <c r="R337" s="9" t="s">
         <v>153</v>
@@ -33364,7 +33364,7 @@
         <v>1060</v>
       </c>
       <c r="Q338" s="9" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
       <c r="R338" s="9" t="s">
         <v>153</v>
@@ -34014,7 +34014,7 @@
         <v>1085</v>
       </c>
       <c r="Q348" s="9" t="s">
-        <v>1188</v>
+        <v>1187</v>
       </c>
       <c r="R348" s="9" t="s">
         <v>153</v>
@@ -34024,7 +34024,7 @@
         <v>194</v>
       </c>
       <c r="T348" s="14">
-        <v>0</v>
+        <v>87</v>
       </c>
     </row>
     <row r="349" spans="1:20" x14ac:dyDescent="0.2">
@@ -34089,7 +34089,7 @@
         <v>293</v>
       </c>
       <c r="T349" s="14">
-        <v>0</v>
+        <v>72</v>
       </c>
     </row>
     <row r="350" spans="1:20" x14ac:dyDescent="0.2">
@@ -34154,7 +34154,7 @@
         <v>117</v>
       </c>
       <c r="T350" s="14">
-        <v>0</v>
+        <v>460</v>
       </c>
     </row>
     <row r="351" spans="1:20" x14ac:dyDescent="0.2">
@@ -34219,7 +34219,7 @@
         <v>165</v>
       </c>
       <c r="T351" s="14">
-        <v>0</v>
+        <v>234</v>
       </c>
     </row>
     <row r="352" spans="1:20" x14ac:dyDescent="0.2">
@@ -34284,7 +34284,7 @@
         <v>83</v>
       </c>
       <c r="T352" s="14">
-        <v>0</v>
+        <v>197</v>
       </c>
     </row>
     <row r="353" spans="1:20" x14ac:dyDescent="0.2">
@@ -34349,7 +34349,7 @@
         <v>85</v>
       </c>
       <c r="T353" s="14">
-        <v>0</v>
+        <v>430</v>
       </c>
     </row>
     <row r="354" spans="1:20" x14ac:dyDescent="0.2">
@@ -34404,7 +34404,7 @@
         <v>1102</v>
       </c>
       <c r="Q354" s="9" t="s">
-        <v>1188</v>
+        <v>1187</v>
       </c>
       <c r="R354" s="9" t="s">
         <v>153</v>
@@ -34414,7 +34414,7 @@
         <v>99</v>
       </c>
       <c r="T354" s="14">
-        <v>0</v>
+        <v>216</v>
       </c>
     </row>
     <row r="355" spans="1:20" x14ac:dyDescent="0.2">
@@ -34479,12 +34479,12 @@
         <v>51</v>
       </c>
       <c r="T355" s="14">
-        <v>0</v>
+        <v>217</v>
       </c>
     </row>
     <row r="356" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A356" s="7" t="s">
-        <v>1106</v>
+        <v>1202</v>
       </c>
       <c r="B356" s="14">
         <v>2020</v>
@@ -34502,7 +34502,7 @@
         <v>321</v>
       </c>
       <c r="G356" s="9" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="H356" s="9">
         <f t="shared" ref="H356" si="185">YEAR(G356)</f>
@@ -34531,7 +34531,7 @@
         <v>632</v>
       </c>
       <c r="P356" s="7" t="s">
-        <v>1108</v>
+        <v>1107</v>
       </c>
       <c r="Q356" s="9" t="s">
         <v>923</v>
@@ -34544,12 +34544,12 @@
         <v>53</v>
       </c>
       <c r="T356" s="14">
-        <v>0</v>
+        <v>518</v>
       </c>
     </row>
     <row r="357" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A357" s="7" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="B357" s="14">
         <v>2025</v>
@@ -34567,7 +34567,7 @@
         <v>123</v>
       </c>
       <c r="G357" s="9" t="s">
-        <v>1110</v>
+        <v>1109</v>
       </c>
       <c r="H357" s="9">
         <f t="shared" ref="H357" si="187">YEAR(G357)</f>
@@ -34596,7 +34596,7 @@
         <v>632</v>
       </c>
       <c r="P357" s="7" t="s">
-        <v>1112</v>
+        <v>1111</v>
       </c>
       <c r="Q357" s="9" t="s">
         <v>470</v>
@@ -34609,12 +34609,12 @@
         <v>50</v>
       </c>
       <c r="T357" s="14">
-        <v>0</v>
+        <v>124</v>
       </c>
     </row>
     <row r="358" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A358" s="7" t="s">
-        <v>1111</v>
+        <v>1110</v>
       </c>
       <c r="B358" s="14">
         <v>2020</v>
@@ -34632,7 +34632,7 @@
         <v>131</v>
       </c>
       <c r="G358" s="9" t="s">
-        <v>1113</v>
+        <v>1112</v>
       </c>
       <c r="H358" s="9">
         <f t="shared" ref="H358" si="189">YEAR(G358)</f>
@@ -34674,12 +34674,12 @@
         <v>16</v>
       </c>
       <c r="T358" s="14">
-        <v>0</v>
+        <v>338</v>
       </c>
     </row>
     <row r="359" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A359" s="7" t="s">
-        <v>1114</v>
+        <v>1113</v>
       </c>
       <c r="B359" s="14">
         <v>2025</v>
@@ -34697,7 +34697,7 @@
         <v>485</v>
       </c>
       <c r="G359" s="9" t="s">
-        <v>1113</v>
+        <v>1112</v>
       </c>
       <c r="H359" s="9">
         <f t="shared" ref="H359" si="191">YEAR(G359)</f>
@@ -34726,7 +34726,7 @@
         <v>632</v>
       </c>
       <c r="P359" s="7" t="s">
-        <v>1117</v>
+        <v>1116</v>
       </c>
       <c r="Q359" s="9" t="s">
         <v>923</v>
@@ -34739,12 +34739,12 @@
         <v>131</v>
       </c>
       <c r="T359" s="14">
-        <v>0</v>
+        <v>135</v>
       </c>
     </row>
     <row r="360" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A360" s="7" t="s">
-        <v>1115</v>
+        <v>1114</v>
       </c>
       <c r="B360" s="14">
         <v>2024</v>
@@ -34762,7 +34762,7 @@
         <v>569</v>
       </c>
       <c r="G360" s="9" t="s">
-        <v>1116</v>
+        <v>1115</v>
       </c>
       <c r="H360" s="9">
         <f t="shared" ref="H360" si="193">YEAR(G360)</f>
@@ -34791,7 +34791,7 @@
         <v>632</v>
       </c>
       <c r="P360" s="7" t="s">
-        <v>1118</v>
+        <v>1117</v>
       </c>
       <c r="Q360" s="9" t="s">
         <v>919</v>
@@ -34804,12 +34804,12 @@
         <v>89</v>
       </c>
       <c r="T360" s="14">
-        <v>0</v>
+        <v>376</v>
       </c>
     </row>
     <row r="361" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A361" s="7" t="s">
-        <v>1119</v>
+        <v>1118</v>
       </c>
       <c r="B361" s="14">
         <v>2024</v>
@@ -34827,7 +34827,7 @@
         <v>236</v>
       </c>
       <c r="G361" s="9" t="s">
-        <v>1120</v>
+        <v>1119</v>
       </c>
       <c r="H361" s="9">
         <f t="shared" ref="H361" si="195">YEAR(G361)</f>
@@ -34856,10 +34856,10 @@
         <v>632</v>
       </c>
       <c r="P361" s="12" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
       <c r="Q361" s="9" t="s">
-        <v>1200</v>
+        <v>1155</v>
       </c>
       <c r="R361" s="9" t="s">
         <v>153</v>
@@ -34869,12 +34869,12 @@
         <v>206</v>
       </c>
       <c r="T361" s="14">
-        <v>0</v>
+        <v>278</v>
       </c>
     </row>
     <row r="362" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A362" s="7" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
       <c r="B362" s="14">
         <v>2024</v>
@@ -34892,7 +34892,7 @@
         <v>265</v>
       </c>
       <c r="G362" s="9" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
       <c r="H362" s="9">
         <f t="shared" ref="H362:H363" si="197">YEAR(G362)</f>
@@ -34921,10 +34921,10 @@
         <v>632</v>
       </c>
       <c r="P362" s="12" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
       <c r="Q362" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="R362" s="9" t="s">
         <v>153</v>
@@ -34934,12 +34934,12 @@
         <v>158</v>
       </c>
       <c r="T362" s="14">
-        <v>0</v>
+        <v>290</v>
       </c>
     </row>
     <row r="363" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A363" s="7" t="s">
-        <v>1125</v>
+        <v>1124</v>
       </c>
       <c r="B363" s="14">
         <v>2025</v>
@@ -34957,7 +34957,7 @@
         <v>362</v>
       </c>
       <c r="G363" s="9" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
       <c r="H363" s="9">
         <f t="shared" si="197"/>
@@ -34986,7 +34986,7 @@
         <v>632</v>
       </c>
       <c r="P363" s="7" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
       <c r="Q363" s="9" t="s">
         <v>538</v>
@@ -34999,12 +34999,12 @@
         <v>65</v>
       </c>
       <c r="T363" s="14">
-        <v>0</v>
+        <v>362</v>
       </c>
     </row>
     <row r="364" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A364" s="7" t="s">
-        <v>1162</v>
+        <v>1161</v>
       </c>
       <c r="B364" s="14">
         <v>2013</v>
@@ -35022,7 +35022,7 @@
         <v>135</v>
       </c>
       <c r="G364" s="9" t="s">
-        <v>1163</v>
+        <v>1162</v>
       </c>
       <c r="H364" s="9">
         <f t="shared" ref="H364" si="199">YEAR(G364)</f>
@@ -35051,10 +35051,10 @@
         <v>632</v>
       </c>
       <c r="P364" s="7" t="s">
-        <v>1164</v>
+        <v>1163</v>
       </c>
       <c r="Q364" s="9" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
       <c r="R364" s="9" t="s">
         <v>153</v>
@@ -35064,12 +35064,12 @@
         <v>47</v>
       </c>
       <c r="T364" s="14">
-        <v>0</v>
+        <v>218</v>
       </c>
     </row>
     <row r="365" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A365" s="7" t="s">
-        <v>1165</v>
+        <v>1164</v>
       </c>
       <c r="B365" s="14">
         <v>2015</v>
@@ -35087,7 +35087,7 @@
         <v>464</v>
       </c>
       <c r="G365" s="9" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
       <c r="H365" s="9">
         <f t="shared" ref="H365" si="201">YEAR(G365)</f>
@@ -35116,10 +35116,10 @@
         <v>632</v>
       </c>
       <c r="P365" s="7" t="s">
-        <v>1167</v>
+        <v>1166</v>
       </c>
       <c r="Q365" s="9" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
       <c r="R365" s="9" t="s">
         <v>153</v>
@@ -35129,12 +35129,12 @@
         <v>46</v>
       </c>
       <c r="T365" s="14">
-        <v>0</v>
+        <v>299</v>
       </c>
     </row>
     <row r="366" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A366" s="7" t="s">
-        <v>1168</v>
+        <v>1167</v>
       </c>
       <c r="B366" s="14">
         <v>2013</v>
@@ -35152,7 +35152,7 @@
         <v>369</v>
       </c>
       <c r="G366" s="9" t="s">
-        <v>1170</v>
+        <v>1169</v>
       </c>
       <c r="H366" s="9">
         <f t="shared" ref="H366" si="203">YEAR(G366)</f>
@@ -35169,7 +35169,7 @@
         <v>153</v>
       </c>
       <c r="L366" s="9" t="s">
-        <v>1169</v>
+        <v>1168</v>
       </c>
       <c r="M366" s="14">
         <v>2</v>
@@ -35181,7 +35181,7 @@
         <v>632</v>
       </c>
       <c r="P366" s="7" t="s">
-        <v>1171</v>
+        <v>1170</v>
       </c>
       <c r="Q366" s="9" t="s">
         <v>1067</v>
@@ -35194,12 +35194,12 @@
         <v>155</v>
       </c>
       <c r="T366" s="14">
-        <v>0</v>
+        <v>284</v>
       </c>
     </row>
     <row r="367" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A367" s="7" t="s">
-        <v>1172</v>
+        <v>1171</v>
       </c>
       <c r="B367" s="14">
         <v>2025</v>
@@ -35217,7 +35217,7 @@
         <v>78</v>
       </c>
       <c r="G367" s="9" t="s">
-        <v>1170</v>
+        <v>1169</v>
       </c>
       <c r="H367" s="9">
         <f t="shared" ref="H367" si="205">YEAR(G367)</f>
@@ -35246,7 +35246,7 @@
         <v>632</v>
       </c>
       <c r="P367" s="38" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="Q367" s="9" t="s">
         <v>1067</v>
@@ -35259,12 +35259,12 @@
         <v>72</v>
       </c>
       <c r="T367" s="14">
-        <v>0</v>
+        <v>501</v>
       </c>
     </row>
     <row r="368" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A368" s="7" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="B368" s="14">
         <v>2025</v>
@@ -35282,7 +35282,7 @@
         <v>43</v>
       </c>
       <c r="G368" s="9" t="s">
-        <v>1175</v>
+        <v>1174</v>
       </c>
       <c r="H368" s="9">
         <f t="shared" ref="H368" si="206">YEAR(G368)</f>
@@ -35311,7 +35311,7 @@
         <v>632</v>
       </c>
       <c r="P368" s="7" t="s">
-        <v>1176</v>
+        <v>1175</v>
       </c>
       <c r="Q368" s="9" t="s">
         <v>919</v>
@@ -35324,12 +35324,12 @@
         <v>94</v>
       </c>
       <c r="T368" s="14">
-        <v>0</v>
+        <v>128</v>
       </c>
     </row>
     <row r="369" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A369" s="7" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="B369" s="41">
         <v>2022</v>
@@ -35347,7 +35347,7 @@
         <v>236</v>
       </c>
       <c r="G369" s="9" t="s">
-        <v>1175</v>
+        <v>1174</v>
       </c>
       <c r="H369" s="9">
         <f t="shared" ref="H369" si="208">YEAR(G369)</f>
@@ -35376,7 +35376,7 @@
         <v>632</v>
       </c>
       <c r="P369" s="7" t="s">
-        <v>1178</v>
+        <v>1177</v>
       </c>
       <c r="Q369" s="9" t="s">
         <v>839</v>
@@ -35389,12 +35389,12 @@
         <v>37</v>
       </c>
       <c r="T369" s="14">
-        <v>0</v>
+        <v>132</v>
       </c>
     </row>
     <row r="370" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A370" s="7" t="s">
-        <v>1179</v>
+        <v>1178</v>
       </c>
       <c r="B370" s="41">
         <v>2024</v>
@@ -35412,7 +35412,7 @@
         <v>445</v>
       </c>
       <c r="G370" s="9" t="s">
-        <v>1175</v>
+        <v>1174</v>
       </c>
       <c r="H370" s="9">
         <f t="shared" ref="H370" si="210">YEAR(G370)</f>
@@ -35441,7 +35441,7 @@
         <v>632</v>
       </c>
       <c r="P370" s="7" t="s">
-        <v>1180</v>
+        <v>1179</v>
       </c>
       <c r="Q370" s="9" t="s">
         <v>919</v>
@@ -35454,12 +35454,12 @@
         <v>148</v>
       </c>
       <c r="T370" s="14">
-        <v>0</v>
+        <v>532</v>
       </c>
     </row>
     <row r="371" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A371" s="7" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
       <c r="B371" s="41">
         <v>2025</v>
@@ -35477,7 +35477,7 @@
         <v>82</v>
       </c>
       <c r="G371" s="9" t="s">
-        <v>1182</v>
+        <v>1181</v>
       </c>
       <c r="H371" s="9">
         <f t="shared" ref="H371" si="212">YEAR(G371)</f>
@@ -35506,7 +35506,7 @@
         <v>632</v>
       </c>
       <c r="P371" s="7" t="s">
-        <v>1183</v>
+        <v>1182</v>
       </c>
       <c r="Q371" s="9" t="s">
         <v>919</v>
@@ -35519,12 +35519,12 @@
         <v>45</v>
       </c>
       <c r="T371" s="14">
-        <v>0</v>
+        <v>334</v>
       </c>
     </row>
     <row r="372" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A372" s="7" t="s">
-        <v>1184</v>
+        <v>1183</v>
       </c>
       <c r="B372" s="41">
         <v>2025</v>
@@ -35542,7 +35542,7 @@
         <v>368</v>
       </c>
       <c r="G372" s="9" t="s">
-        <v>1185</v>
+        <v>1184</v>
       </c>
       <c r="H372" s="9">
         <f t="shared" ref="H372" si="214">YEAR(G372)</f>
@@ -35571,7 +35571,7 @@
         <v>632</v>
       </c>
       <c r="P372" s="7" t="s">
-        <v>1186</v>
+        <v>1185</v>
       </c>
       <c r="Q372" s="9" t="s">
         <v>919</v>
@@ -35584,7 +35584,7 @@
         <v>100</v>
       </c>
       <c r="T372" s="14">
-        <v>0</v>
+        <v>531</v>
       </c>
     </row>
     <row r="373" spans="1:20" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
#53 Reading List: updated to 2026-06-01.
</commit_message>
<xml_diff>
--- a/data/Reading List.xlsx
+++ b/data/Reading List.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dropbox\Repositories\py-nwreadinglist\nwreadinglist\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D78F65C-68D8-4445-9E1A-CD88A6C4AB89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="19425" windowHeight="10425" tabRatio="313" firstSheet="7" activeTab="7"/>
+    <workbookView xWindow="1140" yWindow="435" windowWidth="27105" windowHeight="13995" tabRatio="313" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Detailed2016" sheetId="16" state="hidden" r:id="rId1"/>
@@ -28,7 +29,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Books!$A$1:$T$371</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">Others!$A$1:$Q$5</definedName>
   </definedNames>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -37,6 +38,8 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -44,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5659" uniqueCount="1204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5815" uniqueCount="1233">
   <si>
     <t>Format</t>
   </si>
@@ -3656,16 +3659,103 @@
   </si>
   <si>
     <t>Underlines</t>
+  </si>
+  <si>
+    <t>Learning LangChain</t>
+  </si>
+  <si>
+    <t>2026-05-26</t>
+  </si>
+  <si>
+    <t>Useful. The first part of the book is about RAG, while the second one goes off-topic (multi-agent systems). Overall, an interesting book, well written and not repetitive.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Software Testing with Generative AI </t>
+  </si>
+  <si>
+    <t>Useless. It's a book full of very basic concepts such as prompting ChatGPT to get a generic testing plan. This book brings zero value to the reader.</t>
+  </si>
+  <si>
+    <t>AI-Driven Software Testing</t>
+  </si>
+  <si>
+    <t>Useless. Extremely repetitive and poorly edited book without any practical recipe but only lists of statements. Avoid.</t>
+  </si>
+  <si>
+    <t>Taking Testing Seriously</t>
+  </si>
+  <si>
+    <t>2026-05-28</t>
+  </si>
+  <si>
+    <t>Useless. It's an essay about testing, full of empty statements that bring zero practical value to the reader. 661 pages of absolute void.</t>
+  </si>
+  <si>
+    <t>97 Things Every Data Engineer Should Know</t>
+  </si>
+  <si>
+    <t>Useless. It's a nice idea to have one article per contribution, but the content is quite obvious and a bit repetitive. No practical value.</t>
+  </si>
+  <si>
+    <t>2026-05-31</t>
+  </si>
+  <si>
+    <t>The Value Vector</t>
+  </si>
+  <si>
+    <t>Useless. It's a book full of empty statements that brings zero personal and practical experience. Additionally, the fictional dialogues make the book very hard to read.</t>
+  </si>
+  <si>
+    <t>Python Data Science Cookbook</t>
+  </si>
+  <si>
+    <t>Useless. Few actionable recipes.</t>
+  </si>
+  <si>
+    <t>Production Ready Data Science</t>
+  </si>
+  <si>
+    <t>Useful. Still well written and easy to skim as her first book, but with way less original recipes and more beginner-oriented.</t>
+  </si>
+  <si>
+    <t>Ubuntu System Administration Guide</t>
+  </si>
+  <si>
+    <t>Useless. A list of basic commands and a book without personality.</t>
+  </si>
+  <si>
+    <t>Github Copilot Step By Step</t>
+  </si>
+  <si>
+    <t>Pearson</t>
+  </si>
+  <si>
+    <t>Useless. Obvious concepts and low readibility layout.</t>
+  </si>
+  <si>
+    <t>Atlassian DevOps Toolchain (1st Edition)</t>
+  </si>
+  <si>
+    <t>Useless. Just a showcase of screenshots and possible integrations between Jira and third-party tools.</t>
+  </si>
+  <si>
+    <t>AWS CDK In Practice</t>
+  </si>
+  <si>
+    <t>Useless. This book would be more useful with examples easier to relate to, perhaps multi-language.</t>
+  </si>
+  <si>
+    <t>Developing On AWS With C#</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3698,6 +3788,12 @@
       <i/>
       <sz val="9"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -3795,7 +3891,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3906,16 +4002,7 @@
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3927,6 +4014,10 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3945,9 +4036,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -3985,9 +4076,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -4022,7 +4113,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -4057,7 +4148,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -4230,7 +4321,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:H16"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
@@ -4239,16 +4330,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="14.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="45">
+      <c r="A1" s="42">
         <v>2016</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
-      <c r="H1" s="46"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="43"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="18" t="s">
@@ -5181,7 +5272,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:Q17"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12" outlineLevelCol="1" x14ac:dyDescent="0.2"/>
   <cols>
@@ -5685,7 +5776,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet11"/>
   <dimension ref="A1:H16"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
@@ -5694,16 +5785,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="14.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="45">
+      <c r="A1" s="42">
         <v>2017</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
-      <c r="H1" s="46"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="43"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="18" t="s">
@@ -6636,7 +6727,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet12"/>
   <dimension ref="A1:H16"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
@@ -6645,16 +6736,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="14.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="45">
+      <c r="A1" s="42">
         <v>2018</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
-      <c r="H1" s="46"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="43"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="18" t="s">
@@ -7587,7 +7678,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr codeName="Sheet13"/>
   <dimension ref="A1:H16"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
@@ -7596,16 +7687,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="14.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="45">
+      <c r="A1" s="42">
         <v>2019</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
-      <c r="H1" s="46"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="43"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="18" t="s">
@@ -8538,7 +8629,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr codeName="Sheet14"/>
   <dimension ref="A1:H16"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
@@ -8547,16 +8638,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="14.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="45">
+      <c r="A1" s="42">
         <v>2020</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
-      <c r="H1" s="46"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="43"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="18" t="s">
@@ -9489,7 +9580,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr codeName="Sheet15"/>
   <dimension ref="A1:H16"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
@@ -9498,16 +9589,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="14.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="45">
+      <c r="A1" s="42">
         <v>2021</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
-      <c r="H1" s="46"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="43"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="18" t="s">
@@ -10440,7 +10531,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <sheetPr codeName="Sheet16"/>
   <dimension ref="A1:H16"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
@@ -10449,16 +10540,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="14.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="45">
+      <c r="A1" s="42">
         <v>2022</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
-      <c r="H1" s="46"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="43"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="18" t="s">
@@ -11391,9 +11482,9 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <sheetPr codeName="Sheet5"/>
-  <dimension ref="A1:U380"/>
+  <dimension ref="A1:U400"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="57.42578125" style="1" customWidth="1"/>
@@ -11888,7 +11979,7 @@
       <c r="T7" s="10">
         <v>347</v>
       </c>
-      <c r="U7" s="44">
+      <c r="U7" s="41">
         <v>0</v>
       </c>
     </row>
@@ -12372,7 +12463,7 @@
       <c r="A15" s="7" t="s">
         <v>1190</v>
       </c>
-      <c r="B15" s="43">
+      <c r="B15" s="14">
         <v>2014</v>
       </c>
       <c r="C15" s="9" t="s">
@@ -12384,10 +12475,10 @@
       <c r="E15" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F15" s="43">
+      <c r="F15" s="14">
         <v>272</v>
       </c>
-      <c r="G15" s="42" t="s">
+      <c r="G15" s="9" t="s">
         <v>1191</v>
       </c>
       <c r="H15" s="14">
@@ -24671,7 +24762,7 @@
       <c r="T195" s="10">
         <v>874</v>
       </c>
-      <c r="U195" s="44">
+      <c r="U195" s="41">
         <v>0</v>
       </c>
     </row>
@@ -24739,7 +24830,7 @@
       <c r="T196" s="10">
         <v>110</v>
       </c>
-      <c r="U196" s="44">
+      <c r="U196" s="41">
         <v>2</v>
       </c>
     </row>
@@ -24807,7 +24898,7 @@
       <c r="T197" s="10">
         <v>1352</v>
       </c>
-      <c r="U197" s="44">
+      <c r="U197" s="41">
         <v>3</v>
       </c>
     </row>
@@ -24875,7 +24966,7 @@
       <c r="T198" s="10">
         <v>1977</v>
       </c>
-      <c r="U198" s="44">
+      <c r="U198" s="41">
         <v>14</v>
       </c>
     </row>
@@ -24943,7 +25034,7 @@
       <c r="T199" s="10">
         <v>482</v>
       </c>
-      <c r="U199" s="44">
+      <c r="U199" s="41">
         <v>3</v>
       </c>
     </row>
@@ -25011,7 +25102,7 @@
       <c r="T200" s="10">
         <v>348</v>
       </c>
-      <c r="U200" s="44">
+      <c r="U200" s="41">
         <v>0</v>
       </c>
     </row>
@@ -25079,7 +25170,7 @@
       <c r="T201" s="10">
         <v>392</v>
       </c>
-      <c r="U201" s="44">
+      <c r="U201" s="41">
         <v>3</v>
       </c>
     </row>
@@ -25147,7 +25238,7 @@
       <c r="T202" s="10">
         <v>1715</v>
       </c>
-      <c r="U202" s="44">
+      <c r="U202" s="41">
         <v>7</v>
       </c>
     </row>
@@ -25215,7 +25306,7 @@
       <c r="T203" s="10">
         <v>316</v>
       </c>
-      <c r="U203" s="44">
+      <c r="U203" s="41">
         <v>0</v>
       </c>
     </row>
@@ -25283,7 +25374,7 @@
       <c r="T204" s="10">
         <v>43</v>
       </c>
-      <c r="U204" s="44">
+      <c r="U204" s="41">
         <v>1</v>
       </c>
     </row>
@@ -25351,7 +25442,7 @@
       <c r="T205" s="10">
         <v>133</v>
       </c>
-      <c r="U205" s="44">
+      <c r="U205" s="41">
         <v>0</v>
       </c>
     </row>
@@ -25419,7 +25510,7 @@
       <c r="T206" s="10">
         <v>338</v>
       </c>
-      <c r="U206" s="44">
+      <c r="U206" s="41">
         <v>2</v>
       </c>
     </row>
@@ -25487,7 +25578,7 @@
       <c r="T207" s="10">
         <v>435</v>
       </c>
-      <c r="U207" s="44">
+      <c r="U207" s="41">
         <v>0</v>
       </c>
     </row>
@@ -25555,7 +25646,7 @@
       <c r="T208" s="10">
         <v>156</v>
       </c>
-      <c r="U208" s="44">
+      <c r="U208" s="41">
         <v>1</v>
       </c>
     </row>
@@ -25623,7 +25714,7 @@
       <c r="T209" s="10">
         <v>27</v>
       </c>
-      <c r="U209" s="44">
+      <c r="U209" s="41">
         <v>0</v>
       </c>
     </row>
@@ -25691,7 +25782,7 @@
       <c r="T210" s="10">
         <v>167</v>
       </c>
-      <c r="U210" s="44">
+      <c r="U210" s="41">
         <v>0</v>
       </c>
     </row>
@@ -25759,7 +25850,7 @@
       <c r="T211" s="10">
         <v>152</v>
       </c>
-      <c r="U211" s="44">
+      <c r="U211" s="41">
         <v>2</v>
       </c>
     </row>
@@ -25827,7 +25918,7 @@
       <c r="T212" s="10">
         <v>259</v>
       </c>
-      <c r="U212" s="44">
+      <c r="U212" s="41">
         <v>2</v>
       </c>
     </row>
@@ -25895,7 +25986,7 @@
       <c r="T213" s="10">
         <v>68</v>
       </c>
-      <c r="U213" s="44">
+      <c r="U213" s="41">
         <v>0</v>
       </c>
     </row>
@@ -25963,7 +26054,7 @@
       <c r="T214" s="10">
         <v>165</v>
       </c>
-      <c r="U214" s="44">
+      <c r="U214" s="41">
         <v>2</v>
       </c>
     </row>
@@ -26031,7 +26122,7 @@
       <c r="T215" s="10">
         <v>128</v>
       </c>
-      <c r="U215" s="44">
+      <c r="U215" s="41">
         <v>0</v>
       </c>
     </row>
@@ -28547,7 +28638,7 @@
       <c r="T252" s="10">
         <v>367</v>
       </c>
-      <c r="U252" s="44">
+      <c r="U252" s="41">
         <v>2</v>
       </c>
     </row>
@@ -33165,13 +33256,13 @@
         <v>153</v>
       </c>
       <c r="S320" s="14">
-        <f t="shared" ref="S320:S371" si="129">LEN(P320)</f>
+        <f t="shared" ref="S320:S384" si="129">LEN(P320)</f>
         <v>35</v>
       </c>
       <c r="T320" s="10">
         <v>139</v>
       </c>
-      <c r="U320" s="44">
+      <c r="U320" s="41">
         <v>0</v>
       </c>
     </row>
@@ -33239,7 +33330,7 @@
       <c r="T321" s="10">
         <v>59</v>
       </c>
-      <c r="U321" s="44">
+      <c r="U321" s="41">
         <v>0</v>
       </c>
     </row>
@@ -33307,7 +33398,7 @@
       <c r="T322" s="10">
         <v>524</v>
       </c>
-      <c r="U322" s="44">
+      <c r="U322" s="41">
         <v>1</v>
       </c>
     </row>
@@ -33375,7 +33466,7 @@
       <c r="T323" s="10">
         <v>224</v>
       </c>
-      <c r="U323" s="44">
+      <c r="U323" s="41">
         <v>0</v>
       </c>
     </row>
@@ -33443,7 +33534,7 @@
       <c r="T324" s="10">
         <v>360</v>
       </c>
-      <c r="U324" s="44">
+      <c r="U324" s="41">
         <v>2</v>
       </c>
     </row>
@@ -33511,7 +33602,7 @@
       <c r="T325" s="10">
         <v>32</v>
       </c>
-      <c r="U325" s="44">
+      <c r="U325" s="41">
         <v>0</v>
       </c>
     </row>
@@ -33579,7 +33670,7 @@
       <c r="T326" s="10">
         <v>0</v>
       </c>
-      <c r="U326" s="44">
+      <c r="U326" s="41">
         <v>0</v>
       </c>
     </row>
@@ -36047,7 +36138,7 @@
       <c r="E363" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F363" s="41">
+      <c r="F363" s="14">
         <v>135</v>
       </c>
       <c r="G363" s="9" t="s">
@@ -36070,7 +36161,7 @@
       <c r="L363" s="9" t="s">
         <v>350</v>
       </c>
-      <c r="M363" s="41">
+      <c r="M363" s="14">
         <v>4</v>
       </c>
       <c r="N363" s="35">
@@ -36115,7 +36206,7 @@
       <c r="E364" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F364" s="41">
+      <c r="F364" s="14">
         <v>464</v>
       </c>
       <c r="G364" s="9" t="s">
@@ -36141,7 +36232,7 @@
       <c r="M364" s="14">
         <v>3</v>
       </c>
-      <c r="N364" s="41">
+      <c r="N364" s="14">
         <v>60.99</v>
       </c>
       <c r="O364" s="9" t="s">
@@ -36183,7 +36274,7 @@
       <c r="E365" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F365" s="41">
+      <c r="F365" s="14">
         <v>369</v>
       </c>
       <c r="G365" s="9" t="s">
@@ -36209,7 +36300,7 @@
       <c r="M365" s="14">
         <v>2</v>
       </c>
-      <c r="N365" s="41">
+      <c r="N365" s="14">
         <v>19.989999999999998</v>
       </c>
       <c r="O365" s="9" t="s">
@@ -36251,7 +36342,7 @@
       <c r="E366" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F366" s="41">
+      <c r="F366" s="14">
         <v>78</v>
       </c>
       <c r="G366" s="9" t="s">
@@ -36274,7 +36365,7 @@
       <c r="L366" s="9" t="s">
         <v>570</v>
       </c>
-      <c r="M366" s="41">
+      <c r="M366" s="14">
         <v>5</v>
       </c>
       <c r="N366" s="35">
@@ -36319,7 +36410,7 @@
       <c r="E367" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F367" s="41">
+      <c r="F367" s="14">
         <v>43</v>
       </c>
       <c r="G367" s="9" t="s">
@@ -36375,7 +36466,7 @@
       <c r="A368" s="7" t="s">
         <v>1176</v>
       </c>
-      <c r="B368" s="41">
+      <c r="B368" s="14">
         <v>2022</v>
       </c>
       <c r="C368" s="9" t="s">
@@ -36387,7 +36478,7 @@
       <c r="E368" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F368" s="41">
+      <c r="F368" s="14">
         <v>236</v>
       </c>
       <c r="G368" s="9" t="s">
@@ -36413,7 +36504,7 @@
       <c r="M368" s="14">
         <v>3</v>
       </c>
-      <c r="N368" s="41">
+      <c r="N368" s="14">
         <v>31.99</v>
       </c>
       <c r="O368" s="9" t="s">
@@ -36443,7 +36534,7 @@
       <c r="A369" s="7" t="s">
         <v>1178</v>
       </c>
-      <c r="B369" s="41">
+      <c r="B369" s="14">
         <v>2024</v>
       </c>
       <c r="C369" s="9" t="s">
@@ -36455,7 +36546,7 @@
       <c r="E369" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F369" s="41">
+      <c r="F369" s="14">
         <v>445</v>
       </c>
       <c r="G369" s="9" t="s">
@@ -36481,7 +36572,7 @@
       <c r="M369" s="14">
         <v>1</v>
       </c>
-      <c r="N369" s="41">
+      <c r="N369" s="14">
         <v>43.99</v>
       </c>
       <c r="O369" s="9" t="s">
@@ -36511,7 +36602,7 @@
       <c r="A370" s="7" t="s">
         <v>1180</v>
       </c>
-      <c r="B370" s="41">
+      <c r="B370" s="14">
         <v>2025</v>
       </c>
       <c r="C370" s="9" t="s">
@@ -36523,7 +36614,7 @@
       <c r="E370" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F370" s="41">
+      <c r="F370" s="14">
         <v>82</v>
       </c>
       <c r="G370" s="9" t="s">
@@ -36546,10 +36637,10 @@
       <c r="L370" s="9" t="s">
         <v>343</v>
       </c>
-      <c r="M370" s="41">
-        <v>4</v>
-      </c>
-      <c r="N370" s="41">
+      <c r="M370" s="14">
+        <v>4</v>
+      </c>
+      <c r="N370" s="14">
         <v>79.989999999999995</v>
       </c>
       <c r="O370" s="9" t="s">
@@ -36579,7 +36670,7 @@
       <c r="A371" s="7" t="s">
         <v>1183</v>
       </c>
-      <c r="B371" s="41">
+      <c r="B371" s="14">
         <v>2025</v>
       </c>
       <c r="C371" s="9" t="s">
@@ -36591,18 +36682,18 @@
       <c r="E371" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F371" s="41">
+      <c r="F371" s="14">
         <v>368</v>
       </c>
       <c r="G371" s="9" t="s">
         <v>1184</v>
       </c>
       <c r="H371" s="9">
-        <f t="shared" ref="H371" si="214">YEAR(G371)</f>
+        <f t="shared" ref="H371:H381" si="214">YEAR(G371)</f>
         <v>2025</v>
       </c>
       <c r="I371" s="9">
-        <f t="shared" ref="I371" si="215">MONTH(G371)</f>
+        <f t="shared" ref="I371:I381" si="215">MONTH(G371)</f>
         <v>11</v>
       </c>
       <c r="J371" s="9" t="s">
@@ -36617,7 +36708,7 @@
       <c r="M371" s="14">
         <v>3</v>
       </c>
-      <c r="N371" s="41">
+      <c r="N371" s="14">
         <v>49.99</v>
       </c>
       <c r="O371" s="9" t="s">
@@ -36644,220 +36735,1266 @@
       </c>
     </row>
     <row r="372" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A372" s="9"/>
-      <c r="B372" s="9"/>
-      <c r="C372" s="9"/>
-      <c r="D372" s="9"/>
-      <c r="E372" s="9"/>
-      <c r="F372" s="9"/>
-      <c r="G372" s="9"/>
-      <c r="H372" s="9"/>
-      <c r="I372" s="9"/>
-      <c r="J372" s="9"/>
-      <c r="K372" s="9"/>
-      <c r="L372" s="9"/>
-      <c r="M372" s="9"/>
-      <c r="N372" s="9"/>
-      <c r="O372" s="9"/>
-      <c r="P372" s="9"/>
-      <c r="Q372" s="9"/>
-      <c r="R372" s="9"/>
-      <c r="S372" s="14"/>
-      <c r="T372" s="9"/>
-      <c r="U372" s="14"/>
+      <c r="A372" s="7" t="s">
+        <v>1204</v>
+      </c>
+      <c r="B372" s="44">
+        <v>2025</v>
+      </c>
+      <c r="C372" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D372" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E372" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F372" s="44">
+        <v>297</v>
+      </c>
+      <c r="G372" s="9" t="s">
+        <v>1205</v>
+      </c>
+      <c r="H372" s="9">
+        <f t="shared" si="214"/>
+        <v>2026</v>
+      </c>
+      <c r="I372" s="9">
+        <f t="shared" si="215"/>
+        <v>5</v>
+      </c>
+      <c r="J372" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K372" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L372" s="9" t="s">
+        <v>343</v>
+      </c>
+      <c r="M372" s="14">
+        <v>3</v>
+      </c>
+      <c r="N372" s="44">
+        <v>79.989999999999995</v>
+      </c>
+      <c r="O372" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P372" s="7" t="s">
+        <v>1206</v>
+      </c>
+      <c r="Q372" s="9" t="s">
+        <v>919</v>
+      </c>
+      <c r="R372" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S372" s="14">
+        <f t="shared" si="129"/>
+        <v>170</v>
+      </c>
+      <c r="T372" s="14">
+        <v>0</v>
+      </c>
+      <c r="U372" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="373" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A373" s="9"/>
-      <c r="B373" s="9"/>
-      <c r="C373" s="9"/>
-      <c r="D373" s="9"/>
-      <c r="E373" s="9"/>
-      <c r="F373" s="9"/>
-      <c r="G373" s="9"/>
-      <c r="H373" s="9"/>
-      <c r="I373" s="9"/>
-      <c r="J373" s="9"/>
-      <c r="K373" s="9"/>
-      <c r="L373" s="9"/>
-      <c r="M373" s="9"/>
-      <c r="N373" s="9"/>
-      <c r="O373" s="9"/>
-      <c r="P373" s="9"/>
-      <c r="Q373" s="9"/>
-      <c r="R373" s="9"/>
-      <c r="S373" s="14"/>
-      <c r="T373" s="9"/>
-      <c r="U373" s="14"/>
+      <c r="A373" s="7" t="s">
+        <v>1207</v>
+      </c>
+      <c r="B373" s="44">
+        <v>2025</v>
+      </c>
+      <c r="C373" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D373" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E373" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F373" s="44">
+        <v>306</v>
+      </c>
+      <c r="G373" s="9" t="s">
+        <v>1205</v>
+      </c>
+      <c r="H373" s="9">
+        <f t="shared" si="214"/>
+        <v>2026</v>
+      </c>
+      <c r="I373" s="9">
+        <f t="shared" si="215"/>
+        <v>5</v>
+      </c>
+      <c r="J373" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K373" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L373" s="9" t="s">
+        <v>345</v>
+      </c>
+      <c r="M373" s="44">
+        <v>1</v>
+      </c>
+      <c r="N373" s="44">
+        <v>59.99</v>
+      </c>
+      <c r="O373" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P373" s="12" t="s">
+        <v>1208</v>
+      </c>
+      <c r="Q373" s="9" t="s">
+        <v>919</v>
+      </c>
+      <c r="R373" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S373" s="14">
+        <f t="shared" si="129"/>
+        <v>148</v>
+      </c>
+      <c r="T373" s="14">
+        <v>0</v>
+      </c>
+      <c r="U373" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="374" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A374" s="9"/>
-      <c r="B374" s="9"/>
-      <c r="C374" s="9"/>
-      <c r="D374" s="9"/>
-      <c r="E374" s="9"/>
-      <c r="F374" s="9"/>
-      <c r="G374" s="9"/>
-      <c r="H374" s="9"/>
-      <c r="I374" s="9"/>
-      <c r="J374" s="9"/>
-      <c r="K374" s="9"/>
-      <c r="L374" s="9"/>
-      <c r="M374" s="9"/>
-      <c r="N374" s="9"/>
-      <c r="O374" s="9"/>
-      <c r="P374" s="9"/>
-      <c r="Q374" s="9"/>
-      <c r="R374" s="9"/>
-      <c r="S374" s="14"/>
-      <c r="T374" s="9"/>
-      <c r="U374" s="14"/>
+      <c r="A374" s="7" t="s">
+        <v>1209</v>
+      </c>
+      <c r="B374" s="44">
+        <v>2025</v>
+      </c>
+      <c r="C374" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D374" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E374" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F374" s="44">
+        <v>518</v>
+      </c>
+      <c r="G374" s="9" t="s">
+        <v>1205</v>
+      </c>
+      <c r="H374" s="9">
+        <f t="shared" si="214"/>
+        <v>2026</v>
+      </c>
+      <c r="I374" s="9">
+        <f t="shared" si="215"/>
+        <v>5</v>
+      </c>
+      <c r="J374" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K374" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L374" s="9" t="s">
+        <v>348</v>
+      </c>
+      <c r="M374" s="44">
+        <v>1</v>
+      </c>
+      <c r="N374" s="44">
+        <v>59.99</v>
+      </c>
+      <c r="O374" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P374" s="12" t="s">
+        <v>1210</v>
+      </c>
+      <c r="Q374" s="9" t="s">
+        <v>919</v>
+      </c>
+      <c r="R374" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S374" s="14">
+        <f t="shared" si="129"/>
+        <v>118</v>
+      </c>
+      <c r="T374" s="14">
+        <v>0</v>
+      </c>
+      <c r="U374" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="375" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A375" s="9"/>
-      <c r="B375" s="9"/>
-      <c r="C375" s="9"/>
-      <c r="D375" s="9"/>
-      <c r="E375" s="9"/>
-      <c r="F375" s="9"/>
-      <c r="G375" s="9"/>
-      <c r="H375" s="9"/>
-      <c r="I375" s="9"/>
-      <c r="J375" s="9"/>
-      <c r="K375" s="9"/>
-      <c r="L375" s="9"/>
-      <c r="M375" s="9"/>
-      <c r="N375" s="9"/>
-      <c r="O375" s="9"/>
-      <c r="P375" s="9"/>
-      <c r="Q375" s="9"/>
-      <c r="R375" s="9"/>
-      <c r="S375" s="14"/>
-      <c r="T375" s="9"/>
-      <c r="U375" s="14"/>
+      <c r="A375" s="7" t="s">
+        <v>1211</v>
+      </c>
+      <c r="B375" s="44">
+        <v>2025</v>
+      </c>
+      <c r="C375" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D375" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E375" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F375" s="44">
+        <v>661</v>
+      </c>
+      <c r="G375" s="9" t="s">
+        <v>1212</v>
+      </c>
+      <c r="H375" s="9">
+        <f t="shared" si="214"/>
+        <v>2026</v>
+      </c>
+      <c r="I375" s="9">
+        <f t="shared" si="215"/>
+        <v>5</v>
+      </c>
+      <c r="J375" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K375" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L375" s="9" t="s">
+        <v>352</v>
+      </c>
+      <c r="M375" s="44">
+        <v>1</v>
+      </c>
+      <c r="N375" s="35">
+        <v>63</v>
+      </c>
+      <c r="O375" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P375" s="12" t="s">
+        <v>1213</v>
+      </c>
+      <c r="Q375" s="9" t="s">
+        <v>442</v>
+      </c>
+      <c r="R375" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S375" s="14">
+        <f t="shared" si="129"/>
+        <v>137</v>
+      </c>
+      <c r="T375" s="14">
+        <v>0</v>
+      </c>
+      <c r="U375" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="376" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A376" s="9"/>
-      <c r="B376" s="9"/>
-      <c r="C376" s="9"/>
-      <c r="D376" s="9"/>
-      <c r="E376" s="9"/>
-      <c r="F376" s="9"/>
-      <c r="G376" s="9"/>
-      <c r="H376" s="9"/>
-      <c r="I376" s="9"/>
-      <c r="J376" s="9"/>
-      <c r="K376" s="9"/>
-      <c r="L376" s="9"/>
-      <c r="M376" s="9"/>
-      <c r="N376" s="9"/>
-      <c r="O376" s="9"/>
-      <c r="P376" s="9"/>
-      <c r="Q376" s="9"/>
-      <c r="R376" s="9"/>
-      <c r="S376" s="14"/>
-      <c r="T376" s="9"/>
-      <c r="U376" s="14"/>
+      <c r="A376" s="7" t="s">
+        <v>1214</v>
+      </c>
+      <c r="B376" s="44">
+        <v>2021</v>
+      </c>
+      <c r="C376" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D376" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E376" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F376" s="44">
+        <v>263</v>
+      </c>
+      <c r="G376" s="9" t="s">
+        <v>1212</v>
+      </c>
+      <c r="H376" s="9">
+        <f t="shared" si="214"/>
+        <v>2026</v>
+      </c>
+      <c r="I376" s="9">
+        <f t="shared" si="215"/>
+        <v>5</v>
+      </c>
+      <c r="J376" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K376" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L376" s="9" t="s">
+        <v>343</v>
+      </c>
+      <c r="M376" s="44">
+        <v>2</v>
+      </c>
+      <c r="N376" s="44">
+        <v>49.99</v>
+      </c>
+      <c r="O376" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P376" s="12" t="s">
+        <v>1215</v>
+      </c>
+      <c r="Q376" s="9" t="s">
+        <v>1188</v>
+      </c>
+      <c r="R376" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S376" s="14">
+        <f t="shared" si="129"/>
+        <v>138</v>
+      </c>
+      <c r="T376" s="14">
+        <v>0</v>
+      </c>
+      <c r="U376" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="377" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A377" s="9"/>
-      <c r="B377" s="9"/>
-      <c r="C377" s="9"/>
-      <c r="D377" s="9"/>
-      <c r="E377" s="9"/>
-      <c r="F377" s="9"/>
-      <c r="G377" s="9"/>
-      <c r="H377" s="9"/>
-      <c r="I377" s="9"/>
-      <c r="J377" s="9"/>
-      <c r="K377" s="9"/>
-      <c r="L377" s="9"/>
-      <c r="M377" s="9"/>
-      <c r="N377" s="9"/>
-      <c r="O377" s="9"/>
-      <c r="P377" s="9"/>
-      <c r="Q377" s="9"/>
-      <c r="R377" s="9"/>
-      <c r="S377" s="14"/>
-      <c r="T377" s="9"/>
-      <c r="U377" s="14"/>
+      <c r="A377" s="7" t="s">
+        <v>1217</v>
+      </c>
+      <c r="B377" s="44">
+        <v>2025</v>
+      </c>
+      <c r="C377" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D377" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E377" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F377" s="44">
+        <v>302</v>
+      </c>
+      <c r="G377" s="9" t="s">
+        <v>1216</v>
+      </c>
+      <c r="H377" s="9">
+        <f t="shared" si="214"/>
+        <v>2026</v>
+      </c>
+      <c r="I377" s="9">
+        <f t="shared" si="215"/>
+        <v>5</v>
+      </c>
+      <c r="J377" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K377" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L377" s="9" t="s">
+        <v>348</v>
+      </c>
+      <c r="M377" s="44">
+        <v>1</v>
+      </c>
+      <c r="N377" s="44">
+        <v>59.99</v>
+      </c>
+      <c r="O377" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P377" s="12" t="s">
+        <v>1218</v>
+      </c>
+      <c r="Q377" s="9" t="s">
+        <v>919</v>
+      </c>
+      <c r="R377" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S377" s="14">
+        <f t="shared" si="129"/>
+        <v>168</v>
+      </c>
+      <c r="T377" s="14">
+        <v>0</v>
+      </c>
+      <c r="U377" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="378" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A378" s="9"/>
-      <c r="B378" s="9"/>
-      <c r="C378" s="9"/>
-      <c r="D378" s="9"/>
-      <c r="E378" s="9"/>
-      <c r="F378" s="9"/>
-      <c r="G378" s="9"/>
-      <c r="H378" s="9"/>
-      <c r="I378" s="9"/>
-      <c r="J378" s="9"/>
-      <c r="K378" s="9"/>
-      <c r="L378" s="9"/>
-      <c r="M378" s="9"/>
-      <c r="N378" s="9"/>
-      <c r="O378" s="9"/>
-      <c r="P378" s="9"/>
-      <c r="Q378" s="9"/>
-      <c r="R378" s="9"/>
-      <c r="S378" s="14"/>
-      <c r="T378" s="9"/>
-      <c r="U378" s="14"/>
+      <c r="A378" s="7" t="s">
+        <v>1219</v>
+      </c>
+      <c r="B378" s="44">
+        <v>2025</v>
+      </c>
+      <c r="C378" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D378" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E378" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F378" s="44">
+        <v>186</v>
+      </c>
+      <c r="G378" s="9" t="s">
+        <v>1216</v>
+      </c>
+      <c r="H378" s="9">
+        <f t="shared" si="214"/>
+        <v>2026</v>
+      </c>
+      <c r="I378" s="9">
+        <f t="shared" si="215"/>
+        <v>5</v>
+      </c>
+      <c r="J378" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K378" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L378" s="9" t="s">
+        <v>1033</v>
+      </c>
+      <c r="M378" s="44">
+        <v>2</v>
+      </c>
+      <c r="N378" s="44">
+        <v>32.99</v>
+      </c>
+      <c r="O378" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P378" s="45" t="s">
+        <v>1220</v>
+      </c>
+      <c r="Q378" s="9" t="s">
+        <v>538</v>
+      </c>
+      <c r="R378" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S378" s="14">
+        <f t="shared" si="129"/>
+        <v>32</v>
+      </c>
+      <c r="T378" s="14">
+        <v>0</v>
+      </c>
+      <c r="U378" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="379" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A379" s="9"/>
-      <c r="B379" s="9"/>
-      <c r="C379" s="9"/>
-      <c r="D379" s="9"/>
-      <c r="E379" s="9"/>
-      <c r="F379" s="9"/>
-      <c r="G379" s="9"/>
-      <c r="H379" s="9"/>
-      <c r="I379" s="9"/>
-      <c r="J379" s="9"/>
-      <c r="K379" s="9"/>
-      <c r="L379" s="9"/>
-      <c r="M379" s="9"/>
-      <c r="N379" s="9"/>
-      <c r="O379" s="9"/>
-      <c r="P379" s="9"/>
-      <c r="Q379" s="9"/>
-      <c r="R379" s="9"/>
-      <c r="S379" s="14"/>
-      <c r="T379" s="9"/>
-      <c r="U379" s="14"/>
-    </row>
-    <row r="380" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A380" s="9"/>
-      <c r="B380" s="9"/>
-      <c r="C380" s="9"/>
-      <c r="D380" s="9"/>
-      <c r="E380" s="9"/>
-      <c r="F380" s="9"/>
-      <c r="G380" s="9"/>
-      <c r="H380" s="9"/>
-      <c r="I380" s="9"/>
-      <c r="J380" s="9"/>
-      <c r="K380" s="9"/>
-      <c r="L380" s="9"/>
-      <c r="M380" s="9"/>
-      <c r="N380" s="9"/>
-      <c r="O380" s="9"/>
-      <c r="P380" s="9"/>
-      <c r="Q380" s="9"/>
-      <c r="R380" s="9"/>
-      <c r="S380" s="14"/>
-      <c r="T380" s="9"/>
-      <c r="U380" s="14"/>
+      <c r="A379" s="7" t="s">
+        <v>1221</v>
+      </c>
+      <c r="B379" s="44">
+        <v>2025</v>
+      </c>
+      <c r="C379" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D379" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E379" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F379" s="44">
+        <v>229</v>
+      </c>
+      <c r="G379" s="9" t="s">
+        <v>1216</v>
+      </c>
+      <c r="H379" s="9">
+        <f t="shared" si="214"/>
+        <v>2026</v>
+      </c>
+      <c r="I379" s="9">
+        <f t="shared" si="215"/>
+        <v>5</v>
+      </c>
+      <c r="J379" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K379" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L379" s="9" t="s">
+        <v>570</v>
+      </c>
+      <c r="M379" s="44">
+        <v>3</v>
+      </c>
+      <c r="N379" s="44">
+        <v>37.380000000000003</v>
+      </c>
+      <c r="O379" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P379" s="12" t="s">
+        <v>1222</v>
+      </c>
+      <c r="Q379" s="9" t="s">
+        <v>538</v>
+      </c>
+      <c r="R379" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S379" s="14">
+        <f t="shared" si="129"/>
+        <v>125</v>
+      </c>
+      <c r="T379" s="14">
+        <v>0</v>
+      </c>
+      <c r="U379" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="380" spans="1:21" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A380" s="7" t="s">
+        <v>1223</v>
+      </c>
+      <c r="B380" s="44">
+        <v>2025</v>
+      </c>
+      <c r="C380" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D380" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E380" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F380" s="44">
+        <v>366</v>
+      </c>
+      <c r="G380" s="9" t="s">
+        <v>1216</v>
+      </c>
+      <c r="H380" s="9">
+        <f t="shared" si="214"/>
+        <v>2026</v>
+      </c>
+      <c r="I380" s="9">
+        <f t="shared" si="215"/>
+        <v>5</v>
+      </c>
+      <c r="J380" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K380" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L380" s="9" t="s">
+        <v>842</v>
+      </c>
+      <c r="M380" s="44">
+        <v>1</v>
+      </c>
+      <c r="N380" s="44">
+        <v>39.950000000000003</v>
+      </c>
+      <c r="O380" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P380" s="12" t="s">
+        <v>1224</v>
+      </c>
+      <c r="Q380" s="9" t="s">
+        <v>470</v>
+      </c>
+      <c r="R380" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S380" s="14">
+        <f t="shared" si="129"/>
+        <v>65</v>
+      </c>
+      <c r="T380" s="14">
+        <v>0</v>
+      </c>
+      <c r="U380" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="381" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A381" s="7" t="s">
+        <v>1225</v>
+      </c>
+      <c r="B381" s="44">
+        <v>2025</v>
+      </c>
+      <c r="C381" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D381" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E381" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F381" s="44">
+        <v>418</v>
+      </c>
+      <c r="G381" s="9" t="s">
+        <v>1216</v>
+      </c>
+      <c r="H381" s="9">
+        <f t="shared" si="214"/>
+        <v>2026</v>
+      </c>
+      <c r="I381" s="9">
+        <f t="shared" si="215"/>
+        <v>5</v>
+      </c>
+      <c r="J381" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K381" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L381" s="9" t="s">
+        <v>1226</v>
+      </c>
+      <c r="M381" s="44">
+        <v>1</v>
+      </c>
+      <c r="N381" s="44">
+        <v>54.99</v>
+      </c>
+      <c r="O381" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P381" s="45" t="s">
+        <v>1227</v>
+      </c>
+      <c r="Q381" s="9" t="s">
+        <v>919</v>
+      </c>
+      <c r="R381" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S381" s="14">
+        <f t="shared" si="129"/>
+        <v>53</v>
+      </c>
+      <c r="T381" s="14">
+        <v>0</v>
+      </c>
+      <c r="U381" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="382" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A382" s="7" t="s">
+        <v>1228</v>
+      </c>
+      <c r="B382" s="44">
+        <v>2024</v>
+      </c>
+      <c r="C382" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D382" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E382" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F382" s="44">
+        <v>582</v>
+      </c>
+      <c r="G382" s="9" t="s">
+        <v>1216</v>
+      </c>
+      <c r="H382" s="9">
+        <f t="shared" ref="H382:H384" si="216">YEAR(G382)</f>
+        <v>2026</v>
+      </c>
+      <c r="I382" s="9">
+        <f t="shared" ref="I382:I384" si="217">MONTH(G382)</f>
+        <v>5</v>
+      </c>
+      <c r="J382" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K382" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L382" s="9" t="s">
+        <v>341</v>
+      </c>
+      <c r="M382" s="44">
+        <v>1</v>
+      </c>
+      <c r="N382" s="44">
+        <v>46.99</v>
+      </c>
+      <c r="O382" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P382" s="12" t="s">
+        <v>1229</v>
+      </c>
+      <c r="Q382" s="9" t="s">
+        <v>839</v>
+      </c>
+      <c r="R382" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S382" s="14">
+        <f t="shared" si="129"/>
+        <v>101</v>
+      </c>
+      <c r="T382" s="14">
+        <v>0</v>
+      </c>
+      <c r="U382" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="383" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A383" s="7" t="s">
+        <v>1230</v>
+      </c>
+      <c r="B383" s="44">
+        <v>2023</v>
+      </c>
+      <c r="C383" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D383" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E383" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F383" s="44">
+        <v>196</v>
+      </c>
+      <c r="G383" s="9" t="s">
+        <v>1216</v>
+      </c>
+      <c r="H383" s="9">
+        <f t="shared" si="216"/>
+        <v>2026</v>
+      </c>
+      <c r="I383" s="9">
+        <f t="shared" si="217"/>
+        <v>5</v>
+      </c>
+      <c r="J383" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K383" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L383" s="9" t="s">
+        <v>341</v>
+      </c>
+      <c r="M383" s="44">
+        <v>1</v>
+      </c>
+      <c r="N383" s="44">
+        <v>51.99</v>
+      </c>
+      <c r="O383" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P383" s="12" t="s">
+        <v>1231</v>
+      </c>
+      <c r="Q383" s="9" t="s">
+        <v>839</v>
+      </c>
+      <c r="R383" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S383" s="14">
+        <f t="shared" si="129"/>
+        <v>98</v>
+      </c>
+      <c r="T383" s="14">
+        <v>0</v>
+      </c>
+      <c r="U383" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="384" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A384" s="7" t="s">
+        <v>1232</v>
+      </c>
+      <c r="B384" s="44">
+        <v>2023</v>
+      </c>
+      <c r="C384" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D384" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E384" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F384" s="44">
+        <v>259</v>
+      </c>
+      <c r="G384" s="9" t="s">
+        <v>1216</v>
+      </c>
+      <c r="H384" s="9">
+        <f t="shared" si="216"/>
+        <v>2026</v>
+      </c>
+      <c r="I384" s="9">
+        <f t="shared" si="217"/>
+        <v>5</v>
+      </c>
+      <c r="J384" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K384" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L384" s="9" t="s">
+        <v>343</v>
+      </c>
+      <c r="M384" s="44">
+        <v>2</v>
+      </c>
+      <c r="N384" s="44">
+        <v>56.99</v>
+      </c>
+      <c r="O384" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P384" s="45" t="s">
+        <v>642</v>
+      </c>
+      <c r="Q384" s="9" t="s">
+        <v>441</v>
+      </c>
+      <c r="R384" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S384" s="14">
+        <f t="shared" si="129"/>
+        <v>16</v>
+      </c>
+      <c r="T384" s="14">
+        <v>0</v>
+      </c>
+      <c r="U384" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="385" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A385" s="7"/>
+      <c r="B385" s="9"/>
+      <c r="C385" s="9"/>
+      <c r="D385" s="9"/>
+      <c r="E385" s="9"/>
+      <c r="F385" s="9"/>
+      <c r="G385" s="9"/>
+      <c r="H385" s="9"/>
+      <c r="I385" s="9"/>
+      <c r="J385" s="9"/>
+      <c r="K385" s="9"/>
+      <c r="L385" s="9"/>
+      <c r="M385" s="9"/>
+      <c r="N385" s="9"/>
+      <c r="O385" s="9"/>
+      <c r="P385" s="12"/>
+      <c r="Q385" s="9"/>
+      <c r="R385" s="9"/>
+      <c r="S385" s="14"/>
+      <c r="T385" s="9"/>
+      <c r="U385" s="14"/>
+    </row>
+    <row r="386" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A386" s="7"/>
+      <c r="B386" s="9"/>
+      <c r="C386" s="9"/>
+      <c r="D386" s="9"/>
+      <c r="E386" s="9"/>
+      <c r="F386" s="9"/>
+      <c r="G386" s="9"/>
+      <c r="H386" s="9"/>
+      <c r="I386" s="9"/>
+      <c r="J386" s="9"/>
+      <c r="K386" s="9"/>
+      <c r="L386" s="9"/>
+      <c r="M386" s="9"/>
+      <c r="N386" s="9"/>
+      <c r="O386" s="9"/>
+      <c r="P386" s="12"/>
+      <c r="Q386" s="9"/>
+      <c r="R386" s="9"/>
+      <c r="S386" s="14"/>
+      <c r="T386" s="9"/>
+      <c r="U386" s="14"/>
+    </row>
+    <row r="387" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A387" s="7"/>
+      <c r="B387" s="9"/>
+      <c r="C387" s="9"/>
+      <c r="D387" s="9"/>
+      <c r="E387" s="9"/>
+      <c r="F387" s="9"/>
+      <c r="G387" s="9"/>
+      <c r="H387" s="9"/>
+      <c r="I387" s="9"/>
+      <c r="J387" s="9"/>
+      <c r="K387" s="9"/>
+      <c r="L387" s="9"/>
+      <c r="M387" s="9"/>
+      <c r="N387" s="9"/>
+      <c r="O387" s="9"/>
+      <c r="P387" s="12"/>
+      <c r="Q387" s="9"/>
+      <c r="R387" s="9"/>
+      <c r="S387" s="14"/>
+      <c r="T387" s="9"/>
+      <c r="U387" s="14"/>
+    </row>
+    <row r="388" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A388" s="7"/>
+      <c r="B388" s="9"/>
+      <c r="C388" s="9"/>
+      <c r="D388" s="9"/>
+      <c r="E388" s="9"/>
+      <c r="F388" s="9"/>
+      <c r="G388" s="9"/>
+      <c r="H388" s="9"/>
+      <c r="I388" s="9"/>
+      <c r="J388" s="9"/>
+      <c r="K388" s="9"/>
+      <c r="L388" s="9"/>
+      <c r="M388" s="9"/>
+      <c r="N388" s="9"/>
+      <c r="O388" s="9"/>
+      <c r="P388" s="12"/>
+      <c r="Q388" s="9"/>
+      <c r="R388" s="9"/>
+      <c r="S388" s="14"/>
+      <c r="T388" s="9"/>
+      <c r="U388" s="14"/>
+    </row>
+    <row r="389" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A389" s="7"/>
+      <c r="B389" s="9"/>
+      <c r="C389" s="9"/>
+      <c r="D389" s="9"/>
+      <c r="E389" s="9"/>
+      <c r="F389" s="9"/>
+      <c r="G389" s="9"/>
+      <c r="H389" s="9"/>
+      <c r="I389" s="9"/>
+      <c r="J389" s="9"/>
+      <c r="K389" s="9"/>
+      <c r="L389" s="9"/>
+      <c r="M389" s="9"/>
+      <c r="N389" s="9"/>
+      <c r="O389" s="9"/>
+      <c r="P389" s="12"/>
+      <c r="Q389" s="9"/>
+      <c r="R389" s="9"/>
+      <c r="S389" s="14"/>
+      <c r="T389" s="9"/>
+      <c r="U389" s="14"/>
+    </row>
+    <row r="390" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A390" s="7"/>
+      <c r="B390" s="9"/>
+      <c r="C390" s="9"/>
+      <c r="D390" s="9"/>
+      <c r="E390" s="9"/>
+      <c r="F390" s="9"/>
+      <c r="G390" s="9"/>
+      <c r="H390" s="9"/>
+      <c r="I390" s="9"/>
+      <c r="J390" s="9"/>
+      <c r="K390" s="9"/>
+      <c r="L390" s="9"/>
+      <c r="M390" s="9"/>
+      <c r="N390" s="9"/>
+      <c r="O390" s="9"/>
+      <c r="P390" s="12"/>
+      <c r="Q390" s="9"/>
+      <c r="R390" s="9"/>
+      <c r="S390" s="14"/>
+      <c r="T390" s="9"/>
+      <c r="U390" s="14"/>
+    </row>
+    <row r="391" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A391" s="7"/>
+      <c r="B391" s="9"/>
+      <c r="C391" s="9"/>
+      <c r="D391" s="9"/>
+      <c r="E391" s="9"/>
+      <c r="F391" s="9"/>
+      <c r="G391" s="9"/>
+      <c r="H391" s="9"/>
+      <c r="I391" s="9"/>
+      <c r="J391" s="9"/>
+      <c r="K391" s="9"/>
+      <c r="L391" s="9"/>
+      <c r="M391" s="9"/>
+      <c r="N391" s="9"/>
+      <c r="O391" s="9"/>
+      <c r="P391" s="12"/>
+      <c r="Q391" s="9"/>
+      <c r="R391" s="9"/>
+      <c r="S391" s="14"/>
+      <c r="T391" s="9"/>
+      <c r="U391" s="14"/>
+    </row>
+    <row r="392" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A392" s="7"/>
+      <c r="B392" s="9"/>
+      <c r="C392" s="9"/>
+      <c r="D392" s="9"/>
+      <c r="E392" s="9"/>
+      <c r="F392" s="9"/>
+      <c r="G392" s="9"/>
+      <c r="H392" s="9"/>
+      <c r="I392" s="9"/>
+      <c r="J392" s="9"/>
+      <c r="K392" s="9"/>
+      <c r="L392" s="9"/>
+      <c r="M392" s="9"/>
+      <c r="N392" s="9"/>
+      <c r="O392" s="9"/>
+      <c r="P392" s="12"/>
+      <c r="Q392" s="9"/>
+      <c r="R392" s="9"/>
+      <c r="S392" s="14"/>
+      <c r="T392" s="9"/>
+      <c r="U392" s="14"/>
+    </row>
+    <row r="393" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A393" s="7"/>
+      <c r="B393" s="9"/>
+      <c r="C393" s="9"/>
+      <c r="D393" s="9"/>
+      <c r="E393" s="9"/>
+      <c r="F393" s="9"/>
+      <c r="G393" s="9"/>
+      <c r="H393" s="9"/>
+      <c r="I393" s="9"/>
+      <c r="J393" s="9"/>
+      <c r="K393" s="9"/>
+      <c r="L393" s="9"/>
+      <c r="M393" s="9"/>
+      <c r="N393" s="9"/>
+      <c r="O393" s="9"/>
+      <c r="P393" s="12"/>
+      <c r="Q393" s="9"/>
+      <c r="R393" s="9"/>
+      <c r="S393" s="14"/>
+      <c r="T393" s="9"/>
+      <c r="U393" s="14"/>
+    </row>
+    <row r="394" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A394" s="7"/>
+      <c r="B394" s="9"/>
+      <c r="C394" s="9"/>
+      <c r="D394" s="9"/>
+      <c r="E394" s="9"/>
+      <c r="F394" s="9"/>
+      <c r="G394" s="9"/>
+      <c r="H394" s="9"/>
+      <c r="I394" s="9"/>
+      <c r="J394" s="9"/>
+      <c r="K394" s="9"/>
+      <c r="L394" s="9"/>
+      <c r="M394" s="9"/>
+      <c r="N394" s="9"/>
+      <c r="O394" s="9"/>
+      <c r="P394" s="12"/>
+      <c r="Q394" s="9"/>
+      <c r="R394" s="9"/>
+      <c r="S394" s="14"/>
+      <c r="T394" s="9"/>
+      <c r="U394" s="14"/>
+    </row>
+    <row r="395" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A395" s="7"/>
+      <c r="B395" s="9"/>
+      <c r="C395" s="9"/>
+      <c r="D395" s="9"/>
+      <c r="E395" s="9"/>
+      <c r="F395" s="9"/>
+      <c r="G395" s="9"/>
+      <c r="H395" s="9"/>
+      <c r="I395" s="9"/>
+      <c r="J395" s="9"/>
+      <c r="K395" s="9"/>
+      <c r="L395" s="9"/>
+      <c r="M395" s="9"/>
+      <c r="N395" s="9"/>
+      <c r="O395" s="9"/>
+      <c r="P395" s="12"/>
+      <c r="Q395" s="9"/>
+      <c r="R395" s="9"/>
+      <c r="S395" s="14"/>
+      <c r="T395" s="9"/>
+      <c r="U395" s="14"/>
+    </row>
+    <row r="396" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A396" s="7"/>
+      <c r="B396" s="9"/>
+      <c r="C396" s="9"/>
+      <c r="D396" s="9"/>
+      <c r="E396" s="9"/>
+      <c r="F396" s="9"/>
+      <c r="G396" s="9"/>
+      <c r="H396" s="9"/>
+      <c r="I396" s="9"/>
+      <c r="J396" s="9"/>
+      <c r="K396" s="9"/>
+      <c r="L396" s="9"/>
+      <c r="M396" s="9"/>
+      <c r="N396" s="9"/>
+      <c r="O396" s="9"/>
+      <c r="P396" s="12"/>
+      <c r="Q396" s="9"/>
+      <c r="R396" s="9"/>
+      <c r="S396" s="14"/>
+      <c r="T396" s="9"/>
+      <c r="U396" s="14"/>
+    </row>
+    <row r="397" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A397" s="7"/>
+      <c r="B397" s="9"/>
+      <c r="C397" s="9"/>
+      <c r="D397" s="9"/>
+      <c r="E397" s="9"/>
+      <c r="F397" s="9"/>
+      <c r="G397" s="9"/>
+      <c r="H397" s="9"/>
+      <c r="I397" s="9"/>
+      <c r="J397" s="9"/>
+      <c r="K397" s="9"/>
+      <c r="L397" s="9"/>
+      <c r="M397" s="9"/>
+      <c r="N397" s="9"/>
+      <c r="O397" s="9"/>
+      <c r="P397" s="12"/>
+      <c r="Q397" s="9"/>
+      <c r="R397" s="9"/>
+      <c r="S397" s="14"/>
+      <c r="T397" s="9"/>
+      <c r="U397" s="14"/>
+    </row>
+    <row r="398" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A398" s="7"/>
+      <c r="B398" s="9"/>
+      <c r="C398" s="9"/>
+      <c r="D398" s="9"/>
+      <c r="E398" s="9"/>
+      <c r="F398" s="9"/>
+      <c r="G398" s="9"/>
+      <c r="H398" s="9"/>
+      <c r="I398" s="9"/>
+      <c r="J398" s="9"/>
+      <c r="K398" s="9"/>
+      <c r="L398" s="9"/>
+      <c r="M398" s="9"/>
+      <c r="N398" s="9"/>
+      <c r="O398" s="9"/>
+      <c r="P398" s="12"/>
+      <c r="Q398" s="9"/>
+      <c r="R398" s="9"/>
+      <c r="S398" s="14"/>
+      <c r="T398" s="9"/>
+      <c r="U398" s="14"/>
+    </row>
+    <row r="399" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A399" s="7"/>
+      <c r="B399" s="9"/>
+      <c r="C399" s="9"/>
+      <c r="D399" s="9"/>
+      <c r="E399" s="9"/>
+      <c r="F399" s="9"/>
+      <c r="G399" s="9"/>
+      <c r="H399" s="9"/>
+      <c r="I399" s="9"/>
+      <c r="J399" s="9"/>
+      <c r="K399" s="9"/>
+      <c r="L399" s="9"/>
+      <c r="M399" s="9"/>
+      <c r="N399" s="9"/>
+      <c r="O399" s="9"/>
+      <c r="P399" s="12"/>
+      <c r="Q399" s="9"/>
+      <c r="R399" s="9"/>
+      <c r="S399" s="14"/>
+      <c r="T399" s="9"/>
+      <c r="U399" s="14"/>
+    </row>
+    <row r="400" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A400" s="7"/>
+      <c r="B400" s="9"/>
+      <c r="C400" s="9"/>
+      <c r="D400" s="9"/>
+      <c r="E400" s="9"/>
+      <c r="F400" s="9"/>
+      <c r="G400" s="9"/>
+      <c r="H400" s="9"/>
+      <c r="I400" s="9"/>
+      <c r="J400" s="9"/>
+      <c r="K400" s="9"/>
+      <c r="L400" s="9"/>
+      <c r="M400" s="9"/>
+      <c r="N400" s="9"/>
+      <c r="O400" s="9"/>
+      <c r="P400" s="12"/>
+      <c r="Q400" s="9"/>
+      <c r="R400" s="9"/>
+      <c r="S400" s="14"/>
+      <c r="T400" s="9"/>
+      <c r="U400" s="14"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="8" fitToWidth="0" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <sheetPr codeName="Sheet6"/>
   <dimension ref="A1:Q116"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12" outlineLevelCol="1" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
#53 Reading List: updated to 2026-07-04.
</commit_message>
<xml_diff>
--- a/data/Reading List.xlsx
+++ b/data/Reading List.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dropbox\Repositories\py-nwreadinglist\nwreadinglist\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D78F65C-68D8-4445-9E1A-CD88A6C4AB89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99155C18-56D5-4CFF-AA34-378925775D97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1140" yWindow="435" windowWidth="27105" windowHeight="13995" tabRatio="313" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,6 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -47,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5815" uniqueCount="1233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5875" uniqueCount="1245">
   <si>
     <t>Format</t>
   </si>
@@ -3746,6 +3745,42 @@
   </si>
   <si>
     <t>Developing On AWS With C#</t>
+  </si>
+  <si>
+    <t>Minimal APIs in ASP.NET 9 (2nd Edition)</t>
+  </si>
+  <si>
+    <t>2026-06-02</t>
+  </si>
+  <si>
+    <t>Useful. Clear and well written book.</t>
+  </si>
+  <si>
+    <t>Learning Creative Coding (Version 1.0.1)</t>
+  </si>
+  <si>
+    <t>2026-06-04</t>
+  </si>
+  <si>
+    <t>Useless. The book is mostly motivational and the advanced users are not among the intended targets, but I do apprecciate the layout and the smooth writing style. It could be improved by making it less repetitive, at the end of the day all the chapters convey the same message.</t>
+  </si>
+  <si>
+    <t>Natural Languange Processing With Python</t>
+  </si>
+  <si>
+    <t>2026-06-07</t>
+  </si>
+  <si>
+    <t>Useful. A well-written, smooth and comprehensive book about NLP for beginners. Python examples are simple and clear.</t>
+  </si>
+  <si>
+    <t>The Ultimate Ubuntu Handbook</t>
+  </si>
+  <si>
+    <t>Useful. Ok book for beginners.</t>
+  </si>
+  <si>
+    <t>The Security Metrics Workbook</t>
   </si>
 </sst>
 </file>
@@ -33256,7 +33291,7 @@
         <v>153</v>
       </c>
       <c r="S320" s="14">
-        <f t="shared" ref="S320:S384" si="129">LEN(P320)</f>
+        <f t="shared" ref="S320:S387" si="129">LEN(P320)</f>
         <v>35</v>
       </c>
       <c r="T320" s="10">
@@ -36738,7 +36773,7 @@
       <c r="A372" s="7" t="s">
         <v>1204</v>
       </c>
-      <c r="B372" s="44">
+      <c r="B372" s="14">
         <v>2025</v>
       </c>
       <c r="C372" s="9" t="s">
@@ -36750,7 +36785,7 @@
       <c r="E372" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F372" s="44">
+      <c r="F372" s="14">
         <v>297</v>
       </c>
       <c r="G372" s="9" t="s">
@@ -36776,7 +36811,7 @@
       <c r="M372" s="14">
         <v>3</v>
       </c>
-      <c r="N372" s="44">
+      <c r="N372" s="14">
         <v>79.989999999999995</v>
       </c>
       <c r="O372" s="9" t="s">
@@ -36806,7 +36841,7 @@
       <c r="A373" s="7" t="s">
         <v>1207</v>
       </c>
-      <c r="B373" s="44">
+      <c r="B373" s="14">
         <v>2025</v>
       </c>
       <c r="C373" s="9" t="s">
@@ -36818,7 +36853,7 @@
       <c r="E373" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F373" s="44">
+      <c r="F373" s="14">
         <v>306</v>
       </c>
       <c r="G373" s="9" t="s">
@@ -36841,10 +36876,10 @@
       <c r="L373" s="9" t="s">
         <v>345</v>
       </c>
-      <c r="M373" s="44">
+      <c r="M373" s="14">
         <v>1</v>
       </c>
-      <c r="N373" s="44">
+      <c r="N373" s="14">
         <v>59.99</v>
       </c>
       <c r="O373" s="9" t="s">
@@ -36874,7 +36909,7 @@
       <c r="A374" s="7" t="s">
         <v>1209</v>
       </c>
-      <c r="B374" s="44">
+      <c r="B374" s="14">
         <v>2025</v>
       </c>
       <c r="C374" s="9" t="s">
@@ -36886,7 +36921,7 @@
       <c r="E374" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F374" s="44">
+      <c r="F374" s="14">
         <v>518</v>
       </c>
       <c r="G374" s="9" t="s">
@@ -36909,10 +36944,10 @@
       <c r="L374" s="9" t="s">
         <v>348</v>
       </c>
-      <c r="M374" s="44">
+      <c r="M374" s="14">
         <v>1</v>
       </c>
-      <c r="N374" s="44">
+      <c r="N374" s="14">
         <v>59.99</v>
       </c>
       <c r="O374" s="9" t="s">
@@ -36942,7 +36977,7 @@
       <c r="A375" s="7" t="s">
         <v>1211</v>
       </c>
-      <c r="B375" s="44">
+      <c r="B375" s="14">
         <v>2025</v>
       </c>
       <c r="C375" s="9" t="s">
@@ -36954,7 +36989,7 @@
       <c r="E375" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F375" s="44">
+      <c r="F375" s="14">
         <v>661</v>
       </c>
       <c r="G375" s="9" t="s">
@@ -36977,7 +37012,7 @@
       <c r="L375" s="9" t="s">
         <v>352</v>
       </c>
-      <c r="M375" s="44">
+      <c r="M375" s="14">
         <v>1</v>
       </c>
       <c r="N375" s="35">
@@ -37010,7 +37045,7 @@
       <c r="A376" s="7" t="s">
         <v>1214</v>
       </c>
-      <c r="B376" s="44">
+      <c r="B376" s="14">
         <v>2021</v>
       </c>
       <c r="C376" s="9" t="s">
@@ -37022,7 +37057,7 @@
       <c r="E376" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F376" s="44">
+      <c r="F376" s="14">
         <v>263</v>
       </c>
       <c r="G376" s="9" t="s">
@@ -37045,10 +37080,10 @@
       <c r="L376" s="9" t="s">
         <v>343</v>
       </c>
-      <c r="M376" s="44">
+      <c r="M376" s="14">
         <v>2</v>
       </c>
-      <c r="N376" s="44">
+      <c r="N376" s="14">
         <v>49.99</v>
       </c>
       <c r="O376" s="9" t="s">
@@ -37078,7 +37113,7 @@
       <c r="A377" s="7" t="s">
         <v>1217</v>
       </c>
-      <c r="B377" s="44">
+      <c r="B377" s="14">
         <v>2025</v>
       </c>
       <c r="C377" s="9" t="s">
@@ -37090,7 +37125,7 @@
       <c r="E377" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F377" s="44">
+      <c r="F377" s="14">
         <v>302</v>
       </c>
       <c r="G377" s="9" t="s">
@@ -37113,10 +37148,10 @@
       <c r="L377" s="9" t="s">
         <v>348</v>
       </c>
-      <c r="M377" s="44">
+      <c r="M377" s="14">
         <v>1</v>
       </c>
-      <c r="N377" s="44">
+      <c r="N377" s="14">
         <v>59.99</v>
       </c>
       <c r="O377" s="9" t="s">
@@ -37146,7 +37181,7 @@
       <c r="A378" s="7" t="s">
         <v>1219</v>
       </c>
-      <c r="B378" s="44">
+      <c r="B378" s="14">
         <v>2025</v>
       </c>
       <c r="C378" s="9" t="s">
@@ -37158,7 +37193,7 @@
       <c r="E378" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F378" s="44">
+      <c r="F378" s="14">
         <v>186</v>
       </c>
       <c r="G378" s="9" t="s">
@@ -37181,16 +37216,16 @@
       <c r="L378" s="9" t="s">
         <v>1033</v>
       </c>
-      <c r="M378" s="44">
+      <c r="M378" s="14">
         <v>2</v>
       </c>
-      <c r="N378" s="44">
+      <c r="N378" s="14">
         <v>32.99</v>
       </c>
       <c r="O378" s="9" t="s">
         <v>632</v>
       </c>
-      <c r="P378" s="45" t="s">
+      <c r="P378" s="22" t="s">
         <v>1220</v>
       </c>
       <c r="Q378" s="9" t="s">
@@ -37214,7 +37249,7 @@
       <c r="A379" s="7" t="s">
         <v>1221</v>
       </c>
-      <c r="B379" s="44">
+      <c r="B379" s="14">
         <v>2025</v>
       </c>
       <c r="C379" s="9" t="s">
@@ -37226,7 +37261,7 @@
       <c r="E379" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F379" s="44">
+      <c r="F379" s="14">
         <v>229</v>
       </c>
       <c r="G379" s="9" t="s">
@@ -37249,10 +37284,10 @@
       <c r="L379" s="9" t="s">
         <v>570</v>
       </c>
-      <c r="M379" s="44">
+      <c r="M379" s="14">
         <v>3</v>
       </c>
-      <c r="N379" s="44">
+      <c r="N379" s="14">
         <v>37.380000000000003</v>
       </c>
       <c r="O379" s="9" t="s">
@@ -37282,7 +37317,7 @@
       <c r="A380" s="7" t="s">
         <v>1223</v>
       </c>
-      <c r="B380" s="44">
+      <c r="B380" s="14">
         <v>2025</v>
       </c>
       <c r="C380" s="9" t="s">
@@ -37294,7 +37329,7 @@
       <c r="E380" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F380" s="44">
+      <c r="F380" s="14">
         <v>366</v>
       </c>
       <c r="G380" s="9" t="s">
@@ -37317,10 +37352,10 @@
       <c r="L380" s="9" t="s">
         <v>842</v>
       </c>
-      <c r="M380" s="44">
+      <c r="M380" s="14">
         <v>1</v>
       </c>
-      <c r="N380" s="44">
+      <c r="N380" s="14">
         <v>39.950000000000003</v>
       </c>
       <c r="O380" s="9" t="s">
@@ -37350,7 +37385,7 @@
       <c r="A381" s="7" t="s">
         <v>1225</v>
       </c>
-      <c r="B381" s="44">
+      <c r="B381" s="14">
         <v>2025</v>
       </c>
       <c r="C381" s="9" t="s">
@@ -37362,7 +37397,7 @@
       <c r="E381" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F381" s="44">
+      <c r="F381" s="14">
         <v>418</v>
       </c>
       <c r="G381" s="9" t="s">
@@ -37385,16 +37420,16 @@
       <c r="L381" s="9" t="s">
         <v>1226</v>
       </c>
-      <c r="M381" s="44">
+      <c r="M381" s="14">
         <v>1</v>
       </c>
-      <c r="N381" s="44">
+      <c r="N381" s="14">
         <v>54.99</v>
       </c>
       <c r="O381" s="9" t="s">
         <v>632</v>
       </c>
-      <c r="P381" s="45" t="s">
+      <c r="P381" s="22" t="s">
         <v>1227</v>
       </c>
       <c r="Q381" s="9" t="s">
@@ -37418,7 +37453,7 @@
       <c r="A382" s="7" t="s">
         <v>1228</v>
       </c>
-      <c r="B382" s="44">
+      <c r="B382" s="14">
         <v>2024</v>
       </c>
       <c r="C382" s="9" t="s">
@@ -37430,18 +37465,18 @@
       <c r="E382" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F382" s="44">
+      <c r="F382" s="14">
         <v>582</v>
       </c>
       <c r="G382" s="9" t="s">
         <v>1216</v>
       </c>
       <c r="H382" s="9">
-        <f t="shared" ref="H382:H384" si="216">YEAR(G382)</f>
+        <f t="shared" ref="H382:H389" si="216">YEAR(G382)</f>
         <v>2026</v>
       </c>
       <c r="I382" s="9">
-        <f t="shared" ref="I382:I384" si="217">MONTH(G382)</f>
+        <f t="shared" ref="I382:I389" si="217">MONTH(G382)</f>
         <v>5</v>
       </c>
       <c r="J382" s="9" t="s">
@@ -37453,10 +37488,10 @@
       <c r="L382" s="9" t="s">
         <v>341</v>
       </c>
-      <c r="M382" s="44">
+      <c r="M382" s="14">
         <v>1</v>
       </c>
-      <c r="N382" s="44">
+      <c r="N382" s="14">
         <v>46.99</v>
       </c>
       <c r="O382" s="9" t="s">
@@ -37486,7 +37521,7 @@
       <c r="A383" s="7" t="s">
         <v>1230</v>
       </c>
-      <c r="B383" s="44">
+      <c r="B383" s="14">
         <v>2023</v>
       </c>
       <c r="C383" s="9" t="s">
@@ -37498,7 +37533,7 @@
       <c r="E383" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F383" s="44">
+      <c r="F383" s="14">
         <v>196</v>
       </c>
       <c r="G383" s="9" t="s">
@@ -37521,10 +37556,10 @@
       <c r="L383" s="9" t="s">
         <v>341</v>
       </c>
-      <c r="M383" s="44">
+      <c r="M383" s="14">
         <v>1</v>
       </c>
-      <c r="N383" s="44">
+      <c r="N383" s="14">
         <v>51.99</v>
       </c>
       <c r="O383" s="9" t="s">
@@ -37554,7 +37589,7 @@
       <c r="A384" s="7" t="s">
         <v>1232</v>
       </c>
-      <c r="B384" s="44">
+      <c r="B384" s="14">
         <v>2023</v>
       </c>
       <c r="C384" s="9" t="s">
@@ -37566,7 +37601,7 @@
       <c r="E384" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F384" s="44">
+      <c r="F384" s="14">
         <v>259</v>
       </c>
       <c r="G384" s="9" t="s">
@@ -37589,16 +37624,16 @@
       <c r="L384" s="9" t="s">
         <v>343</v>
       </c>
-      <c r="M384" s="44">
+      <c r="M384" s="14">
         <v>2</v>
       </c>
-      <c r="N384" s="44">
+      <c r="N384" s="14">
         <v>56.99</v>
       </c>
       <c r="O384" s="9" t="s">
         <v>632</v>
       </c>
-      <c r="P384" s="45" t="s">
+      <c r="P384" s="22" t="s">
         <v>642</v>
       </c>
       <c r="Q384" s="9" t="s">
@@ -37619,119 +37654,344 @@
       </c>
     </row>
     <row r="385" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A385" s="7"/>
-      <c r="B385" s="9"/>
-      <c r="C385" s="9"/>
-      <c r="D385" s="9"/>
-      <c r="E385" s="9"/>
-      <c r="F385" s="9"/>
-      <c r="G385" s="9"/>
-      <c r="H385" s="9"/>
-      <c r="I385" s="9"/>
-      <c r="J385" s="9"/>
-      <c r="K385" s="9"/>
-      <c r="L385" s="9"/>
-      <c r="M385" s="9"/>
-      <c r="N385" s="9"/>
-      <c r="O385" s="9"/>
-      <c r="P385" s="12"/>
-      <c r="Q385" s="9"/>
-      <c r="R385" s="9"/>
-      <c r="S385" s="14"/>
-      <c r="T385" s="9"/>
-      <c r="U385" s="14"/>
+      <c r="A385" s="7" t="s">
+        <v>1233</v>
+      </c>
+      <c r="B385" s="14">
+        <v>2024</v>
+      </c>
+      <c r="C385" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D385" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E385" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F385" s="44">
+        <v>252</v>
+      </c>
+      <c r="G385" s="9" t="s">
+        <v>1234</v>
+      </c>
+      <c r="H385" s="9">
+        <f t="shared" si="216"/>
+        <v>2026</v>
+      </c>
+      <c r="I385" s="9">
+        <f t="shared" si="217"/>
+        <v>6</v>
+      </c>
+      <c r="J385" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K385" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L385" s="9" t="s">
+        <v>341</v>
+      </c>
+      <c r="M385" s="44">
+        <v>3</v>
+      </c>
+      <c r="N385" s="44">
+        <v>36.99</v>
+      </c>
+      <c r="O385" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P385" s="45" t="s">
+        <v>1235</v>
+      </c>
+      <c r="Q385" s="9" t="s">
+        <v>441</v>
+      </c>
+      <c r="R385" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S385" s="14">
+        <f t="shared" si="129"/>
+        <v>36</v>
+      </c>
+      <c r="T385" s="14">
+        <v>0</v>
+      </c>
+      <c r="U385" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="386" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A386" s="7"/>
-      <c r="B386" s="9"/>
-      <c r="C386" s="9"/>
-      <c r="D386" s="9"/>
-      <c r="E386" s="9"/>
-      <c r="F386" s="9"/>
-      <c r="G386" s="9"/>
-      <c r="H386" s="9"/>
-      <c r="I386" s="9"/>
-      <c r="J386" s="9"/>
-      <c r="K386" s="9"/>
-      <c r="L386" s="9"/>
-      <c r="M386" s="9"/>
-      <c r="N386" s="9"/>
-      <c r="O386" s="9"/>
-      <c r="P386" s="12"/>
-      <c r="Q386" s="9"/>
-      <c r="R386" s="9"/>
-      <c r="S386" s="14"/>
-      <c r="T386" s="9"/>
-      <c r="U386" s="14"/>
+      <c r="A386" s="7" t="s">
+        <v>1236</v>
+      </c>
+      <c r="B386" s="14">
+        <v>2025</v>
+      </c>
+      <c r="C386" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D386" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E386" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F386" s="44">
+        <v>152</v>
+      </c>
+      <c r="G386" s="9" t="s">
+        <v>1237</v>
+      </c>
+      <c r="H386" s="9">
+        <f t="shared" si="216"/>
+        <v>2026</v>
+      </c>
+      <c r="I386" s="9">
+        <f t="shared" si="217"/>
+        <v>6</v>
+      </c>
+      <c r="J386" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K386" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L386" s="9" t="s">
+        <v>570</v>
+      </c>
+      <c r="M386" s="44">
+        <v>3</v>
+      </c>
+      <c r="N386" s="35">
+        <v>0</v>
+      </c>
+      <c r="O386" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P386" s="12" t="s">
+        <v>1238</v>
+      </c>
+      <c r="Q386" s="9" t="s">
+        <v>442</v>
+      </c>
+      <c r="R386" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S386" s="14">
+        <f t="shared" si="129"/>
+        <v>276</v>
+      </c>
+      <c r="T386" s="14">
+        <v>0</v>
+      </c>
+      <c r="U386" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="387" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A387" s="7"/>
-      <c r="B387" s="9"/>
-      <c r="C387" s="9"/>
-      <c r="D387" s="9"/>
-      <c r="E387" s="9"/>
-      <c r="F387" s="9"/>
-      <c r="G387" s="9"/>
-      <c r="H387" s="9"/>
-      <c r="I387" s="9"/>
-      <c r="J387" s="9"/>
-      <c r="K387" s="9"/>
-      <c r="L387" s="9"/>
-      <c r="M387" s="9"/>
-      <c r="N387" s="9"/>
-      <c r="O387" s="9"/>
-      <c r="P387" s="12"/>
-      <c r="Q387" s="9"/>
-      <c r="R387" s="9"/>
-      <c r="S387" s="14"/>
-      <c r="T387" s="9"/>
-      <c r="U387" s="14"/>
+      <c r="A387" s="7" t="s">
+        <v>1239</v>
+      </c>
+      <c r="B387" s="14">
+        <v>2025</v>
+      </c>
+      <c r="C387" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D387" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E387" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F387" s="44">
+        <v>137</v>
+      </c>
+      <c r="G387" s="9" t="s">
+        <v>1240</v>
+      </c>
+      <c r="H387" s="9">
+        <f t="shared" si="216"/>
+        <v>2026</v>
+      </c>
+      <c r="I387" s="9">
+        <f t="shared" si="217"/>
+        <v>6</v>
+      </c>
+      <c r="J387" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K387" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L387" s="9" t="s">
+        <v>570</v>
+      </c>
+      <c r="M387" s="44">
+        <v>3</v>
+      </c>
+      <c r="N387" s="44">
+        <v>9.99</v>
+      </c>
+      <c r="O387" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P387" s="12" t="s">
+        <v>1241</v>
+      </c>
+      <c r="Q387" s="9" t="s">
+        <v>538</v>
+      </c>
+      <c r="R387" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S387" s="14">
+        <f t="shared" si="129"/>
+        <v>116</v>
+      </c>
+      <c r="T387" s="14">
+        <v>0</v>
+      </c>
+      <c r="U387" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="388" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A388" s="7"/>
-      <c r="B388" s="9"/>
-      <c r="C388" s="9"/>
-      <c r="D388" s="9"/>
-      <c r="E388" s="9"/>
-      <c r="F388" s="9"/>
-      <c r="G388" s="9"/>
-      <c r="H388" s="9"/>
-      <c r="I388" s="9"/>
-      <c r="J388" s="9"/>
-      <c r="K388" s="9"/>
-      <c r="L388" s="9"/>
-      <c r="M388" s="9"/>
-      <c r="N388" s="9"/>
-      <c r="O388" s="9"/>
-      <c r="P388" s="12"/>
-      <c r="Q388" s="9"/>
-      <c r="R388" s="9"/>
-      <c r="S388" s="14"/>
-      <c r="T388" s="9"/>
-      <c r="U388" s="14"/>
+      <c r="A388" s="7" t="s">
+        <v>1242</v>
+      </c>
+      <c r="B388" s="14">
+        <v>2025</v>
+      </c>
+      <c r="C388" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D388" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E388" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F388" s="44">
+        <v>356</v>
+      </c>
+      <c r="G388" s="9" t="s">
+        <v>1240</v>
+      </c>
+      <c r="H388" s="9">
+        <f t="shared" si="216"/>
+        <v>2026</v>
+      </c>
+      <c r="I388" s="9">
+        <f t="shared" si="217"/>
+        <v>6</v>
+      </c>
+      <c r="J388" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K388" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L388" s="9" t="s">
+        <v>341</v>
+      </c>
+      <c r="M388" s="44">
+        <v>2</v>
+      </c>
+      <c r="N388" s="44">
+        <v>54.99</v>
+      </c>
+      <c r="O388" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P388" s="45" t="s">
+        <v>1243</v>
+      </c>
+      <c r="Q388" s="9" t="s">
+        <v>470</v>
+      </c>
+      <c r="R388" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S388" s="14">
+        <f t="shared" ref="S388" si="218">LEN(P388)</f>
+        <v>30</v>
+      </c>
+      <c r="T388" s="14">
+        <v>0</v>
+      </c>
+      <c r="U388" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="389" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A389" s="7"/>
-      <c r="B389" s="9"/>
-      <c r="C389" s="9"/>
-      <c r="D389" s="9"/>
-      <c r="E389" s="9"/>
-      <c r="F389" s="9"/>
-      <c r="G389" s="9"/>
-      <c r="H389" s="9"/>
-      <c r="I389" s="9"/>
-      <c r="J389" s="9"/>
-      <c r="K389" s="9"/>
-      <c r="L389" s="9"/>
-      <c r="M389" s="9"/>
-      <c r="N389" s="9"/>
-      <c r="O389" s="9"/>
-      <c r="P389" s="12"/>
-      <c r="Q389" s="9"/>
-      <c r="R389" s="9"/>
-      <c r="S389" s="14"/>
-      <c r="T389" s="9"/>
-      <c r="U389" s="14"/>
+      <c r="A389" s="7" t="s">
+        <v>1244</v>
+      </c>
+      <c r="B389" s="44">
+        <v>2026</v>
+      </c>
+      <c r="C389" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D389" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E389" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F389" s="44">
+        <v>122</v>
+      </c>
+      <c r="G389" s="9" t="s">
+        <v>1240</v>
+      </c>
+      <c r="H389" s="9">
+        <f t="shared" si="216"/>
+        <v>2026</v>
+      </c>
+      <c r="I389" s="9">
+        <f t="shared" si="217"/>
+        <v>6</v>
+      </c>
+      <c r="J389" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K389" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L389" s="9" t="s">
+        <v>570</v>
+      </c>
+      <c r="M389" s="44">
+        <v>3</v>
+      </c>
+      <c r="N389" s="44">
+        <v>19.989999999999998</v>
+      </c>
+      <c r="O389" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P389" s="45" t="s">
+        <v>1243</v>
+      </c>
+      <c r="Q389" s="9" t="s">
+        <v>923</v>
+      </c>
+      <c r="R389" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S389" s="14">
+        <f t="shared" ref="S389" si="219">LEN(P389)</f>
+        <v>30</v>
+      </c>
+      <c r="T389" s="14">
+        <v>0</v>
+      </c>
+      <c r="U389" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="390" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A390" s="7"/>

</xml_diff>